<commit_message>
eval: hold Task 5 cases out of the RAG corpus and re-run Task 2-7
Task 5's 17 company cases were being indexed into the knowledge base, so
case-type questions retrieved the answer key itself and inflated the
metrics. They are now held-out benchmark data:

- backend/scripts/build_case_corpus.py writes to
  data/evaluation/case_benchmark/ instead of data/raw/case/ + data/metadata/
- corpus re-ingested from Task 1 evidence only: 30 docs / 2872 chunks
- registry rebuilt to 30 entries (no RELOC_*/PLUS1_*/RETURN_*)

Task 2:
- 8 case-question golds reverted to their Task 1 ids (revision log kept)
- manual scoring sheet rebuilt against the new retrieval set and re-keyed
  by evidence_id instead of rank: Relevance 1.753 / Authority 1.813 /
  Hit@5 100% / Coverage 1.867

Derived outputs refreshed: Task 3 baseline 0.920/0.893/0.885,
Task 4 optimised 0.940/0.931/0.874, Task 6 risk recall 0.461 -> 0.779.
</commit_message>
<xml_diff>
--- a/Task2_manual_scoring_v3.xlsx
+++ b/Task2_manual_scoring_v3.xlsx
@@ -607,12 +607,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>RELOC_006</t>
+          <t>CASE_005</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>蜂巢能源 SVOLT：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>新易盛：2022年设立泰国基地，一二期已投产</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -639,12 +639,12 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>蜂巢能源泰国电池工厂已投产，直接案例</t>
+          <t>新易盛泰国基地一二期已投产，直接案例</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>澎湃新闻</t>
+          <t>国盛证券（经腾讯新闻转载）</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>RELOC_001; RELOC_002; RELOC_006; CASE_004; CASE_005; CASE_006; CASE_008</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_008</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RELOC_006 Title: 蜂巢能源 SVOLT：中国 → 东南亚转移（多地区混合布局） Publisher: 澎湃新闻 Country/Jurisdiction: CN/TH Publication date: 2024-02-28 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池 Claim: 在泰国春武里府是拉差市建设电池工厂（模组 PACK + 电芯），2024-02-28 正式投产并批量交付，配套长</t>
+          <t>摘要 在过去几周的周报中，我们反复强调光模块行业正处于高景气周期，AI算力需求持续爆发推动高端光模块需求快速增长，供给将成为核心矛盾。 近期我们调研发现，头部厂商在大陆和泰国加速扩产，预计2026年一季度将迎来产能集中释放，驱动业绩进入新一轮爬坡期。 【算力需求强劲，瓶颈在于供给】 算力产业链正处于高景气周期，AI模型持续创新演进推动算力需求快速增长。 业绩全面超预期： 谷歌新一代大模型Gemini 3表现优异，Scaling Law持续有效； 英伟达发布三季度财报，业绩及指引全面超预期。 谷歌与英伟达的强势表现，共同印证了模型创新与算力建设正在形成相互</t>
         </is>
       </c>
     </row>
@@ -684,12 +684,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>RETURN_004</t>
+          <t>CASE_004</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>蜂巢能源 SVOLT（欧洲业务）：重新评估 / 回流中国（维持现有海外布局（收缩新增））</t>
+          <t>中际旭创：泰国工厂产能与国内基本齐平</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -703,25 +703,25 @@
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>1</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>欧洲业务收缩，与泰国建厂无关 ｜ 人工判定与Auto(1)不同，请复核</t>
+          <t>中际旭创泰国工厂产能与国内齐平，直接案例</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>36氪 / 财新网</t>
+          <t>国盛证券（经腾讯新闻转载）</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>RELOC_001; RELOC_002; RELOC_006; CASE_004; CASE_005; CASE_006; CASE_008</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_008</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RETURN_004 Title: 蜂巢能源 SVOLT（欧洲业务）：重新评估 / 回流中国（维持现有海外布局（收缩新增）） Publisher: 36氪 / 财新网 Country/Jurisdiction: CN/DE Publication date: 2024-10-28 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池 Claim: 2024-05 取消勃兰登堡州电芯超级工厂计划，2024-10 宣布停建</t>
+          <t>摘要 在过去几周的周报中，我们反复强调光模块行业正处于高景气周期，AI算力需求持续爆发推动高端光模块需求快速增长，供给将成为核心矛盾。 近期我们调研发现，头部厂商在大陆和泰国加速扩产，预计2026年一季度将迎来产能集中释放，驱动业绩进入新一轮爬坡期。 【算力需求强劲，瓶颈在于供给】 算力产业链正处于高景气周期，AI模型持续创新演进推动算力需求快速增长。 业绩全面超预期： 谷歌新一代大模型Gemini 3表现优异，Scaling Law持续有效； 英伟达发布三季度财报，业绩及指引全面超预期。 谷歌与英伟达的强势表现，共同印证了模型创新与算力建设正在形成相互</t>
         </is>
       </c>
     </row>
@@ -761,12 +761,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>RELOC_003</t>
+          <t>CASE_001</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>国轩高科 Gotion High-Tech：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>Dawang Metals：客户订单转移印度后回流，企业放弃海外建厂</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -786,19 +786,19 @@
         <v>1</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>1</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>国轩为越南基地，非泰国 ｜ 人工判定与Auto(1)不同，请复核</t>
+          <t>Dawang Metals 为订单转印度后回流案例，可作建厂节奏反向参照，但非泰国布局</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>澎湃新闻 / 盖世汽车社区</t>
+          <t>路透社（Reuters）</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>RELOC_001; RELOC_002; RELOC_006; CASE_004; CASE_005; CASE_006; CASE_008</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_008</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RELOC_003 Title: 国轩高科 Gotion High-Tech：中国 → 东南亚转移（多地区混合布局） Publisher: 澎湃新闻 / 盖世汽车社区 Country/Jurisdiction: CN/VN Publication date: 2022-11-19 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池 Claim: 与 Vingroup 旗下 VinES 合资（国轩 51% / VinE</t>
+          <t>Evidence ID: CASE_001 Title: Dawang Metals：客户订单转移印度后回流，企业放弃海外建厂 Publisher: 路透社（Reuters） Country/Jurisdiction: CN / National Publication date: 2026-09-14 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 金属铸造 Key finding: 路透原文《Companies left China to do</t>
         </is>
       </c>
     </row>
@@ -838,12 +838,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>RELOC_002</t>
+          <t>CASE_006</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>长安汽车 Changan Automobile：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>天孚通信：泰国一期投产、二期2025年投入使用</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -853,29 +853,29 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
         <v>2</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>2</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>长安泰国整车工厂投产，直接案例</t>
+          <t>天孚通信泰国一期投产、二期2025启用，直接案例</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>易车 / 证券之星（投资者互动平台）</t>
+          <t>国盛证券（经腾讯新闻转载）</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>RELOC_001; RELOC_002; RELOC_006; CASE_004; CASE_005; CASE_006; CASE_008</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_008</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RELOC_002 Title: 长安汽车 Changan Automobile：中国 → 东南亚转移（多地区混合布局） Publisher: 易车 / 证券之星（投资者互动平台） Country/Jurisdiction: CN/TH Publication date: 2025-05-16 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 整车/汽车 Claim: 在泰国罗勇府建设整车工厂，2025-05-16 竣工投产</t>
+          <t>摘要 在过去几周的周报中，我们反复强调光模块行业正处于高景气周期，AI算力需求持续爆发推动高端光模块需求快速增长，供给将成为核心矛盾。 近期我们调研发现，头部厂商在大陆和泰国加速扩产，预计2026年一季度将迎来产能集中释放，驱动业绩进入新一轮爬坡期。 【算力需求强劲，瓶颈在于供给】 算力产业链正处于高景气周期，AI模型持续创新演进推动算力需求快速增长。 业绩全面超预期： 谷歌新一代大模型Gemini 3表现优异，Scaling Law持续有效； 英伟达发布三季度财报，业绩及指引全面超预期。 谷歌与英伟达的强势表现，共同印证了模型创新与算力建设正在形成相互</t>
         </is>
       </c>
     </row>
@@ -915,12 +915,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>RELOC_001</t>
+          <t>CASE_008</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>比亚迪 BYD：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>光模块厂商选择东南亚建厂以规避与欧美客户合作风险（中际旭创互动平台回复等）</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -930,29 +930,29 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
         <v>2</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>2</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>比亚迪泰国整车工厂投产，直接案例</t>
+          <t>光模块厂商东南亚建厂以规避欧美客户合作风险，直接说明泰国布局</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>东方财富网（转比亚迪官方）</t>
+          <t>中国基金报</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>RELOC_001; RELOC_002; RELOC_006; CASE_004; CASE_005; CASE_006; CASE_008</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_008</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -977,7 +977,7 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RELOC_001 Title: 比亚迪 BYD：中国 → 东南亚转移（多地区混合布局） Publisher: 东方财富网（转比亚迪官方） Country/Jurisdiction: CN/TH Publication date: 2024-07-04 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 整车/汽车 Claim: 2022-09 与 WHA 签约，在泰国罗勇府建全资乘用车工厂；2024-07-04 竣工投产，年</t>
+          <t>中国基金报记者 文夕 全球科技巨头持续加码算力，光模块环节厂商已成最大赢家之一。 7月14日，市值超1600亿元的全球光模块龙头中际旭创披露了一份“炸裂”的半年业绩预告。 数据显示，中际旭创预计上半年实现归母净利润21. 5亿元-25亿元，增长幅度上限超300%，而业绩下限水平甚至已可比肩去年全年。 半年业绩或超去年全年 中际旭创业绩预告显示，该公司预计上半年实现净利润21. 5亿元-25亿元，同比增长250. 3%-307. 33%。 而且，中际旭创还称，今年上半年确认股权激励费用减少公司合并净利润约9300万元。 对于上半年业绩大幅增长，中际旭创解释</t>
         </is>
       </c>
     </row>
@@ -992,12 +992,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>RETURN_001</t>
+          <t>CASE_007</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份 Yunnan Energy New Material (Semcorp)：重新评估 / 回流中国（提高中国生产比例）</t>
+          <t>华工正源：马来西亚工厂，公开表述为规避地缘风险</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1007,29 +1007,29 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
         <v>2</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>2</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>恩捷终止马来西亚项目：马来西亚布局决策的直接案例</t>
+          <t>华工正源马来西亚工厂，公开表述为规避地缘风险，直接案例</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份公告（经东方财富网 / 央广网报道）</t>
+          <t>C114通信网</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>RELOC_004; RETURN_001; PLUS1_004; CASE_007; CASE_008; CASE_010</t>
+          <t>CASE_007; CASE_008; CASE_010</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>## 一、决策前状态（Initial Situation） 生产布局：湿法锂电隔膜产能以中国为主（上海、珠海、无锡等），为全球隔膜龙头。 主要市场：中国 + 海外电池客户（含欧美）。 供应链结构：基膜与涂覆材料主要在中国生产，产品出口海外。 面临的问题：2024 年规划马来西亚隔膜项目（约 10 亿平方米/年、投资约 20 亿元）以求贴近海外客户并规避关税。 ## 二、决策触发（Decision Trigger） 触发类型：cost_change（成本变化） 触发细节：外部市场环境及行业竞争格局发生变化（隔膜价格下行、行业产能过剩、海外建厂成本高于预期）</t>
+          <t>资讯 视频 6G 光通信 物联网 量子通信 卫星互联网 数智低空 Cloud&amp;AI 政策 运营商 设备商 终端 财经 市场 会展 直播 2026/3/25 16:29 2026十大光模块厂商，光模块厂商有哪些 C114通信网 26 1 2026年，随着 AI 算力需求持续爆发与全球数据中心带宽升级加速，光模块行业迎来“800G普及+1. 6T放量”的双轮驱动阶段。 据行业预测，2026年全球800G光模块需求量有望突破4000万只，1. 6T需求亦进入商业化元年。 在这场高速光互联的竞逐中，中国光模块厂商凭借技术突破与产能优势占据全球主导地位。 本文综合</t>
         </is>
       </c>
     </row>
@@ -1069,44 +1069,44 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>RELOC_004</t>
+          <t>CASE_010</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>亿纬锂能 EVE Energy：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>白宫点名东南亚为非法转运高风险地区，并推出AI执法工具</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>原产地与转运</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
         <v>2</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>2</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>亿纬锂能马来西亚工厂投产，直接案例</t>
+          <t>白宫点名东南亚（含马来西亚）为转运高风险，美国官方判断</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>新浪财经</t>
+          <t>美国白宫（经律所解读）</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>RELOC_004; RETURN_001; PLUS1_004; CASE_007; CASE_008; CASE_010</t>
+          <t>CASE_007; CASE_008; CASE_010</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>## 二、决策触发（Decision Trigger） 触发类型：tariff_pressure（关税压力） 触发细节：对美出口关税与'去中国化'供应链要求，迫使企业在东南亚布局产能以规避税率。 ## 三、实际决策（Actual Decision） 决策分类：多地区混合布局 决策内容：在马来西亚吉打州居林县建设海外工厂，二期于 2026 年 2 月投产运营，建筑面积约 60 万平方米，系公司首个海外大型锂电厂房项目，形成年产约 6.8 亿只圆柱电池产能；同时推进匈牙利、美国、印尼项目，中国产能保留。 ## 四、相关风险（Related Risk） 风险类</t>
+          <t>Evidence ID: CASE_010 Title: 白宫点名东南亚为非法转运高风险地区，并推出AI执法工具 Publisher: 美国白宫（经律所解读） Country/Jurisdiction: US / Federal Publication date: 2026-08-13 Status: CURRENT Topic: 原产地与转运 Applicability scope: GENERAL Related industries: 通用 Key finding: 由WH_001与WH_002组成。对已在越南/泰国/马来西亚布局的企业，原产地举证</t>
         </is>
       </c>
     </row>
@@ -1146,44 +1146,44 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>CASE_007</t>
+          <t>CASE_003</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>华工正源：马来西亚工厂，公开表述为规避地缘风险</t>
+          <t>同一反规避调查中被认定“未规避”的企业（Hanwha、Jinko马来西亚、Boviet越南）</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>反规避</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>2</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>华工正源马来西亚工厂，公开表述为规避地缘风险，直接案例</t>
+          <t>美国商务部反规避认定（含马来西亚企业），直接反映美方对马来西亚原产地的官方判断 ｜ 人工判定与Auto(0)不同，请复核</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>C114通信网</t>
+          <t>美国商务部（经律所解读）</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>RELOC_004; RETURN_001; PLUS1_004; CASE_007; CASE_008; CASE_010</t>
+          <t>CASE_007; CASE_008; CASE_010</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>资讯 视频 6G 光通信 物联网 量子通信 卫星互联网 数智低空 Cloud&amp;AI 政策 运营商 设备商 终端 财经 市场 会展 直播 2026/3/25 16:29 2026十大光模块厂商，光模块厂商有哪些 C114通信网 26 1 2026年，随着 AI 算力需求持续爆发与全球数据中心带宽升级加速，光模块行业迎来“800G普及+1. 6T放量”的双轮驱动阶段。 据行业预测，2026年全球800G光模块需求量有望突破4000万只，1. 6T需求亦进入商业化元年。 在这场高速光互联的竞逐中，中国光模块厂商凭借技术突破与产能优势占据全球主导地位。 本文综合</t>
+          <t>Evidence ID: CASE_003 Title: 同一反规避调查中被认定“未规避”的企业（Hanwha、Jinko马来西亚、Boviet越南） Publisher: 美国商务部（经律所解读） Country/Jurisdiction: 马来西亚/越南 Publication date: 2023-08-18 Status: CURRENT Topic: 反规避 Applicability scope: GENERAL Related industries: 光伏 Key finding: 与CASE_002构成对照：同一规则下，供应链结构不同导致</t>
         </is>
       </c>
     </row>
@@ -1223,44 +1223,44 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>PLUS1_004</t>
+          <t>CASE_002</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>晶科能源 JinkoSolar：China + 1 战略（多地区混合布局）</t>
+          <t>美国对东南亚四国光伏产品反规避认定：视为中国原产并适用对华双反</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>反规避</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>晶科含马来西亚枢纽，但为光伏多地区结构，非马来西亚布局主案例 ｜ 人工判定与Auto(2)不同，请复核</t>
+          <t>美国商务部认定东南亚四国光伏视为中国原产，直接反映美方对马来西亚原产地的官方判断 ｜ 人工判定与Auto(0)不同，请复核</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>东方财富财富号</t>
+          <t>美国商务部（经律所解读）</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>RELOC_004; RETURN_001; PLUS1_004; CASE_007; CASE_008; CASE_010</t>
+          <t>CASE_007; CASE_008; CASE_010</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>## 一、决策前状态（Initial Situation） 生产布局：硅片—电池—组件一体化产能以中国为核心。 主要市场：全球（中国、欧洲、美国、新兴市场）。 供应链结构：硅料、硅片主要在中国，组件通过海外基地与出口进入欧美。 面临的问题：美国对东南亚四国光伏产品的双反与反规避调查，使'中国—东南亚—美国'路径的关税优势不稳定（参见 Task 1 的 CASE_002/CASE_003）。 ## 二、决策触发（Decision Trigger） 触发类型：tariff_pressure（关税压力） 触发细节：美国对东南亚光伏组件的双反/反规避认定，以及美</t>
+          <t>Evidence ID: CASE_002 Title: 美国对东南亚四国光伏产品反规避认定：视为中国原产并适用对华双反 Publisher: 美国商务部（经律所解读） Country/Jurisdiction: 柬埔寨/马来西亚/泰国/越南 Publication date: 2023-08-18 Status: CURRENT Topic: 反规避 Applicability scope: GENERAL Related industries: 光伏 Key finding: 2022年4月立案，2023年8月终裁。使用中国组件在东南亚完成的电池和组</t>
         </is>
       </c>
     </row>
@@ -1300,44 +1300,44 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>CASE_010</t>
+          <t>TRD_003</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>白宫点名东南亚为非法转运高风险地区，并推出AI执法工具</t>
+          <t>中国对越南、泰国、马来西亚出口 HS 8541/8542（中间品），2018–2025年度</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>原产地与转运</t>
+          <t>贸易流</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>2</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>白宫点名东南亚（含马来西亚）为转运高风险，美国官方判断</t>
+          <t>中国对马/越/泰中间品出口数据，间接支持企业马来西亚布局判断</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>美国白宫（经律所解读）</t>
+          <t>联合国商品贸易统计数据库（UN Comtrade）</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>RELOC_004; RETURN_001; PLUS1_004; CASE_007; CASE_008; CASE_010</t>
+          <t>CASE_007; CASE_008; CASE_010</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: CASE_010 Title: 白宫点名东南亚为非法转运高风险地区，并推出AI执法工具 Publisher: 美国白宫（经律所解读） Country/Jurisdiction: US / Federal Publication date: 2026-08-13 Status: CURRENT Topic: 原产地与转运 Applicability scope: GENERAL Related industries: 通用 Key finding: 由WH_001与WH_002组成。对已在越南/泰国/马来西亚布局的企业，原产地举证</t>
+          <t>Evidence ID: TRD_003 Title: 中国对越南、泰国、马来西亚出口 HS 8541/8542（中间品），2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: CN / National Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: ◆电子/光电 Key finding: 看东南亚产能是否依赖中国中间</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; RETURN_001; RETURN_002; RETURN_003; RETURN_004</t>
+          <t>CASE_001; CASE_002; CASE_003</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1454,12 +1454,12 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>RETURN_001</t>
+          <t>CASE_008</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份 Yunnan Energy New Material (Semcorp)：重新评估 / 回流中国（提高中国生产比例）</t>
+          <t>光模块厂商选择东南亚建厂以规避与欧美客户合作风险（中际旭创互动平台回复等）</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1469,29 +1469,29 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>终止马来西亚项目、资源回投国内，直接回流实例</t>
+          <t>东南亚建厂规避风险案例，与「回流中国」方向相反，仅作同类布局参照</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份公告（经东方财富网 / 央广网报道）</t>
+          <t>中国基金报</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; RETURN_001; RETURN_002; RETURN_003; RETURN_004</t>
+          <t>CASE_001; CASE_002; CASE_003</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RETURN_001 Title: 恩捷股份 Yunnan Energy New Material (Semcorp)：重新评估 / 回流中国（提高中国生产比例） Publisher: 恩捷股份公告（经东方财富网 / 央广网报道） Country/Jurisdiction: CN/MY Publication date: 2026-05-22 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 电池材料 Claim: 2026</t>
+          <t>Evidence ID: CASE_008 Title: 光模块厂商选择东南亚建厂以规避与欧美客户合作风险（中际旭创互动平台回复等） Publisher: 中国基金报 Country/Jurisdiction: CN / National Publication date: 2024-07-14 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 光模块 Key finding: 文中引用中际旭创互动平台回复，可据此到互动易查原始问答，升级为一手证据。</t>
         </is>
       </c>
     </row>
@@ -1531,12 +1531,12 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>RETURN_004</t>
+          <t>CASE_007</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>蜂巢能源 SVOLT（欧洲业务）：重新评估 / 回流中国（维持现有海外布局（收缩新增））</t>
+          <t>华工正源：马来西亚工厂，公开表述为规避地缘风险</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1550,25 +1550,25 @@
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>1</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>1</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>停建德国工厂、终止欧洲业务，资源集中中国，直接实例</t>
+          <t>马来西亚工厂案例，与「回流中国」方向相反，仅作同类布局参照</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>36氪 / 财新网</t>
+          <t>C114通信网</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; RETURN_001; RETURN_002; RETURN_003; RETURN_004</t>
+          <t>CASE_001; CASE_002; CASE_003</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RETURN_004 Title: 蜂巢能源 SVOLT（欧洲业务）：重新评估 / 回流中国（维持现有海外布局（收缩新增）） Publisher: 36氪 / 财新网 Country/Jurisdiction: CN/DE Publication date: 2024-10-28 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池 Claim: 2024-05 取消勃兰登堡州电芯超级工厂计划，2024-10 宣布停建</t>
+          <t>在AI算力基础设施持续扩张的背景下，具备高速率产品量产能力、全球化交付能力与核心器件自研能力的厂商，将在下一阶段竞争中占据主动。 对于下游客户而言，根据自身场景需求在“规模稳定”、“性价比”、“行业定制”三者之间做出选择，已成为当前光模块采购决策的关键。 C114中国通信网版权说明：凡注明来源为“C114通信网”的文章皆属C114版权所有，除与C114签署内容授权协议的单位外，其他单位未经允许禁止转载、摘编，违者必究。 如需使用，请联系021-54451141（汪先生）。 其中编译类仅出于传递更多信息之目的，系C114对海外相关站点最新信息的翻译稿，仅供</t>
         </is>
       </c>
     </row>
@@ -1608,12 +1608,12 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>RETURN_002</t>
+          <t>CASE_006</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>富士康 Foxconn / 苹果 Apple（供应链）：重新评估 / 回流中国（提高中国生产比例）</t>
+          <t>天孚通信：泰国一期投产、二期2025年投入使用</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>1</v>
@@ -1640,12 +1640,12 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>富士康撤回印度工程团队、重新评估海外布局，「订单/产能回流中国」未获证实，部分相关 ｜ 人工判定与Auto(2)不同，请复核</t>
+          <t>泰国工厂案例，与「回流中国」方向相反，仅作同类布局参照</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>新浪科技 / 中关村在线</t>
+          <t>国盛证券（经腾讯新闻转载）</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; RETURN_001; RETURN_002; RETURN_003; RETURN_004</t>
+          <t>CASE_001; CASE_002; CASE_003</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RETURN_002 Title: 富士康 Foxconn / 苹果 Apple（供应链）：重新评估 / 回流中国（提高中国生产比例） Publisher: 新浪科技 / 中关村在线 Country/Jurisdiction: TW/CN/IN Publication date: 2025-07-03 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 电子制造 Claim: 2025 年 7 月及 12 月，富士康两度要求/</t>
+          <t>截至9月30日，阿里云在全球29个地区运营着91个可用区，并宣布在巴西、法国和荷兰新建数据中心。 同时，阿里上线千问App，向AI to C领域发力。 公测版APP上线一周的下载量已超1000万。 未来，千问还将陆续接入电商、地图、本地生活等阿里业务生态场景。 在财报电话会上，阿里巴巴高管表示，目前看到客户对AI的需求非常旺盛，阿里云AI服务器上架节奏其实还是严重跟不上客户订单的增长速度，在手积压订单数量还在持续扩大。 8. 中国首个光量子计算机制造工厂！ 从“艺术品”到“工业品”蜕变 据C114报道，11月24日，“国际量子年大湾区活动周”主题活动——</t>
         </is>
       </c>
     </row>
@@ -1685,12 +1685,12 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>RETURN_003</t>
+          <t>CASE_004</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>制造业外迁企业（行业层面）：重新评估 / 回流中国（提高中国生产比例）</t>
+          <t>中际旭创：泰国工厂产能与国内基本齐平</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1704,25 +1704,25 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>1</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>1</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>行业层面订单与产能回流中国，直接实例</t>
+          <t>泰国工厂案例，与「回流中国」方向相反，仅作同类布局参照</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>路透社（经环球网 / 新浪转载）</t>
+          <t>国盛证券（经腾讯新闻转载）</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; RETURN_001; RETURN_002; RETURN_003; RETURN_004</t>
+          <t>CASE_001; CASE_002; CASE_003</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RETURN_003 Title: 制造业外迁企业（行业层面）：重新评估 / 回流中国（提高中国生产比例） Publisher: 路透社（经环球网 / 新浪转载） Country/Jurisdiction: CN/VN/TH/IN Publication date: 2026-09-14 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 通用制造 Claim: 部分跨国企业将订单与产能重新回流中国，同时保留东南亚既有布局，形</t>
+          <t>截至9月30日，阿里云在全球29个地区运营着91个可用区，并宣布在巴西、法国和荷兰新建数据中心。 同时，阿里上线千问App，向AI to C领域发力。 公测版APP上线一周的下载量已超1000万。 未来，千问还将陆续接入电商、地图、本地生活等阿里业务生态场景。 在财报电话会上，阿里巴巴高管表示，目前看到客户对AI的需求非常旺盛，阿里云AI服务器上架节奏其实还是严重跟不上客户订单的增长速度，在手积压订单数量还在持续扩大。 8. 中国首个光量子计算机制造工厂！ 从“艺术品”到“工业品”蜕变 据C114报道，11月24日，“国际量子年大湾区活动周”主题活动——</t>
         </is>
       </c>
     </row>
@@ -1762,12 +1762,12 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>RELOC_005</t>
+          <t>CASE_008</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>欣旺达 Sunwoda：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>光模块厂商选择东南亚建厂以规避与欧美客户合作风险（中际旭创互动平台回复等）</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1794,12 +1794,12 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>越南扩产以规避关税，服务海外客户的布局案例</t>
+          <t>东南亚建厂以规避与欧美客户合作风险，布局与客户关系直接说明</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>东方财富网 / 腾讯新闻</t>
+          <t>中国基金报</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>CASE_004; CASE_005; CASE_006; CASE_007; CASE_008; RELOC_003; RELOC_004; RELOC_005; RELOC_006</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_007; CASE_008</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RELOC_005 Title: 欣旺达 Sunwoda：中国 → 东南亚转移（多地区混合布局） Publisher: 东方财富网 / 腾讯新闻 Country/Jurisdiction: CN/VN Publication date: 2024-07-16 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池/消费电池 Claim: 2024-07-15 公告拟通过下属子公司香港欣威设立越南锂威有限公司，投建越南锂威</t>
+          <t>中国基金报记者 文夕 全球科技巨头持续加码算力，光模块环节厂商已成最大赢家之一。 7月14日，市值超1600亿元的全球光模块龙头中际旭创披露了一份“炸裂”的半年业绩预告。 数据显示，中际旭创预计上半年实现归母净利润21. 5亿元-25亿元，增长幅度上限超300%，而业绩下限水平甚至已可比肩去年全年。 半年业绩或超去年全年 中际旭创业绩预告显示，该公司预计上半年实现净利润21. 5亿元-25亿元，同比增长250. 3%-307. 33%。 而且，中际旭创还称，今年上半年确认股权激励费用减少公司合并净利润约9300万元。 对于上半年业绩大幅增长，中际旭创解释</t>
         </is>
       </c>
     </row>
@@ -1839,12 +1839,12 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>RELOC_004</t>
+          <t>CASE_007</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>亿纬锂能 EVE Energy：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>华工正源：马来西亚工厂，公开表述为规避地缘风险</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1871,12 +1871,12 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>马来西亚制造—欧美市场的结构，直接说明布局与客户关系</t>
+          <t>马来西亚工厂公开表述为规避地缘风险，直接说明</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>新浪财经</t>
+          <t>C114通信网</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>CASE_004; CASE_005; CASE_006; CASE_007; CASE_008; RELOC_003; RELOC_004; RELOC_005; RELOC_006</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_007; CASE_008</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>## 二、决策触发（Decision Trigger） 触发类型：tariff_pressure（关税压力） 触发细节：对美出口关税与'去中国化'供应链要求，迫使企业在东南亚布局产能以规避税率。 ## 三、实际决策（Actual Decision） 决策分类：多地区混合布局 决策内容：在马来西亚吉打州居林县建设海外工厂，二期于 2026 年 2 月投产运营，建筑面积约 60 万平方米，系公司首个海外大型锂电厂房项目，形成年产约 6.8 亿只圆柱电池产能；同时推进匈牙利、美国、印尼项目，中国产能保留。 ## 四、相关风险（Related Risk） 风险类</t>
+          <t>在AI算力基础设施持续扩张的背景下，具备高速率产品量产能力、全球化交付能力与核心器件自研能力的厂商，将在下一阶段竞争中占据主动。 对于下游客户而言，根据自身场景需求在“规模稳定”、“性价比”、“行业定制”三者之间做出选择，已成为当前光模块采购决策的关键。 C114中国通信网版权说明：凡注明来源为“C114通信网”的文章皆属C114版权所有，除与C114签署内容授权协议的单位外，其他单位未经允许禁止转载、摘编，违者必究。 如需使用，请联系021-54451141（汪先生）。 其中编译类仅出于传递更多信息之目的，系C114对海外相关站点最新信息的翻译稿，仅供</t>
         </is>
       </c>
     </row>
@@ -1916,12 +1916,12 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>RELOC_003</t>
+          <t>CASE_004</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>国轩高科 Gotion High-Tech：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>中际旭创：泰国工厂产能与国内基本齐平</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1948,12 +1948,12 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>越南电池基地服务海外客户，布局案例</t>
+          <t>泰国工厂产能与国内齐平，直接说明海外布局</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>澎湃新闻 / 盖世汽车社区</t>
+          <t>国盛证券（经腾讯新闻转载）</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>CASE_004; CASE_005; CASE_006; CASE_007; CASE_008; RELOC_003; RELOC_004; RELOC_005; RELOC_006</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_007; CASE_008</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RELOC_003 Title: 国轩高科 Gotion High-Tech：中国 → 东南亚转移（多地区混合布局） Publisher: 澎湃新闻 / 盖世汽车社区 Country/Jurisdiction: CN/VN Publication date: 2022-11-19 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池 Claim: 与 Vingroup 旗下 VinES 合资（国轩 51% / VinE</t>
+          <t>玻色量子这座工厂的意义，不仅在于“造出一台量子计算机”，更在于建立了一套可复制、可扩展的量子硬件制造标准。 它标志着我国在量子计算从“实验室走向生产线”的关键一步，也为未来构建自主可控的量子产业链打下了坚实基础。 9. 谷歌TPU硬刚英伟达！ AI芯片市场从英伟达垄断转向多元化 据C114报道，当前全球AI大模型和芯片领域掀起新一轮军备竞赛。 美国白宫周一发布声明称，总统特朗普签署了一项行政命令，启动一项旨在利用AI变革科学研究方式、加速科学发现的全新国家计划“创世纪计划”。 在 AI大模型和芯片竞争背景下，对算力存在巨大需求。 谷歌近日发布了最新的大语</t>
         </is>
       </c>
     </row>
@@ -1993,12 +1993,12 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>RELOC_006</t>
+          <t>CASE_005</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>蜂巢能源 SVOLT：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>新易盛：2022年设立泰国基地，一二期已投产</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -2025,12 +2025,12 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>泰国电池厂配套中国车企在泰车型，布局与客户关系直接</t>
+          <t>泰国基地服务海外客户，直接说明布局与客户关系</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>澎湃新闻</t>
+          <t>国盛证券（经腾讯新闻转载）</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>CASE_004; CASE_005; CASE_006; CASE_007; CASE_008; RELOC_003; RELOC_004; RELOC_005; RELOC_006</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_007; CASE_008</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RELOC_006 Title: 蜂巢能源 SVOLT：中国 → 东南亚转移（多地区混合布局） Publisher: 澎湃新闻 Country/Jurisdiction: CN/TH Publication date: 2024-02-28 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池 Claim: 在泰国春武里府是拉差市建设电池工厂（模组 PACK + 电芯），2024-02-28 正式投产并批量交付，配套长</t>
+          <t>玻色量子这座工厂的意义，不仅在于“造出一台量子计算机”，更在于建立了一套可复制、可扩展的量子硬件制造标准。 它标志着我国在量子计算从“实验室走向生产线”的关键一步，也为未来构建自主可控的量子产业链打下了坚实基础。 9. 谷歌TPU硬刚英伟达！ AI芯片市场从英伟达垄断转向多元化 据C114报道，当前全球AI大模型和芯片领域掀起新一轮军备竞赛。 美国白宫周一发布声明称，总统特朗普签署了一项行政命令，启动一项旨在利用AI变革科学研究方式、加速科学发现的全新国家计划“创世纪计划”。 在 AI大模型和芯片竞争背景下，对算力存在巨大需求。 谷歌近日发布了最新的大语</t>
         </is>
       </c>
     </row>
@@ -2070,12 +2070,12 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>RETURN_001</t>
+          <t>CASE_006</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份 Yunnan Energy New Material (Semcorp)：重新评估 / 回流中国（提高中国生产比例）</t>
+          <t>天孚通信：泰国一期投产、二期2025年投入使用</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -2085,29 +2085,29 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>回流案例，说明海外布局风险，但非“东南亚扩产服务欧美客户”的直接说明</t>
+          <t>泰国一期投产、二期在建，直接说明海外布局</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份公告（经东方财富网 / 央广网报道）</t>
+          <t>国盛证券（经腾讯新闻转载）</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>CASE_004; CASE_005; CASE_006; CASE_007; CASE_008; RELOC_003; RELOC_004; RELOC_005; RELOC_006</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_007; CASE_008</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>## 一、决策前状态（Initial Situation） 生产布局：湿法锂电隔膜产能以中国为主（上海、珠海、无锡等），为全球隔膜龙头。 主要市场：中国 + 海外电池客户（含欧美）。 供应链结构：基膜与涂覆材料主要在中国生产，产品出口海外。 面临的问题：2024 年规划马来西亚隔膜项目（约 10 亿平方米/年、投资约 20 亿元）以求贴近海外客户并规避关税。 ## 二、决策触发（Decision Trigger） 触发类型：cost_change（成本变化） 触发细节：外部市场环境及行业竞争格局发生变化（隔膜价格下行、行业产能过剩、海外建厂成本高于预期）</t>
+          <t>玻色量子这座工厂的意义，不仅在于“造出一台量子计算机”，更在于建立了一套可复制、可扩展的量子硬件制造标准。 它标志着我国在量子计算从“实验室走向生产线”的关键一步，也为未来构建自主可控的量子产业链打下了坚实基础。 9. 谷歌TPU硬刚英伟达！ AI芯片市场从英伟达垄断转向多元化 据C114报道，当前全球AI大模型和芯片领域掀起新一轮军备竞赛。 美国白宫周一发布声明称，总统特朗普签署了一项行政命令，启动一项旨在利用AI变革科学研究方式、加速科学发现的全新国家计划“创世纪计划”。 在 AI大模型和芯片竞争背景下，对算力存在巨大需求。 谷歌近日发布了最新的大语</t>
         </is>
       </c>
     </row>
@@ -2378,44 +2378,44 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>RELOC_005</t>
+          <t>CASE_010</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>欣旺达 Sunwoda：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>白宫点名东南亚为非法转运高风险地区，并推出AI执法工具</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>原产地与转运</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>越南消费电池建厂案例，与规避认定无关 ｜ 人工判定与Auto(1)不同，请复核</t>
+          <t>白宫点名东南亚转运高风险并推AI执法，直接说明认定规避的官方立场</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>东方财富网 / 腾讯新闻</t>
+          <t>美国白宫（经律所解读）</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -2440,7 +2440,7 @@
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RELOC_005 Title: 欣旺达 Sunwoda：中国 → 东南亚转移（多地区混合布局） Publisher: 东方财富网 / 腾讯新闻 Country/Jurisdiction: CN/VN Publication date: 2024-07-16 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池/消费电池 Claim: 2024-07-15 公告拟通过下属子公司香港欣威设立越南锂威有限公司，投建越南锂威</t>
+          <t>进口商应预期，如果新关税措施后采购模式发生变化，来自高关税国家的货物经由中介管辖区转运，或声称的原产国缺乏有意义生产证据，原产地主张将受到更严格的审查。 这些事实模式可能引发信息请求、货物搁置、审计查询、EAPA指控或罚款调查。 新的检测工具和执法能力 CBP及其他机构越来越多地拥有先进的数据工具，使转运更容易被识别。 报告描述了一个人工智能驱动的执法平台“侦探边境”，集成了进口数据分析、供应链地图、路由历史、所有权和关联分析、贸易流异常、产能比较以及计算机视觉，以识别高风险货物和潜在的虚假原产地索赔。 CBP的执法行动已经加快。 报告指出，自2025年</t>
         </is>
       </c>
     </row>
@@ -2455,12 +2455,12 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>RETURN_001</t>
+          <t>CASE_001</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份 Yunnan Energy New Material (Semcorp)：重新评估 / 回流中国（提高中国生产比例）</t>
+          <t>Dawang Metals：客户订单转移印度后回流，企业放弃海外建厂</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -2470,29 +2470,29 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="G26" s="2" t="n">
         <v>1</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>终止海外项目案例，与规避认定无关 ｜ 人工判定与Auto(1)不同，请复核</t>
+          <t>印度订单回流案例，与规避/未规避认定无关 ｜ 人工判定与Auto(1)不同，请复核</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份公告（经东方财富网 / 央广网报道）</t>
+          <t>路透社（Reuters）</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>## 一、决策前状态（Initial Situation） 生产布局：湿法锂电隔膜产能以中国为主（上海、珠海、无锡等），为全球隔膜龙头。 主要市场：中国 + 海外电池客户（含欧美）。 供应链结构：基膜与涂覆材料主要在中国生产，产品出口海外。 面临的问题：2024 年规划马来西亚隔膜项目（约 10 亿平方米/年、投资约 20 亿元）以求贴近海外客户并规避关税。 ## 二、决策触发（Decision Trigger） 触发类型：cost_change（成本变化） 触发细节：外部市场环境及行业竞争格局发生变化（隔膜价格下行、行业产能过剩、海外建厂成本高于预期）</t>
+          <t>Evidence ID: CASE_001 Title: Dawang Metals：客户订单转移印度后回流，企业放弃海外建厂 Publisher: 路透社（Reuters） Country/Jurisdiction: CN / National Publication date: 2026-09-14 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 金属铸造 Key finding: 路透原文《Companies left China to do</t>
         </is>
       </c>
     </row>
@@ -4149,17 +4149,17 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>RETURN_001</t>
+          <t>CASE_010</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份 Yunnan Energy New Material (Semcorp)：重新评估 / 回流中国（提高中国生产比例）</t>
+          <t>白宫点名东南亚为非法转运高风险地区，并推出AI执法工具</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>原产地与转运</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -4168,25 +4168,25 @@
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H48" s="2" t="n">
         <v>2</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J48" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>终止马来西亚项目，与该假设无关 ｜ 人工判定与Auto(1)不同，请复核</t>
+          <t>官方执法立场，说明原产地改判风险</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份公告（经东方财富网 / 央广网报道）</t>
+          <t>美国白宫（经律所解读）</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
@@ -4211,7 +4211,7 @@
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t>## 一、决策前状态（Initial Situation） 生产布局：湿法锂电隔膜产能以中国为主（上海、珠海、无锡等），为全球隔膜龙头。 主要市场：中国 + 海外电池客户（含欧美）。 供应链结构：基膜与涂覆材料主要在中国生产，产品出口海外。 面临的问题：2024 年规划马来西亚隔膜项目（约 10 亿平方米/年、投资约 20 亿元）以求贴近海外客户并规避关税。 ## 二、决策触发（Decision Trigger） 触发类型：cost_change（成本变化） 触发细节：外部市场环境及行业竞争格局发生变化（隔膜价格下行、行业产能过剩、海外建厂成本高于预期）</t>
+          <t>进口商应预期，如果新关税措施后采购模式发生变化，来自高关税国家的货物经由中介管辖区转运，或声称的原产国缺乏有意义生产证据，原产地主张将受到更严格的审查。 这些事实模式可能引发信息请求、货物搁置、审计查询、EAPA指控或罚款调查。 新的检测工具和执法能力 CBP及其他机构越来越多地拥有先进的数据工具，使转运更容易被识别。 报告描述了一个人工智能驱动的执法平台“侦探边境”，集成了进口数据分析、供应链地图、路由历史、所有权和关联分析、贸易流异常、产能比较以及计算机视觉，以识别高风险货物和潜在的虚假原产地索赔。 CBP的执法行动已经加快。 报告指出，自2025年</t>
         </is>
       </c>
     </row>
@@ -4226,44 +4226,44 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>RETURN_004</t>
+          <t>TRD_003</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>蜂巢能源 SVOLT（欧洲业务）：重新评估 / 回流中国（维持现有海外布局（收缩新增））</t>
+          <t>中国对越南、泰国、马来西亚出口 HS 8541/8542（中间品），2018–2025年度</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>贸易流</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="G49" s="2" t="n">
         <v>1</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>欧洲业务收缩，与该假设无关 ｜ 人工判定与Auto(1)不同，请复核</t>
+          <t>中间品出口数据，可作原产地认定背景，非执法判例本身</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>36氪 / 财新网</t>
+          <t>联合国商品贸易统计数据库（UN Comtrade）</t>
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr">
@@ -4288,7 +4288,7 @@
       </c>
       <c r="Q49" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RETURN_004 Title: 蜂巢能源 SVOLT（欧洲业务）：重新评估 / 回流中国（维持现有海外布局（收缩新增）） Publisher: 36氪 / 财新网 Country/Jurisdiction: CN/DE Publication date: 2024-10-28 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池 Claim: 2024-05 取消勃兰登堡州电芯超级工厂计划，2024-10 宣布停建</t>
+          <t>Evidence ID: TRD_003 Title: 中国对越南、泰国、马来西亚出口 HS 8541/8542（中间品），2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: CN / National Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: ◆电子/光电 Key finding: 看东南亚产能是否依赖中国中间</t>
         </is>
       </c>
     </row>
@@ -4303,12 +4303,12 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>CASE_010</t>
+          <t>WH_002</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>白宫点名东南亚为非法转运高风险地区，并推出AI执法工具</t>
+          <t>The Great Transshipment Scam: Rise, Scope, and Costs（白宫非法转运报告）</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -4335,12 +4335,12 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>官方执法立场，说明原产地改判风险</t>
+          <t>白宫非法转运报告，官方执法立场直接证据</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>美国白宫（经律所解读）</t>
+          <t>美国白宫贸易与制造业政策办公室</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr">
@@ -4365,7 +4365,7 @@
       </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>进口商应预期，如果新关税措施后采购模式发生变化，来自高关税国家的货物经由中介管辖区转运，或声称的原产国缺乏有意义生产证据，原产地主张将受到更严格的审查。 这些事实模式可能引发信息请求、货物搁置、审计查询、EAPA指控或罚款调查。 新的检测工具和执法能力 CBP及其他机构越来越多地拥有先进的数据工具，使转运更容易被识别。 报告描述了一个人工智能驱动的执法平台“侦探边境”，集成了进口数据分析、供应链地图、路由历史、所有权和关联分析、贸易流异常、产能比较以及计算机视觉，以识别高风险货物和潜在的虚假原产地索赔。 CBP的执法行动已经加快。 报告指出，自2025年</t>
+          <t>Evidence ID: WH_002 Title: The Great Transshipment Scam: Rise, Scope, and Costs（白宫非法转运报告） Publisher: 美国白宫贸易与制造业政策办公室 Country/Jurisdiction: US / Federal Publication date: 2026-08-13 Status: CURRENT Topic: 原产地与转运 Applicability scope: GENERAL Related industries: 通用 Key finding: 点名40</t>
         </is>
       </c>
     </row>
@@ -4380,44 +4380,44 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>RELOC_005</t>
+          <t>WH_001</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>欣旺达 Sunwoda：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>Executive Order 14411: Strengthening Customs Enforcement（加强海关执法行政令）</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>原产地与转运</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G51" s="2" t="n">
         <v>1</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J51" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>越南建厂案例，不提供执法判断 ｜ 人工判定与Auto(1)不同，请复核</t>
+          <t>EO14411 加强海关执法，直接回答执法趋势 ｜ 人工判定与Auto(1)不同，请复核</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>东方财富网 / 腾讯新闻</t>
+          <t>美国白宫</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
@@ -4442,7 +4442,7 @@
       </c>
       <c r="Q51" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RELOC_005 Title: 欣旺达 Sunwoda：中国 → 东南亚转移（多地区混合布局） Publisher: 东方财富网 / 腾讯新闻 Country/Jurisdiction: CN/VN Publication date: 2024-07-16 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池/消费电池 Claim: 2024-07-15 公告拟通过下属子公司香港欣威设立越南锂威有限公司，投建越南锂威</t>
+          <t>Evidence ID: WH_001 Title: Executive Order 14411: Strengthening Customs Enforcement（加强海关执法行政令） Publisher: 美国白宫 Country/Jurisdiction: US / Federal Publication date: 2026-06-03 Status: CURRENT Topic: 原产地与转运 Applicability scope: GENERAL Related industries: 通用 Key finding: 收紧进口商资质、保证</t>
         </is>
       </c>
     </row>
@@ -4534,17 +4534,17 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>RETURN_001</t>
+          <t>CNGOV_001</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份 Yunnan Energy New Material (Semcorp)：重新评估 / 回流中国（提高中国生产比例）</t>
+          <t>国务院关于对外投资的规定（国务院令第837号）</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>对外投资</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -4553,25 +4553,25 @@
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H53" s="2" t="n">
         <v>2</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J53" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>企业终止海外项目案例，可作立项风险的实例参考，但非制度/环境证据 ｜ 人工判定与Auto(0)不同，请复核</t>
+          <t>中国对外投资官方规则，直接</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份公告（经东方财富网 / 央广网报道）</t>
+          <t>中华人民共和国国务院</t>
         </is>
       </c>
       <c r="M53" s="2" t="inlineStr">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="Q53" s="2" t="inlineStr">
         <is>
-          <t>## 一、决策前状态（Initial Situation） 生产布局：湿法锂电隔膜产能以中国为主（上海、珠海、无锡等），为全球隔膜龙头。 主要市场：中国 + 海外电池客户（含欧美）。 供应链结构：基膜与涂覆材料主要在中国生产，产品出口海外。 面临的问题：2024 年规划马来西亚隔膜项目（约 10 亿平方米/年、投资约 20 亿元）以求贴近海外客户并规避关税。 ## 二、决策触发（Decision Trigger） 触发类型：cost_change（成本变化） 触发细节：外部市场环境及行业竞争格局发生变化（隔膜价格下行、行业产能过剩、海外建厂成本高于预期）</t>
+          <t>中华⼈⺠共和国国务院令中华⼈⺠共和国国务院令 第 837 号 《国务院关于对外投资的规定》已经2026年4⽉17⽇国务院第83次常务会议通过，现予公布，⾃2026年7⽉1⽇起施⾏。 总 理 李 强 2026年5⽉5⽇ 国务院关于对外投资的规定国务院关于对外投资的规定 第⼀条第⼀条 为了推进⾼⽔平对外开放，促进对外投资⾼质量发展，有效实施对外投资管理，保护投资者及其对外投资合法权益，维护国家主权、安全、发展利益，根据《中华⼈⺠共和国对外关系法》、《中华⼈⺠共和国对外贸易法》等法律，制定本规定。第⼆条第⼆条 中华⼈⺠共和国境内（以下简称中国境内）投资者对外投</t>
         </is>
       </c>
     </row>
@@ -4611,12 +4611,12 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>CNGOV_001</t>
+          <t>UNCTAD_001</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>国务院关于对外投资的规定（国务院令第837号）</t>
+          <t>World Investment Report 2026: International Investment in a Turbulent Era</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -4626,7 +4626,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="G54" s="2" t="n">
@@ -4643,12 +4643,12 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>中国对外投资官方规则，直接</t>
+          <t>世界投资报告，国际投资环境直接证据</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>中华人民共和国国务院</t>
+          <t>联合国贸易和发展会议（UNCTAD）</t>
         </is>
       </c>
       <c r="M54" s="2" t="inlineStr">
@@ -4673,7 +4673,7 @@
       </c>
       <c r="Q54" s="2" t="inlineStr">
         <is>
-          <t>中华⼈⺠共和国国务院令中华⼈⺠共和国国务院令 第 837 号 《国务院关于对外投资的规定》已经2026年4⽉17⽇国务院第83次常务会议通过，现予公布，⾃2026年7⽉1⽇起施⾏。 总 理 李 强 2026年5⽉5⽇ 国务院关于对外投资的规定国务院关于对外投资的规定 第⼀条第⼀条 为了推进⾼⽔平对外开放，促进对外投资⾼质量发展，有效实施对外投资管理，保护投资者及其对外投资合法权益，维护国家主权、安全、发展利益，根据《中华⼈⺠共和国对外关系法》、《中华⼈⺠共和国对外贸易法》等法律，制定本规定。第⼆条第⼆条 中华⼈⺠共和国境内（以下简称中国境内）投资者对外投</t>
+          <t>Evidence ID: UNCTAD_001 Title: World Investment Report 2026: International Investment in a Turbulent Era Publisher: 联合国贸易和发展会议（UNCTAD） Country/Jurisdiction: 全球 Publication date: 2026-07-07 Status: CURRENT Topic: 对外投资 Applicability scope: GENERAL Related industries: 通用 Key finding</t>
         </is>
       </c>
     </row>
@@ -4688,44 +4688,44 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>RETURN_004</t>
+          <t>WEF_001</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>蜂巢能源 SVOLT（欧洲业务）：重新评估 / 回流中国（维持现有海外布局（收缩新增））</t>
+          <t>Global Risks Report 2026（全球风险报告2026，第21版）</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>宏观风险</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="G55" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I55" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J55" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>企业终止欧洲业务，同为企业层面立项参考 ｜ 人工判定与Auto(0)不同，请复核</t>
+          <t>全球风险报告，宏观风险框架，非投资制度/环境证据</t>
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>36氪 / 财新网</t>
+          <t>世界经济论坛（WEF）</t>
         </is>
       </c>
       <c r="M55" s="2" t="inlineStr">
@@ -4750,7 +4750,7 @@
       </c>
       <c r="Q55" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RETURN_004 Title: 蜂巢能源 SVOLT（欧洲业务）：重新评估 / 回流中国（维持现有海外布局（收缩新增）） Publisher: 36氪 / 财新网 Country/Jurisdiction: CN/DE Publication date: 2024-10-28 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池 Claim: 2024-05 取消勃兰登堡州电芯超级工厂计划，2024-10 宣布停建</t>
+          <t>Lashley, Senior Fellow Don Marshall, Professor Kenisha Chase, Research Assistant Benin Institut de Recherche Empirique en Economie Politique - IREEP Leonard Wantchekon, President Stéphania Houngan, Research Associate Bolivia (Plurinational State of), Costa Rica, Dominican Republi</t>
         </is>
       </c>
     </row>
@@ -4765,12 +4765,12 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>RELOC_004</t>
+          <t>CASE_001</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>亿纬锂能 EVE Energy：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>Dawang Metals：客户订单转移印度后回流，企业放弃海外建厂</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -4797,12 +4797,12 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>企业海外建厂案例，同为企业层面立项参考 ｜ 人工判定与Auto(0)不同，请复核</t>
+          <t>企业放弃海外建厂个案，可作立项风险实例，非制度/环境证据 ｜ 人工判定与Auto(0)不同，请复核</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>新浪财经</t>
+          <t>路透社（Reuters）</t>
         </is>
       </c>
       <c r="M56" s="2" t="inlineStr">
@@ -4827,7 +4827,7 @@
       </c>
       <c r="Q56" s="2" t="inlineStr">
         <is>
-          <t>## 二、决策触发（Decision Trigger） 触发类型：tariff_pressure（关税压力） 触发细节：对美出口关税与'去中国化'供应链要求，迫使企业在东南亚布局产能以规避税率。 ## 三、实际决策（Actual Decision） 决策分类：多地区混合布局 决策内容：在马来西亚吉打州居林县建设海外工厂，二期于 2026 年 2 月投产运营，建筑面积约 60 万平方米，系公司首个海外大型锂电厂房项目，形成年产约 6.8 亿只圆柱电池产能；同时推进匈牙利、美国、印尼项目，中国产能保留。 ## 四、相关风险（Related Risk） 风险类</t>
+          <t>Evidence ID: CASE_001 Title: Dawang Metals：客户订单转移印度后回流，企业放弃海外建厂 Publisher: 路透社（Reuters） Country/Jurisdiction: CN / National Publication date: 2026-09-14 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 金属铸造 Key finding: 路透原文《Companies left China to do</t>
         </is>
       </c>
     </row>
@@ -5073,22 +5073,22 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>RETURN_001</t>
+          <t>TRD_003</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份 Yunnan Energy New Material (Semcorp)：重新评估 / 回流中国（提高中国生产比例）</t>
+          <t>中国对越南、泰国、马来西亚出口 HS 8541/8542（中间品），2018–2025年度</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>贸易流</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="G60" s="2" t="n">
@@ -5098,19 +5098,19 @@
         <v>2</v>
       </c>
       <c r="I60" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J60" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>企业个案，与碎片化趋势判断无关</t>
+          <t>UN Comtrade 贸易流数据，可作碎片化趋势间接佐证，非投资判断证据 ｜ 人工判定与Auto(0)不同，请复核</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份公告（经东方财富网 / 央广网报道）</t>
+          <t>联合国商品贸易统计数据库（UN Comtrade）</t>
         </is>
       </c>
       <c r="M60" s="2" t="inlineStr">
@@ -5135,7 +5135,7 @@
       </c>
       <c r="Q60" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RETURN_001 Title: 恩捷股份 Yunnan Energy New Material (Semcorp)：重新评估 / 回流中国（提高中国生产比例） Publisher: 恩捷股份公告（经东方财富网 / 央广网报道） Country/Jurisdiction: CN/MY Publication date: 2026-05-22 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 电池材料 Claim: 2026</t>
+          <t>Evidence ID: TRD_003 Title: 中国对越南、泰国、马来西亚出口 HS 8541/8542（中间品），2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: CN / National Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: ◆电子/光电 Key finding: 看东南亚产能是否依赖中国中间</t>
         </is>
       </c>
     </row>
@@ -5150,12 +5150,12 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>RELOC_005</t>
+          <t>CASE_007</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>欣旺达 Sunwoda：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>华工正源：马来西亚工厂，公开表述为规避地缘风险</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -5182,12 +5182,12 @@
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>企业建厂案例，与趋势判断无关</t>
+          <t>企业个案，与地缘经济碎片化趋势判断无关</t>
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>东方财富网 / 腾讯新闻</t>
+          <t>C114通信网</t>
         </is>
       </c>
       <c r="M61" s="2" t="inlineStr">
@@ -5212,7 +5212,7 @@
       </c>
       <c r="Q61" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RELOC_005 Title: 欣旺达 Sunwoda：中国 → 东南亚转移（多地区混合布局） Publisher: 东方财富网 / 腾讯新闻 Country/Jurisdiction: CN/VN Publication date: 2024-07-16 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池/消费电池 Claim: 2024-07-15 公告拟通过下属子公司香港欣威设立越南锂威有限公司，投建越南锂威</t>
+          <t>资讯 视频 6G 光通信 物联网 量子通信 卫星互联网 数智低空 Cloud&amp;AI 政策 运营商 设备商 终端 财经 市场 会展 直播 2026/3/25 16:29 2026十大光模块厂商，光模块厂商有哪些 C114通信网 26 1 2026年，随着 AI 算力需求持续爆发与全球数据中心带宽升级加速，光模块行业迎来“800G普及+1. 6T放量”的双轮驱动阶段。 据行业预测，2026年全球800G光模块需求量有望突破4000万只，1. 6T需求亦进入商业化元年。 在这场高速光互联的竞逐中，中国光模块厂商凭借技术突破与产能优势占据全球主导地位。 本文综合</t>
         </is>
       </c>
     </row>
@@ -5304,44 +5304,44 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>RETURN_004</t>
+          <t>IMF_001</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>蜂巢能源 SVOLT（欧洲业务）：重新评估 / 回流中国（维持现有海外布局（收缩新增））</t>
+          <t>World Economic Outlook, April 2023, Chapter 4: Geoeconomic Fragmentation and Foreign Direct Investment</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>对外投资</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I63" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J63" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>企业欧洲布局收缩，可作不确定性的具体例证，但非高权威全球证据</t>
+          <t>FDI与地缘经济碎片化框架，直接</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>36氪 / 财新网</t>
+          <t>国际货币基金组织（IMF）</t>
         </is>
       </c>
       <c r="M63" s="2" t="inlineStr">
@@ -5366,7 +5366,7 @@
       </c>
       <c r="Q63" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RETURN_004 Title: 蜂巢能源 SVOLT（欧洲业务）：重新评估 / 回流中国（维持现有海外布局（收缩新增）） Publisher: 36氪 / 财新网 Country/Jurisdiction: CN/DE Publication date: 2024-10-28 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池 Claim: 2024-05 取消勃兰登堡州电芯超级工厂计划，2024-10 宣布停建</t>
+          <t>Evidence ID: IMF_001 Title: World Economic Outlook, April 2023, Chapter 4: Geoeconomic Fragmentation and Foreign Direct Investment Publisher: 国际货币基金组织（IMF） Country/Jurisdiction: 全球 Publication date: 2023-04 Status: CURRENT Topic: 对外投资 Applicability scope: GENERAL Related industri</t>
         </is>
       </c>
     </row>
@@ -5381,17 +5381,17 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>IMF_001</t>
+          <t>WTO_001</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>World Economic Outlook, April 2023, Chapter 4: Geoeconomic Fragmentation and Foreign Direct Investment</t>
+          <t>Global Trade Outlook and Statistics（2026年3月版）</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>对外投资</t>
+          <t>贸易流</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -5413,12 +5413,12 @@
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>FDI与地缘经济碎片化框架，直接</t>
+          <t>货物贸易增速放缓，直接</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>国际货币基金组织（IMF）</t>
+          <t>世界贸易组织（WTO）</t>
         </is>
       </c>
       <c r="M64" s="2" t="inlineStr">
@@ -5443,7 +5443,7 @@
       </c>
       <c r="Q64" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: IMF_001 Title: World Economic Outlook, April 2023, Chapter 4: Geoeconomic Fragmentation and Foreign Direct Investment Publisher: 国际货币基金组织（IMF） Country/Jurisdiction: 全球 Publication date: 2023-04 Status: CURRENT Topic: 对外投资 Applicability scope: GENERAL Related industri</t>
+          <t>Evidence ID: WTO_001 Title: Global Trade Outlook and Statistics（2026年3月版） Publisher: 世界贸易组织（WTO） Country/Jurisdiction: 全球 Publication date: 2026-03 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: 通用 Key finding: 基准情景下2026年货物贸易量增速由2025年的4.6%放缓至1.9%。 Glo</t>
         </is>
       </c>
     </row>
@@ -5458,44 +5458,44 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>RETURN_001</t>
+          <t>WEF_001</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份 Yunnan Energy New Material (Semcorp)：重新评估 / 回流中国（提高中国生产比例）</t>
+          <t>Global Risks Report 2026（全球风险报告2026，第21版）</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>宏观风险</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="G65" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H65" s="2" t="n">
         <v>2</v>
       </c>
       <c r="I65" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J65" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>企业终止海外项目，同为例证，非宏观证据</t>
+          <t>全球风险报告将地缘经济对抗列为首要风险，直接支撑判断</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份公告（经东方财富网 / 央广网报道）</t>
+          <t>世界经济论坛（WEF）</t>
         </is>
       </c>
       <c r="M65" s="2" t="inlineStr">
@@ -5520,7 +5520,7 @@
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>## 一、决策前状态（Initial Situation） 生产布局：湿法锂电隔膜产能以中国为主（上海、珠海、无锡等），为全球隔膜龙头。 主要市场：中国 + 海外电池客户（含欧美）。 供应链结构：基膜与涂覆材料主要在中国生产，产品出口海外。 面临的问题：2024 年规划马来西亚隔膜项目（约 10 亿平方米/年、投资约 20 亿元）以求贴近海外客户并规避关税。 ## 二、决策触发（Decision Trigger） 触发类型：cost_change（成本变化） 触发细节：外部市场环境及行业竞争格局发生变化（隔膜价格下行、行业产能过剩、海外建厂成本高于预期）</t>
+          <t>Evidence ID: WEF_001 Title: Global Risks Report 2026（全球风险报告2026，第21版） Publisher: 世界经济论坛（WEF） Country/Jurisdiction: 全球 Publication date: 2026-01-14 Status: CURRENT Topic: 宏观风险 Applicability scope: GENERAL Related industries: 通用 Key finding: 地缘经济对抗列为2026年首要风险。仅作PPT背景。</t>
         </is>
       </c>
     </row>
@@ -5535,22 +5535,22 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>WTO_001</t>
+          <t>MCK_001</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Global Trade Outlook and Statistics（2026年3月版）</t>
+          <t>The art, science, and technology of geopolitical scenario planning</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>贸易流</t>
+          <t>宏观风险</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>A+</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G66" s="2" t="n">
@@ -5567,12 +5567,12 @@
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>货物贸易增速放缓，直接</t>
+          <t>地缘政治情景规划方法，直接支撑海外布局不确定性分析</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>世界贸易组织（WTO）</t>
+          <t>麦肯锡（McKinsey）</t>
         </is>
       </c>
       <c r="M66" s="2" t="inlineStr">
@@ -5597,7 +5597,7 @@
       </c>
       <c r="Q66" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: WTO_001 Title: Global Trade Outlook and Statistics（2026年3月版） Publisher: 世界贸易组织（WTO） Country/Jurisdiction: 全球 Publication date: 2026-03 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: 通用 Key finding: 基准情景下2026年货物贸易量增速由2025年的4.6%放缓至1.9%。 Glo</t>
+          <t>Evidence ID: MCK_001 Title: The art, science, and technology of geopolitical scenario planning Publisher: 麦肯锡（McKinsey） Country/Jurisdiction: 全球 Publication date: 2026-06-10 Status: CURRENT Topic: 宏观风险 Applicability scope: GENERAL Related industries: 通用 Key finding: 基于2026年2月对202</t>
         </is>
       </c>
     </row>
@@ -6459,44 +6459,44 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>RELOC_006</t>
+          <t>TRD_003</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>蜂巢能源 SVOLT：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>中国对越南、泰国、马来西亚出口 HS 8541/8542（中间品），2018–2025年度</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>贸易流</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="G78" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I78" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J78" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>泰国电池厂案例，佐证产能转移，非贸易数据</t>
+          <t>中国对越/泰/马中间品出口，直接</t>
         </is>
       </c>
       <c r="L78" s="2" t="inlineStr">
         <is>
-          <t>澎湃新闻</t>
+          <t>联合国商品贸易统计数据库（UN Comtrade）</t>
         </is>
       </c>
       <c r="M78" s="2" t="inlineStr">
@@ -6521,7 +6521,7 @@
       </c>
       <c r="Q78" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RELOC_006 Title: 蜂巢能源 SVOLT：中国 → 东南亚转移（多地区混合布局） Publisher: 澎湃新闻 Country/Jurisdiction: CN/TH Publication date: 2024-02-28 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池 Claim: 在泰国春武里府是拉差市建设电池工厂（模组 PACK + 电芯），2024-02-28 正式投产并批量交付，配套长</t>
+          <t>Evidence ID: TRD_003 Title: 中国对越南、泰国、马来西亚出口 HS 8541/8542（中间品），2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: CN / National Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: ◆电子/光电 Key finding: 看东南亚产能是否依赖中国中间</t>
         </is>
       </c>
     </row>
@@ -6536,44 +6536,44 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>RELOC_003</t>
+          <t>WH_002</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>国轩高科 Gotion High-Tech：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>The Great Transshipment Scam: Rise, Scope, and Costs（白宫非法转运报告）</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>原产地与转运</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G79" s="2" t="n">
         <v>1</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I79" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J79" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K79" s="2" t="inlineStr">
         <is>
-          <t>越南电池厂案例，佐证产能转移</t>
+          <t>白宫非法转运报告，供应链迁移相关政策证据直接来源 ｜ 人工判定与Auto(1)不同，请复核</t>
         </is>
       </c>
       <c r="L79" s="2" t="inlineStr">
         <is>
-          <t>澎湃新闻 / 盖世汽车社区</t>
+          <t>美国白宫贸易与制造业政策办公室</t>
         </is>
       </c>
       <c r="M79" s="2" t="inlineStr">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="Q79" s="2" t="inlineStr">
         <is>
-          <t>## 一、决策前状态（Initial Situation） 生产布局：电芯产能集中于中国（合肥、庐江、南京等基地），海外仅有销售与研发。 主要市场：中国动力电池市场为主，海外客户（大众等）快速增加。 供应链结构：正极、负极、隔膜主要来自中国供应商，磷酸铁锂（LFP）技术路线自主。 面临的问题：整车客户在东南亚建厂后要求就近配套；纯从中国出口电池面临关税与交期风险，且越南本地无 LFP 电芯产能。 ## 二、决策触发（Decision Trigger） 触发类型：market_access（市场准入） 触发细节：越南 VinFast 本地化生产需要就近电池</t>
+          <t>Evidence ID: WH_002 Title: The Great Transshipment Scam: Rise, Scope, and Costs（白宫非法转运报告） Publisher: 美国白宫贸易与制造业政策办公室 Country/Jurisdiction: US / Federal Publication date: 2026-08-13 Status: CURRENT Topic: 原产地与转运 Applicability scope: GENERAL Related industries: 通用 Key finding: 点名40</t>
         </is>
       </c>
     </row>
@@ -6613,44 +6613,44 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>RELOC_004</t>
+          <t>TRD_002</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>亿纬锂能 EVE Energy：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>美国自越南、泰国、马来西亚、柬埔寨进口光伏组件HS 854140，2018–2025年度</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>贸易流</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="G80" s="2" t="n">
         <v>1</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I80" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J80" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t>马来西亚电池厂案例，佐证产能转移</t>
+          <t>同区域同模式的贸易转移数据（光伏组件），可作模式类比，非EV/电池口径</t>
         </is>
       </c>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t>新浪财经</t>
+          <t>联合国商品贸易统计数据库（UN Comtrade）</t>
         </is>
       </c>
       <c r="M80" s="2" t="inlineStr">
@@ -6675,7 +6675,7 @@
       </c>
       <c r="Q80" s="2" t="inlineStr">
         <is>
-          <t>## 二、决策触发（Decision Trigger） 触发类型：tariff_pressure（关税压力） 触发细节：对美出口关税与'去中国化'供应链要求，迫使企业在东南亚布局产能以规避税率。 ## 三、实际决策（Actual Decision） 决策分类：多地区混合布局 决策内容：在马来西亚吉打州居林县建设海外工厂，二期于 2026 年 2 月投产运营，建筑面积约 60 万平方米，系公司首个海外大型锂电厂房项目，形成年产约 6.8 亿只圆柱电池产能；同时推进匈牙利、美国、印尼项目，中国产能保留。 ## 四、相关风险（Related Risk） 风险类</t>
+          <t>Evidence ID: TRD_002 Title: 美国自越南、泰国、马来西亚、柬埔寨进口光伏组件HS 854140，2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: US / Federal Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: ◆光伏 Key finding: HS 2022版起光伏组件编码调整（旧</t>
         </is>
       </c>
     </row>
@@ -6690,44 +6690,44 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>TRD_003</t>
+          <t>CASE_003</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>中国对越南、泰国、马来西亚出口 HS 8541/8542（中间品），2018–2025年度</t>
+          <t>同一反规避调查中被认定“未规避”的企业（Hanwha、Jinko马来西亚、Boviet越南）</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>贸易流</t>
+          <t>反规避</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>A+</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G81" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
         <v>2</v>
       </c>
       <c r="I81" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J81" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K81" s="2" t="inlineStr">
         <is>
-          <t>中国对越/泰/马中间品出口，直接</t>
+          <t>反规避「未规避」判例，涉及区域原产地认定，间接相关 ｜ 人工判定与Auto(0)不同，请复核</t>
         </is>
       </c>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t>联合国商品贸易统计数据库（UN Comtrade）</t>
+          <t>美国商务部（经律所解读）</t>
         </is>
       </c>
       <c r="M81" s="2" t="inlineStr">
@@ -6752,7 +6752,7 @@
       </c>
       <c r="Q81" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: TRD_003 Title: 中国对越南、泰国、马来西亚出口 HS 8541/8542（中间品），2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: CN / National Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: ◆电子/光电 Key finding: 看东南亚产能是否依赖中国中间</t>
+          <t>Evidence ID: CASE_003 Title: 同一反规避调查中被认定“未规避”的企业（Hanwha、Jinko马来西亚、Boviet越南） Publisher: 美国商务部（经律所解读） Country/Jurisdiction: 马来西亚/越南 Publication date: 2023-08-18 Status: CURRENT Topic: 反规避 Applicability scope: GENERAL Related industries: 光伏 Key finding: 与CASE_002构成对照：同一规则下，供应链结构不同导致</t>
         </is>
       </c>
     </row>
@@ -6921,44 +6921,44 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>RELOC_005</t>
+          <t>WH_002</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>欣旺达 Sunwoda：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>The Great Transshipment Scam: Rise, Scope, and Costs（白宫非法转运报告）</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>原产地与转运</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G84" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I84" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J84" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K84" s="2" t="inlineStr">
         <is>
-          <t>欣旺达越南基地：越南建厂但仍依赖中国材料，依赖例证</t>
+          <t>非法转运报告，原产地风险直接</t>
         </is>
       </c>
       <c r="L84" s="2" t="inlineStr">
         <is>
-          <t>东方财富网 / 腾讯新闻</t>
+          <t>美国白宫贸易与制造业政策办公室</t>
         </is>
       </c>
       <c r="M84" s="2" t="inlineStr">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="Q84" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RELOC_005 Title: 欣旺达 Sunwoda：中国 → 东南亚转移（多地区混合布局） Publisher: 东方财富网 / 腾讯新闻 Country/Jurisdiction: CN/VN Publication date: 2024-07-16 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池/消费电池 Claim: 2024-07-15 公告拟通过下属子公司香港欣威设立越南锂威有限公司，投建越南锂威</t>
+          <t>Evidence ID: WH_002 Title: The Great Transshipment Scam: Rise, Scope, and Costs（白宫非法转运报告） Publisher: 美国白宫贸易与制造业政策办公室 Country/Jurisdiction: US / Federal Publication date: 2026-08-13 Status: CURRENT Topic: 原产地与转运 Applicability scope: GENERAL Related industries: 通用 Key finding: 点名40</t>
         </is>
       </c>
     </row>
@@ -6998,44 +6998,44 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>RELOC_003</t>
+          <t>WTO_001</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>国轩高科 Gotion High-Tech：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>Global Trade Outlook and Statistics（2026年3月版）</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>贸易流</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="G85" s="2" t="n">
         <v>1</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I85" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J85" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K85" s="2" t="inlineStr">
         <is>
-          <t>国轩高科越南基地：正负极材料仍来自中国，依赖例证</t>
+          <t>全球贸易展望，提供背景但非中间品依赖/原产地风险的直接证据</t>
         </is>
       </c>
       <c r="L85" s="2" t="inlineStr">
         <is>
-          <t>澎湃新闻 / 盖世汽车社区</t>
+          <t>世界贸易组织（WTO）</t>
         </is>
       </c>
       <c r="M85" s="2" t="inlineStr">
@@ -7060,7 +7060,7 @@
       </c>
       <c r="Q85" s="2" t="inlineStr">
         <is>
-          <t>## 一、决策前状态（Initial Situation） 生产布局：电芯产能集中于中国（合肥、庐江、南京等基地），海外仅有销售与研发。 主要市场：中国动力电池市场为主，海外客户（大众等）快速增加。 供应链结构：正极、负极、隔膜主要来自中国供应商，磷酸铁锂（LFP）技术路线自主。 面临的问题：整车客户在东南亚建厂后要求就近配套；纯从中国出口电池面临关税与交期风险，且越南本地无 LFP 电芯产能。 ## 二、决策触发（Decision Trigger） 触发类型：market_access（市场准入） 触发细节：越南 VinFast 本地化生产需要就近电池</t>
+          <t>35 Appendix Table 1: Leading exporters and importers in world merchandise trade, 2025 (Billion dollars and percentage) Rank Exporters Value Share Annual percentage change Rank Importers Value Share Annual percentage change 1 China 3,772 14. 4 5 1 United States of America 3,507 13</t>
         </is>
       </c>
     </row>
@@ -7075,12 +7075,12 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>WH_002</t>
+          <t>CSIS_001</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>The Great Transshipment Scam: Rise, Scope, and Costs（白宫非法转运报告）</t>
+          <t>The Visibility Gap: How AI Can Stop Chinese Transshipment Under USMCA</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -7090,7 +7090,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G86" s="2" t="n">
@@ -7107,12 +7107,12 @@
       </c>
       <c r="K86" s="2" t="inlineStr">
         <is>
-          <t>非法转运报告，原产地风险直接</t>
+          <t>转运可见性分析，直接支持原产地风险判断</t>
         </is>
       </c>
       <c r="L86" s="2" t="inlineStr">
         <is>
-          <t>美国白宫贸易与制造业政策办公室</t>
+          <t>战略与国际研究中心（CSIS）</t>
         </is>
       </c>
       <c r="M86" s="2" t="inlineStr">
@@ -7137,7 +7137,7 @@
       </c>
       <c r="Q86" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: WH_002 Title: The Great Transshipment Scam: Rise, Scope, and Costs（白宫非法转运报告） Publisher: 美国白宫贸易与制造业政策办公室 Country/Jurisdiction: US / Federal Publication date: 2026-08-13 Status: CURRENT Topic: 原产地与转运 Applicability scope: GENERAL Related industries: 通用 Key finding: 点名40</t>
+          <t>Evidence ID: CSIS_001 Title: The Visibility Gap: How AI Can Stop Chinese Transshipment Under USMCA Publisher: 战略与国际研究中心（CSIS） Country/Jurisdiction: US / Federal Publication date: 2026-08 Status: CURRENT Topic: 原产地与转运 Applicability scope: GENERAL Related industries: 通用 Key finding</t>
         </is>
       </c>
     </row>
@@ -7152,44 +7152,44 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>RELOC_005</t>
+          <t>TRD_003</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>欣旺达 Sunwoda：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>中国对越南、泰国、马来西亚出口 HS 8541/8542（中间品），2018–2025年度</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>贸易流</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="G87" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I87" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J87" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K87" s="2" t="inlineStr">
         <is>
-          <t>越南仅承担电芯制造、材料仍由中国供应，支持“未隔离风险”</t>
+          <t>中国对东南亚中间品出口数据，直接支撑「依赖未隔离」判断</t>
         </is>
       </c>
       <c r="L87" s="2" t="inlineStr">
         <is>
-          <t>东方财富网 / 腾讯新闻</t>
+          <t>联合国商品贸易统计数据库（UN Comtrade）</t>
         </is>
       </c>
       <c r="M87" s="2" t="inlineStr">
@@ -7204,7 +7204,7 @@
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_002; CASE_003; CASE_008; TRD_003; RELOC_001; RELOC_003; RELOC_006; RETURN_001</t>
+          <t>CASE_001; CASE_002; CASE_003; CASE_008; TRD_003</t>
         </is>
       </c>
       <c r="P87" s="2" t="inlineStr">
@@ -7214,7 +7214,7 @@
       </c>
       <c r="Q87" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RELOC_005 Title: 欣旺达 Sunwoda：中国 → 东南亚转移（多地区混合布局） Publisher: 东方财富网 / 腾讯新闻 Country/Jurisdiction: CN/VN Publication date: 2024-07-16 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池/消费电池 Claim: 2024-07-15 公告拟通过下属子公司香港欣威设立越南锂威有限公司，投建越南锂威</t>
+          <t>Evidence ID: TRD_003 Title: 中国对越南、泰国、马来西亚出口 HS 8541/8542（中间品），2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: CN / National Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: ◆电子/光电 Key finding: 看东南亚产能是否依赖中国中间</t>
         </is>
       </c>
     </row>
@@ -7229,44 +7229,44 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>RELOC_006</t>
+          <t>CASE_002</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>蜂巢能源 SVOLT：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>美国对东南亚四国光伏产品反规避认定：视为中国原产并适用对华双反</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>反规避</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G88" s="2" t="n">
         <v>2</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I88" s="3" t="n">
         <v>2</v>
       </c>
       <c r="J88" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K88" s="2" t="inlineStr">
         <is>
-          <t>泰国仅承担模组PACK、电芯材料仍从中国输入，直接支持</t>
+          <t>反规避「认定规避」，直接支撑风险未隔离</t>
         </is>
       </c>
       <c r="L88" s="2" t="inlineStr">
         <is>
-          <t>澎湃新闻</t>
+          <t>美国商务部（经律所解读）</t>
         </is>
       </c>
       <c r="M88" s="2" t="inlineStr">
@@ -7281,7 +7281,7 @@
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_002; CASE_003; CASE_008; TRD_003; RELOC_001; RELOC_003; RELOC_006; RETURN_001</t>
+          <t>CASE_001; CASE_002; CASE_003; CASE_008; TRD_003</t>
         </is>
       </c>
       <c r="P88" s="2" t="inlineStr">
@@ -7291,7 +7291,7 @@
       </c>
       <c r="Q88" s="2" t="inlineStr">
         <is>
-          <t>## 三、实际决策（Actual Decision） 决策分类：多地区混合布局 决策内容：在泰国春武里府是拉差市建设电池工厂（模组 PACK + 电芯），2024-02-28 正式投产并批量交付，配套长城欧拉、合众/哪吒等中国车企在泰车型；当年计划交付超 2 万套 PACK；中国产能保留。 ## 四、相关风险（Related Risk） 风险类别：Trade Risk; Market Access Risk; Operational Risk ## 五、后续结果（Outcome） 成本影响：本地 PACK 组装降低关税与物流成本，投资规模小于整线电芯厂。</t>
+          <t>Evidence ID: CASE_002 Title: 美国对东南亚四国光伏产品反规避认定：视为中国原产并适用对华双反 Publisher: 美国商务部（经律所解读） Country/Jurisdiction: 柬埔寨/马来西亚/泰国/越南 Publication date: 2023-08-18 Status: CURRENT Topic: 反规避 Applicability scope: GENERAL Related industries: 光伏 Key finding: 2022年4月立案，2023年8月终裁。使用中国组件在东南亚完成的电池和组</t>
         </is>
       </c>
     </row>
@@ -7306,12 +7306,12 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>RELOC_004</t>
+          <t>CASE_008</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>亿纬锂能 EVE Energy：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>光模块厂商选择东南亚建厂以规避与欧美客户合作风险（中际旭创互动平台回复等）</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -7325,25 +7325,25 @@
         </is>
       </c>
       <c r="G89" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H89" s="2" t="n">
         <v>1</v>
       </c>
       <c r="I89" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J89" s="3" t="n">
         <v>1</v>
       </c>
       <c r="K89" s="2" t="inlineStr">
         <is>
-          <t>材料仍由中国输入，例证</t>
+          <t>东南亚建厂规避欧美客户风险，直接案例</t>
         </is>
       </c>
       <c r="L89" s="2" t="inlineStr">
         <is>
-          <t>新浪财经</t>
+          <t>中国基金报</t>
         </is>
       </c>
       <c r="M89" s="2" t="inlineStr">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_002; CASE_003; CASE_008; TRD_003; RELOC_001; RELOC_003; RELOC_006; RETURN_001</t>
+          <t>CASE_001; CASE_002; CASE_003; CASE_008; TRD_003</t>
         </is>
       </c>
       <c r="P89" s="2" t="inlineStr">
@@ -7368,7 +7368,7 @@
       </c>
       <c r="Q89" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RELOC_004 Title: 亿纬锂能 EVE Energy：中国 → 东南亚转移（多地区混合布局） Publisher: 新浪财经 Country/Jurisdiction: CN/MY Publication date: 2026-02-06 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池/储能 Claim: 在马来西亚吉打州居林县建设海外工厂，二期于 2026 年 2 月投产运营，建筑面积约 60 万平</t>
+          <t>Evidence ID: CASE_008 Title: 光模块厂商选择东南亚建厂以规避与欧美客户合作风险（中际旭创互动平台回复等） Publisher: 中国基金报 Country/Jurisdiction: CN / National Publication date: 2024-07-14 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 光模块 Key finding: 文中引用中际旭创互动平台回复，可据此到互动易查原始问答，升级为一手证据。</t>
         </is>
       </c>
     </row>
@@ -7383,22 +7383,22 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>RELOC_002</t>
+          <t>TRD_001</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>长安汽车 Changan Automobile：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>贸易流</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="G90" s="2" t="n">
@@ -7415,12 +7415,12 @@
       </c>
       <c r="K90" s="2" t="inlineStr">
         <is>
-          <t>零部件本地化仍在爬坡、依赖中泰跨境供应，例证</t>
+          <t>美国进口贸易数据，可作布局结果佐证，非风险隔离证据</t>
         </is>
       </c>
       <c r="L90" s="2" t="inlineStr">
         <is>
-          <t>易车 / 证券之星（投资者互动平台）</t>
+          <t>联合国商品贸易统计数据库（UN Comtrade）</t>
         </is>
       </c>
       <c r="M90" s="2" t="inlineStr">
@@ -7435,7 +7435,7 @@
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_002; CASE_003; CASE_008; TRD_003; RELOC_001; RELOC_003; RELOC_006; RETURN_001</t>
+          <t>CASE_001; CASE_002; CASE_003; CASE_008; TRD_003</t>
         </is>
       </c>
       <c r="P90" s="2" t="inlineStr">
@@ -7445,7 +7445,7 @@
       </c>
       <c r="Q90" s="2" t="inlineStr">
         <is>
-          <t>## 二、决策触发（Decision Trigger） 触发类型：market_access（市场准入） 触发细节：泰国 EV3.5 补贴政策要求本地生产，才能享受补贴与关税优惠。 ## 三、实际决策（Actual Decision） 决策分类：多地区混合布局 决策内容：在泰国罗勇府建设整车工厂，2025-05-16 竣工投产，全球累计第 2859 万辆（深蓝 S05）在泰下线；中国产能保留。 ## 四、相关风险（Related Risk） 风险类别：Trade Risk; Market Access Risk; Operational Risk ##</t>
+          <t>Evidence ID: TRD_001 Title: 美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: US / Federal Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: ◆电子/光电 Key finding: HS 851762仅为光</t>
         </is>
       </c>
     </row>
@@ -7460,12 +7460,12 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>RETURN_001</t>
+          <t>CASE_001</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份 Yunnan Energy New Material (Semcorp)：重新评估 / 回流中国（提高中国生产比例）</t>
+          <t>Dawang Metals：客户订单转移印度后回流，企业放弃海外建厂</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -7475,29 +7475,29 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="G91" s="2" t="n">
         <v>2</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I91" s="3" t="n">
         <v>2</v>
       </c>
       <c r="J91" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K91" s="2" t="inlineStr">
         <is>
-          <t>终止海外项目、对单一中国基地依赖上升，直接说明风险未隔离</t>
+          <t>订单转移印度后回流，直接说明海外迁移未达预期</t>
         </is>
       </c>
       <c r="L91" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份公告（经东方财富网 / 央广网报道）</t>
+          <t>路透社（Reuters）</t>
         </is>
       </c>
       <c r="M91" s="2" t="inlineStr">
@@ -7512,7 +7512,7 @@
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_002; CASE_003; CASE_008; TRD_003; RELOC_001; RELOC_003; RELOC_006; RETURN_001</t>
+          <t>CASE_001; CASE_002; CASE_003; CASE_008; TRD_003</t>
         </is>
       </c>
       <c r="P91" s="2" t="inlineStr">
@@ -7522,7 +7522,7 @@
       </c>
       <c r="Q91" s="2" t="inlineStr">
         <is>
-          <t>## 一、决策前状态（Initial Situation） 生产布局：湿法锂电隔膜产能以中国为主（上海、珠海、无锡等），为全球隔膜龙头。 主要市场：中国 + 海外电池客户（含欧美）。 供应链结构：基膜与涂覆材料主要在中国生产，产品出口海外。 面临的问题：2024 年规划马来西亚隔膜项目（约 10 亿平方米/年、投资约 20 亿元）以求贴近海外客户并规避关税。 ## 二、决策触发（Decision Trigger） 触发类型：cost_change（成本变化） 触发细节：外部市场环境及行业竞争格局发生变化（隔膜价格下行、行业产能过剩、海外建厂成本高于预期）</t>
+          <t>Evidence ID: CASE_001 Title: Dawang Metals：客户订单转移印度后回流，企业放弃海外建厂 Publisher: 路透社（Reuters） Country/Jurisdiction: CN / National Publication date: 2026-09-14 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 金属铸造 Key finding: 路透原文《Companies left China to do</t>
         </is>
       </c>
     </row>
@@ -7537,12 +7537,12 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>RELOC_005</t>
+          <t>CASE_001</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>欣旺达 Sunwoda：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>Dawang Metals：客户订单转移印度后回流，企业放弃海外建厂</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -7556,7 +7556,7 @@
         </is>
       </c>
       <c r="G92" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H92" s="2" t="n">
         <v>1</v>
@@ -7569,12 +7569,12 @@
       </c>
       <c r="K92" s="2" t="inlineStr">
         <is>
-          <t>欣旺达越南扩产，供应链布局调整的直接案例 ｜ 人工判定与Auto(1)不同，请复核</t>
+          <t>订单回流、放弃海外建厂，直接说明布局调整与执行风险</t>
         </is>
       </c>
       <c r="L92" s="2" t="inlineStr">
         <is>
-          <t>东方财富网 / 腾讯新闻</t>
+          <t>路透社（Reuters）</t>
         </is>
       </c>
       <c r="M92" s="2" t="inlineStr">
@@ -7589,7 +7589,7 @@
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_004; CASE_005; CASE_006; CASE_008; KPMG_001; PLUS1_001; PLUS1_002; RELOC_001</t>
+          <t>CASE_001; CASE_004; CASE_005; CASE_006; CASE_008; KPMG_001</t>
         </is>
       </c>
       <c r="P92" s="2" t="inlineStr">
@@ -7599,7 +7599,7 @@
       </c>
       <c r="Q92" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RELOC_005 Title: 欣旺达 Sunwoda：中国 → 东南亚转移（多地区混合布局） Publisher: 东方财富网 / 腾讯新闻 Country/Jurisdiction: CN/VN Publication date: 2024-07-16 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池/消费电池 Claim: 2024-07-15 公告拟通过下属子公司香港欣威设立越南锂威有限公司，投建越南锂威</t>
+          <t>Evidence ID: CASE_001 Title: Dawang Metals：客户订单转移印度后回流，企业放弃海外建厂 Publisher: 路透社（Reuters） Country/Jurisdiction: CN / National Publication date: 2026-09-14 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 金属铸造 Key finding: 路透原文《Companies left China to do</t>
         </is>
       </c>
     </row>
@@ -7614,12 +7614,12 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>RETURN_001</t>
+          <t>KPMG_001</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份 Yunnan Energy New Material (Semcorp)：重新评估 / 回流中国（提高中国生产比例）</t>
+          <t>KPMG 2026 US Supply Chain Survey</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -7629,11 +7629,11 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G93" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H93" s="2" t="n">
         <v>2</v>
@@ -7646,12 +7646,12 @@
       </c>
       <c r="K93" s="2" t="inlineStr">
         <is>
-          <t>终止海外项目、资源回投国内，直接说明执行风险 ｜ 人工判定与Auto(1)不同，请复核</t>
+          <t>KPMG供应链调查，直接提供企业执行风险证据</t>
         </is>
       </c>
       <c r="L93" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份公告（经东方财富网 / 央广网报道）</t>
+          <t>毕马威（KPMG）</t>
         </is>
       </c>
       <c r="M93" s="2" t="inlineStr">
@@ -7666,7 +7666,7 @@
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_004; CASE_005; CASE_006; CASE_008; KPMG_001; PLUS1_001; PLUS1_002; RELOC_001</t>
+          <t>CASE_001; CASE_004; CASE_005; CASE_006; CASE_008; KPMG_001</t>
         </is>
       </c>
       <c r="P93" s="2" t="inlineStr">
@@ -7676,7 +7676,7 @@
       </c>
       <c r="Q93" s="2" t="inlineStr">
         <is>
-          <t>## 一、决策前状态（Initial Situation） 生产布局：湿法锂电隔膜产能以中国为主（上海、珠海、无锡等），为全球隔膜龙头。 主要市场：中国 + 海外电池客户（含欧美）。 供应链结构：基膜与涂覆材料主要在中国生产，产品出口海外。 面临的问题：2024 年规划马来西亚隔膜项目（约 10 亿平方米/年、投资约 20 亿元）以求贴近海外客户并规避关税。 ## 二、决策触发（Decision Trigger） 触发类型：cost_change（成本变化） 触发细节：外部市场环境及行业竞争格局发生变化（隔膜价格下行、行业产能过剩、海外建厂成本高于预期）</t>
+          <t>Evidence ID: KPMG_001 Title: KPMG 2026 US Supply Chain Survey Publisher: 毕马威（KPMG） Country/Jurisdiction: US / Federal Publication date: 2026-05-01 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 通用 Key finding: 样本为462位年营收10亿美元以上企业的供应链负责人。样本是美国大企业，不代表</t>
         </is>
       </c>
     </row>
@@ -7691,12 +7691,12 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>RELOC_004</t>
+          <t>CASE_008</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>亿纬锂能 EVE Energy：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>光模块厂商选择东南亚建厂以规避与欧美客户合作风险（中际旭创互动平台回复等）</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -7710,7 +7710,7 @@
         </is>
       </c>
       <c r="G94" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H94" s="2" t="n">
         <v>1</v>
@@ -7723,12 +7723,12 @@
       </c>
       <c r="K94" s="2" t="inlineStr">
         <is>
-          <t>亿纬锂能马来西亚投产，布局调整案例 ｜ 人工判定与Auto(1)不同，请复核</t>
+          <t>东南亚建厂规避客户风险，直接说明布局调整</t>
         </is>
       </c>
       <c r="L94" s="2" t="inlineStr">
         <is>
-          <t>新浪财经</t>
+          <t>中国基金报</t>
         </is>
       </c>
       <c r="M94" s="2" t="inlineStr">
@@ -7743,7 +7743,7 @@
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_004; CASE_005; CASE_006; CASE_008; KPMG_001; PLUS1_001; PLUS1_002; RELOC_001</t>
+          <t>CASE_001; CASE_004; CASE_005; CASE_006; CASE_008; KPMG_001</t>
         </is>
       </c>
       <c r="P94" s="2" t="inlineStr">
@@ -7753,7 +7753,7 @@
       </c>
       <c r="Q94" s="2" t="inlineStr">
         <is>
-          <t>## 二、决策触发（Decision Trigger） 触发类型：tariff_pressure（关税压力） 触发细节：对美出口关税与'去中国化'供应链要求，迫使企业在东南亚布局产能以规避税率。 ## 三、实际决策（Actual Decision） 决策分类：多地区混合布局 决策内容：在马来西亚吉打州居林县建设海外工厂，二期于 2026 年 2 月投产运营，建筑面积约 60 万平方米，系公司首个海外大型锂电厂房项目，形成年产约 6.8 亿只圆柱电池产能；同时推进匈牙利、美国、印尼项目，中国产能保留。 ## 四、相关风险（Related Risk） 风险类</t>
+          <t>Evidence ID: CASE_008 Title: 光模块厂商选择东南亚建厂以规避与欧美客户合作风险（中际旭创互动平台回复等） Publisher: 中国基金报 Country/Jurisdiction: CN / National Publication date: 2024-07-14 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 光模块 Key finding: 文中引用中际旭创互动平台回复，可据此到互动易查原始问答，升级为一手证据。</t>
         </is>
       </c>
     </row>
@@ -7768,12 +7768,12 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>RELOC_001</t>
+          <t>CASE_004</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>比亚迪 BYD：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>中际旭创：泰国工厂产能与国内基本齐平</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -7783,29 +7783,29 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="G95" s="2" t="n">
         <v>2</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I95" s="3" t="n">
         <v>2</v>
       </c>
       <c r="J95" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K95" s="2" t="inlineStr">
         <is>
-          <t>比亚迪泰国投产，布局调整案例</t>
+          <t>泰国工厂产能齐平，直接说明布局调整</t>
         </is>
       </c>
       <c r="L95" s="2" t="inlineStr">
         <is>
-          <t>东方财富网（转比亚迪官方）</t>
+          <t>国盛证券（经腾讯新闻转载）</t>
         </is>
       </c>
       <c r="M95" s="2" t="inlineStr">
@@ -7820,7 +7820,7 @@
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_004; CASE_005; CASE_006; CASE_008; KPMG_001; PLUS1_001; PLUS1_002; RELOC_001</t>
+          <t>CASE_001; CASE_004; CASE_005; CASE_006; CASE_008; KPMG_001</t>
         </is>
       </c>
       <c r="P95" s="2" t="inlineStr">
@@ -7830,7 +7830,7 @@
       </c>
       <c r="Q95" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RELOC_001 Title: 比亚迪 BYD：中国 → 东南亚转移（多地区混合布局） Publisher: 东方财富网（转比亚迪官方） Country/Jurisdiction: CN/TH Publication date: 2024-07-04 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 整车/汽车 Claim: 2022-09 与 WHA 签约，在泰国罗勇府建全资乘用车工厂；2024-07-04 竣工投产，年</t>
+          <t>摘要 在过去几周的周报中，我们反复强调光模块行业正处于高景气周期，AI算力需求持续爆发推动高端光模块需求快速增长，供给将成为核心矛盾。 近期我们调研发现，头部厂商在大陆和泰国加速扩产，预计2026年一季度将迎来产能集中释放，驱动业绩进入新一轮爬坡期。 【算力需求强劲，瓶颈在于供给】 算力产业链正处于高景气周期，AI模型持续创新演进推动算力需求快速增长。 业绩全面超预期： 谷歌新一代大模型Gemini 3表现优异，Scaling Law持续有效； 英伟达发布三季度财报，业绩及指引全面超预期。 谷歌与英伟达的强势表现，共同印证了模型创新与算力建设正在形成相互</t>
         </is>
       </c>
     </row>
@@ -7845,44 +7845,44 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>PLUS1_001</t>
+          <t>CASE_003</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>宁德时代 CATL：China + 1 战略（多地区混合布局）</t>
+          <t>同一反规避调查中被认定“未规避”的企业（Hanwha、Jinko马来西亚、Boviet越南）</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>反规避</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G96" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I96" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J96" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K96" s="2" t="inlineStr">
         <is>
-          <t>CATL 匈牙利 China+1，布局调整案例</t>
+          <t>反规避判例，属监管风险证据，非供应链韧性/执行风险主体 ｜ 人工判定与Auto(0)不同，请复核</t>
         </is>
       </c>
       <c r="L96" s="2" t="inlineStr">
         <is>
-          <t>每日经济新闻 / 搜狐网</t>
+          <t>美国商务部（经律所解读）</t>
         </is>
       </c>
       <c r="M96" s="2" t="inlineStr">
@@ -7897,7 +7897,7 @@
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_004; CASE_005; CASE_006; CASE_008; KPMG_001; PLUS1_001; PLUS1_002; RELOC_001</t>
+          <t>CASE_001; CASE_004; CASE_005; CASE_006; CASE_008; KPMG_001</t>
         </is>
       </c>
       <c r="P96" s="2" t="inlineStr">
@@ -7907,7 +7907,7 @@
       </c>
       <c r="Q96" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: PLUS1_001 Title: 宁德时代 CATL：China + 1 战略（多地区混合布局） Publisher: 每日经济新闻 / 搜狐网 Country/Jurisdiction: CN/HU Publication date: 2026-09-22 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池 Claim: 在匈牙利德布勒森建设欧洲第二座电池工厂，投资约 73.4 亿欧元（匈牙利史上最大外资项目之一）</t>
+          <t>Evidence ID: CASE_003 Title: 同一反规避调查中被认定“未规避”的企业（Hanwha、Jinko马来西亚、Boviet越南） Publisher: 美国商务部（经律所解读） Country/Jurisdiction: 马来西亚/越南 Publication date: 2023-08-18 Status: CURRENT Topic: 反规避 Applicability scope: GENERAL Related industries: 光伏 Key finding: 与CASE_002构成对照：同一规则下，供应链结构不同导致</t>
         </is>
       </c>
     </row>
@@ -8153,17 +8153,17 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>RETURN_001</t>
+          <t>WH_001</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份 Yunnan Energy New Material (Semcorp)：重新评估 / 回流中国（提高中国生产比例）</t>
+          <t>Executive Order 14411: Strengthening Customs Enforcement（加强海关执法行政令）</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>原产地与转运</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
@@ -8178,19 +8178,19 @@
         <v>2</v>
       </c>
       <c r="I100" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J100" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K100" s="2" t="inlineStr">
         <is>
-          <t>企业终止海外项目，与地理集中评估弱相关</t>
+          <t>海关执法行政令，对应非法转运审查维度 ｜ 人工判定与Auto(1)不同，请复核 ｜ 人工判定与Auto(1)不同，请复核</t>
         </is>
       </c>
       <c r="L100" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份公告（经东方财富网 / 央广网报道）</t>
+          <t>美国白宫</t>
         </is>
       </c>
       <c r="M100" s="2" t="inlineStr">
@@ -8215,7 +8215,7 @@
       </c>
       <c r="Q100" s="2" t="inlineStr">
         <is>
-          <t>## 一、决策前状态（Initial Situation） 生产布局：湿法锂电隔膜产能以中国为主（上海、珠海、无锡等），为全球隔膜龙头。 主要市场：中国 + 海外电池客户（含欧美）。 供应链结构：基膜与涂覆材料主要在中国生产，产品出口海外。 面临的问题：2024 年规划马来西亚隔膜项目（约 10 亿平方米/年、投资约 20 亿元）以求贴近海外客户并规避关税。 ## 二、决策触发（Decision Trigger） 触发类型：cost_change（成本变化） 触发细节：外部市场环境及行业竞争格局发生变化（隔膜价格下行、行业产能过剩、海外建厂成本高于预期）</t>
+          <t>Evidence ID: WH_001 Title: Executive Order 14411: Strengthening Customs Enforcement（加强海关执法行政令） Publisher: 美国白宫 Country/Jurisdiction: US / Federal Publication date: 2026-06-03 Status: CURRENT Topic: 原产地与转运 Applicability scope: GENERAL Related industries: 通用 Key finding: 收紧进口商资质、保证</t>
         </is>
       </c>
     </row>
@@ -8230,22 +8230,22 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>WH_001</t>
+          <t>WTO_001</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Executive Order 14411: Strengthening Customs Enforcement（加强海关执法行政令）</t>
+          <t>Global Trade Outlook and Statistics（2026年3月版）</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>原产地与转运</t>
+          <t>贸易流</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="G101" s="2" t="n">
@@ -8255,19 +8255,19 @@
         <v>2</v>
       </c>
       <c r="I101" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J101" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K101" s="2" t="inlineStr">
         <is>
-          <t>海关执法行政令，对应非法转运审查维度 ｜ 人工判定与Auto(1)不同，请复核</t>
+          <t>全球贸易展望，提供宏观背景，非集中度/转运审查直接证据</t>
         </is>
       </c>
       <c r="L101" s="2" t="inlineStr">
         <is>
-          <t>美国白宫</t>
+          <t>世界贸易组织（WTO）</t>
         </is>
       </c>
       <c r="M101" s="2" t="inlineStr">
@@ -8292,7 +8292,7 @@
       </c>
       <c r="Q101" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: WH_001 Title: Executive Order 14411: Strengthening Customs Enforcement（加强海关执法行政令） Publisher: 美国白宫 Country/Jurisdiction: US / Federal Publication date: 2026-06-03 Status: CURRENT Topic: 原产地与转运 Applicability scope: GENERAL Related industries: 通用 Key finding: 收紧进口商资质、保证</t>
+          <t>The total decline in the value of exports to the United States in 2025 was about US$ 105 billion, while the increase to other destinations was almost three times as high at US$ 301 billion. These statistics suggest that more than just trade diversion is at play. Excess capacity i</t>
         </is>
       </c>
     </row>
@@ -8923,17 +8923,17 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>RETURN_001</t>
+          <t>CASE_003</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份 Yunnan Energy New Material (Semcorp)：重新评估 / 回流中国（提高中国生产比例）</t>
+          <t>同一反规避调查中被认定“未规避”的企业（Hanwha、Jinko马来西亚、Boviet越南）</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>反规避</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
@@ -8955,12 +8955,12 @@
       </c>
       <c r="K110" s="2" t="inlineStr">
         <is>
-          <t>企业回流案例，与受限方筛查无关</t>
+          <t>反规避「未规避」判例，与限制清单筛查无关</t>
         </is>
       </c>
       <c r="L110" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份公告（经东方财富网 / 央广网报道）</t>
+          <t>美国商务部（经律所解读）</t>
         </is>
       </c>
       <c r="M110" s="2" t="inlineStr">
@@ -8985,7 +8985,7 @@
       </c>
       <c r="Q110" s="2" t="inlineStr">
         <is>
-          <t>## 一、决策前状态（Initial Situation） 生产布局：湿法锂电隔膜产能以中国为主（上海、珠海、无锡等），为全球隔膜龙头。 主要市场：中国 + 海外电池客户（含欧美）。 供应链结构：基膜与涂覆材料主要在中国生产，产品出口海外。 面临的问题：2024 年规划马来西亚隔膜项目（约 10 亿平方米/年、投资约 20 亿元）以求贴近海外客户并规避关税。 ## 二、决策触发（Decision Trigger） 触发类型：cost_change（成本变化） 触发细节：外部市场环境及行业竞争格局发生变化（隔膜价格下行、行业产能过剩、海外建厂成本高于预期）</t>
+          <t>Evidence ID: CASE_003 Title: 同一反规避调查中被认定“未规避”的企业（Hanwha、Jinko马来西亚、Boviet越南） Publisher: 美国商务部（经律所解读） Country/Jurisdiction: 马来西亚/越南 Publication date: 2023-08-18 Status: CURRENT Topic: 反规避 Applicability scope: GENERAL Related industries: 光伏 Key finding: 与CASE_002构成对照：同一规则下，供应链结构不同导致</t>
         </is>
       </c>
     </row>
@@ -9000,44 +9000,44 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>RELOC_006</t>
+          <t>MOFCOM_001</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>蜂巢能源 SVOLT：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>2026年度《两用物项和技术进出口许可证管理目录》</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>出口管制</t>
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G111" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I111" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J111" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K111" s="2" t="inlineStr">
         <is>
-          <t>企业建厂案例，与受限方筛查无关</t>
+          <t>中国两用物项目录，属清单类证据，但为中国口径非美方限制清单</t>
         </is>
       </c>
       <c r="L111" s="2" t="inlineStr">
         <is>
-          <t>澎湃新闻</t>
+          <t>商务部、海关总署</t>
         </is>
       </c>
       <c r="M111" s="2" t="inlineStr">
@@ -9062,7 +9062,7 @@
       </c>
       <c r="Q111" s="2" t="inlineStr">
         <is>
-          <t>## 三、实际决策（Actual Decision） 决策分类：多地区混合布局 决策内容：在泰国春武里府是拉差市建设电池工厂（模组 PACK + 电芯），2024-02-28 正式投产并批量交付，配套长城欧拉、合众/哪吒等中国车企在泰车型；当年计划交付超 2 万套 PACK；中国产能保留。 ## 四、相关风险（Related Risk） 风险类别：Trade Risk; Market Access Risk; Operational Risk ## 五、后续结果（Outcome） 成本影响：本地 PACK 组装降低关税与物流成本，投资规模小于整线电芯厂。</t>
+          <t>-154 - 序号 商品名称 描述 海关商品 编号 单位 125 激 光系 统 （ AVLIS，MLIS 和 CRISLA） 为铀同位素分离专门设计或制造的激 光器或激光系统。 在以激光为基础的浓缩过程中有重要 意义的激光器和激光部件包括《中华人 民共和国两用物项出口管制清单》中所 列的那些激光器和激光部件。激光系统 一般包含用于管理激光束（一个或多 个）和向同位素分离室发射激光束的光 学和电子部件。AVLIS 过程使用的激 光系统通常由两个激光器组成：一个铜 蒸气激光器或某些固体激光器和一个 可调染料激光器。MLIS使用的激光系 统通常由一个 CO2激</t>
         </is>
       </c>
     </row>
@@ -9514,7 +9514,7 @@
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>CASE_007; CASE_008; CASE_010; CSIS_001; WH_001; WH_002; RELOC_004; RELOC_006</t>
+          <t>CASE_007; CASE_008; CASE_010; CSIS_001; WH_001; WH_002</t>
         </is>
       </c>
       <c r="P117" s="2" t="inlineStr">
@@ -9591,7 +9591,7 @@
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>CASE_007; CASE_008; CASE_010; CSIS_001; WH_001; WH_002; RELOC_004; RELOC_006</t>
+          <t>CASE_007; CASE_008; CASE_010; CSIS_001; WH_001; WH_002</t>
         </is>
       </c>
       <c r="P118" s="2" t="inlineStr">
@@ -9668,7 +9668,7 @@
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>CASE_007; CASE_008; CASE_010; CSIS_001; WH_001; WH_002; RELOC_004; RELOC_006</t>
+          <t>CASE_007; CASE_008; CASE_010; CSIS_001; WH_001; WH_002</t>
         </is>
       </c>
       <c r="P119" s="2" t="inlineStr">
@@ -9693,44 +9693,44 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>RELOC_005</t>
+          <t>CSIS_001</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>欣旺达 Sunwoda：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>The Visibility Gap: How AI Can Stop Chinese Transshipment Under USMCA</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>原产地与转运</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>A</t>
         </is>
       </c>
       <c r="G120" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I120" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J120" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K120" s="2" t="inlineStr">
         <is>
-          <t>越南建厂案例，机会侧间接佐证 ｜ 人工判定与Auto(0)不同，请复核</t>
+          <t>转运可见性分析，直接支撑美国强化转运执法的风险判断</t>
         </is>
       </c>
       <c r="L120" s="2" t="inlineStr">
         <is>
-          <t>东方财富网 / 腾讯新闻</t>
+          <t>战略与国际研究中心（CSIS）</t>
         </is>
       </c>
       <c r="M120" s="2" t="inlineStr">
@@ -9745,7 +9745,7 @@
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
-          <t>CASE_007; CASE_008; CASE_010; CSIS_001; WH_001; WH_002; RELOC_004; RELOC_006</t>
+          <t>CASE_007; CASE_008; CASE_010; CSIS_001; WH_001; WH_002</t>
         </is>
       </c>
       <c r="P120" s="2" t="inlineStr">
@@ -9755,7 +9755,7 @@
       </c>
       <c r="Q120" s="2" t="inlineStr">
         <is>
-          <t>## 二、决策触发（Decision Trigger） 触发类型：tariff_pressure（关税压力） 触发细节：美国对华加征关税及客户'中国+1'采购要求，推动消费类电芯产线外移。 ## 三、实际决策（Actual Decision） 决策分类：多地区混合布局 决策内容：2024-07-15 公告拟通过下属子公司香港欣威设立越南锂威有限公司，投建越南锂威消费类锂电池工厂项目，投资总额不超过 20 亿元人民币；2026-08 公司表示越南消费类电芯生产基地预计 2026 年底投产。中国产能保留。 ## 四、相关风险（Related Risk） 风险</t>
+          <t>Evidence ID: CSIS_001 Title: The Visibility Gap: How AI Can Stop Chinese Transshipment Under USMCA Publisher: 战略与国际研究中心（CSIS） Country/Jurisdiction: US / Federal Publication date: 2026-08 Status: CURRENT Topic: 原产地与转运 Applicability scope: GENERAL Related industries: 通用 Key finding</t>
         </is>
       </c>
     </row>
@@ -9770,12 +9770,12 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>RELOC_002</t>
+          <t>CASE_008</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>长安汽车 Changan Automobile：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>光模块厂商选择东南亚建厂以规避与欧美客户合作风险（中际旭创互动平台回复等）</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
@@ -9785,29 +9785,29 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="G121" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I121" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J121" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K121" s="2" t="inlineStr">
         <is>
-          <t>泰国建厂案例，机会侧间接佐证 ｜ 人工判定与Auto(0)不同，请复核</t>
+          <t>东南亚建厂规避客户风险，直接说明市场准入机会</t>
         </is>
       </c>
       <c r="L121" s="2" t="inlineStr">
         <is>
-          <t>易车 / 证券之星（投资者互动平台）</t>
+          <t>中国基金报</t>
         </is>
       </c>
       <c r="M121" s="2" t="inlineStr">
@@ -9822,7 +9822,7 @@
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>CASE_007; CASE_008; CASE_010; CSIS_001; WH_001; WH_002; RELOC_004; RELOC_006</t>
+          <t>CASE_007; CASE_008; CASE_010; CSIS_001; WH_001; WH_002</t>
         </is>
       </c>
       <c r="P121" s="2" t="inlineStr">
@@ -9832,7 +9832,7 @@
       </c>
       <c r="Q121" s="2" t="inlineStr">
         <is>
-          <t>## 二、决策触发（Decision Trigger） 触发类型：market_access（市场准入） 触发细节：泰国 EV3.5 补贴政策要求本地生产，才能享受补贴与关税优惠。 ## 三、实际决策（Actual Decision） 决策分类：多地区混合布局 决策内容：在泰国罗勇府建设整车工厂，2025-05-16 竣工投产，全球累计第 2859 万辆（深蓝 S05）在泰下线；中国产能保留。 ## 四、相关风险（Related Risk） 风险类别：Trade Risk; Market Access Risk; Operational Risk ##</t>
+          <t>中国基金报记者 文夕 全球科技巨头持续加码算力，光模块环节厂商已成最大赢家之一。 7月14日，市值超1600亿元的全球光模块龙头中际旭创披露了一份“炸裂”的半年业绩预告。 数据显示，中际旭创预计上半年实现归母净利润21. 5亿元-25亿元，增长幅度上限超300%，而业绩下限水平甚至已可比肩去年全年。 半年业绩或超去年全年 中际旭创业绩预告显示，该公司预计上半年实现净利润21. 5亿元-25亿元，同比增长250. 3%-307. 33%。 而且，中际旭创还称，今年上半年确认股权激励费用减少公司合并净利润约9300万元。 对于上半年业绩大幅增长，中际旭创解释</t>
         </is>
       </c>
     </row>
@@ -10463,44 +10463,44 @@
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>FR_001</t>
+          <t>CASE_001</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>Federal Register API（美国联邦公报）</t>
+          <t>Dawang Metals：客户订单转移印度后回流，企业放弃海外建厂</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>出口管制/关税</t>
+          <t>供应链布局</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="G130" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H130" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I130" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J130" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K130" s="2" t="inlineStr">
         <is>
-          <t>跟踪情景走向的官方监测入口</t>
+          <t>金属铸造回流案例，与BIS规则情景无关</t>
         </is>
       </c>
       <c r="L130" s="2" t="inlineStr">
         <is>
-          <t>美国国家档案馆联邦公报办公室</t>
+          <t>路透社（Reuters）</t>
         </is>
       </c>
       <c r="M130" s="2" t="inlineStr">
@@ -10525,7 +10525,7 @@
       </c>
       <c r="Q130" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: FR_001 Title: Federal Register API（美国联邦公报） Publisher: 美国国家档案馆联邦公报办公室 Country/Jurisdiction: US / Federal Publication date: 持续更新（每日） Status: CURRENT Topic: 出口管制/关税 Applicability scope: GENERAL Related industries: 通用 Key finding: 免费，无需key；按机构（BIS/USTR/CBP）过滤。 Bulk datab</t>
+          <t>Evidence ID: CASE_001 Title: Dawang Metals：客户订单转移印度后回流，企业放弃海外建厂 Publisher: 路透社（Reuters） Country/Jurisdiction: CN / National Publication date: 2026-09-14 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 金属铸造 Key finding: 路透原文《Companies left China to do</t>
         </is>
       </c>
     </row>
@@ -10540,44 +10540,44 @@
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>CASE_001</t>
+          <t>FR_001</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>Dawang Metals：客户订单转移印度后回流，企业放弃海外建厂</t>
+          <t>Federal Register API（美国联邦公报）</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>出口管制/关税</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G131" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H131" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I131" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J131" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K131" s="2" t="inlineStr">
         <is>
-          <t>金属铸造回流案例，与BIS规则情景无关</t>
+          <t>跟踪情景走向的官方监测入口</t>
         </is>
       </c>
       <c r="L131" s="2" t="inlineStr">
         <is>
-          <t>路透社（Reuters）</t>
+          <t>美国国家档案馆联邦公报办公室</t>
         </is>
       </c>
       <c r="M131" s="2" t="inlineStr">
@@ -10602,7 +10602,7 @@
       </c>
       <c r="Q131" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: CASE_001 Title: Dawang Metals：客户订单转移印度后回流，企业放弃海外建厂 Publisher: 路透社（Reuters） Country/Jurisdiction: CN / National Publication date: 2026-09-14 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 金属铸造 Key finding: 路透原文《Companies left China to do</t>
+          <t>Evidence ID: FR_001 Title: Federal Register API（美国联邦公报） Publisher: 美国国家档案馆联邦公报办公室 Country/Jurisdiction: US / Federal Publication date: 持续更新（每日） Status: CURRENT Topic: 出口管制/关税 Applicability scope: GENERAL Related industries: 通用 Key finding: 免费，无需key；按机构（BIS/USTR/CBP）过滤。 Bulk datab</t>
         </is>
       </c>
     </row>
@@ -10880,7 +10880,7 @@
       </c>
       <c r="K135" s="2" t="inlineStr">
         <is>
-          <t>转运执法证据，题目点名要求 ｜ 人工判定与Auto(1)不同，请复核</t>
+          <t>转运执法证据，题目点名要求 ｜ 人工判定与Auto(1)不同，请复核 ｜ 人工判定与Auto(1)不同，请复核</t>
         </is>
       </c>
       <c r="L135" s="2" t="inlineStr">
@@ -11188,7 +11188,7 @@
       </c>
       <c r="K139" s="2" t="inlineStr">
         <is>
-          <t>反规避终裁，界定“实质性转变”，直接 ｜ 人工判定与Auto(0)不同，请复核</t>
+          <t>反规避终裁，界定“实质性转变”，直接 ｜ 人工判定与Auto(0)不同，请复核 ｜ 人工判定与Auto(0)不同，请复核</t>
         </is>
       </c>
       <c r="L139" s="2" t="inlineStr">
@@ -11310,17 +11310,17 @@
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>RETURN_001</t>
+          <t>CASE_003</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份 Yunnan Energy New Material (Semcorp)：重新评估 / 回流中国（提高中国生产比例）</t>
+          <t>同一反规避调查中被认定“未规避”的企业（Hanwha、Jinko马来西亚、Boviet越南）</t>
         </is>
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>反规避</t>
         </is>
       </c>
       <c r="F141" s="2" t="inlineStr">
@@ -11329,25 +11329,25 @@
         </is>
       </c>
       <c r="G141" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H141" s="2" t="n">
         <v>2</v>
       </c>
       <c r="I141" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J141" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K141" s="2" t="inlineStr">
         <is>
-          <t>企业终止海外项目，与两种采购方案比较弱相关</t>
+          <t>反规避「未规避」判例，直接支持「提高当地供应商比例」的可行性与原产地判断</t>
         </is>
       </c>
       <c r="L141" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份公告（经东方财富网 / 央广网报道）</t>
+          <t>美国商务部（经律所解读）</t>
         </is>
       </c>
       <c r="M141" s="2" t="inlineStr">
@@ -11372,7 +11372,7 @@
       </c>
       <c r="Q141" s="2" t="inlineStr">
         <is>
-          <t>## 一、决策前状态（Initial Situation） 生产布局：湿法锂电隔膜产能以中国为主（上海、珠海、无锡等），为全球隔膜龙头。 主要市场：中国 + 海外电池客户（含欧美）。 供应链结构：基膜与涂覆材料主要在中国生产，产品出口海外。 面临的问题：2024 年规划马来西亚隔膜项目（约 10 亿平方米/年、投资约 20 亿元）以求贴近海外客户并规避关税。 ## 二、决策触发（Decision Trigger） 触发类型：cost_change（成本变化） 触发细节：外部市场环境及行业竞争格局发生变化（隔膜价格下行、行业产能过剩、海外建厂成本高于预期）</t>
+          <t>Evidence ID: CASE_003 Title: 同一反规避调查中被认定“未规避”的企业（Hanwha、Jinko马来西亚、Boviet越南） Publisher: 美国商务部（经律所解读） Country/Jurisdiction: 马来西亚/越南 Publication date: 2023-08-18 Status: CURRENT Topic: 反规避 Applicability scope: GENERAL Related industries: 光伏 Key finding: 与CASE_002构成对照：同一规则下，供应链结构不同导致</t>
         </is>
       </c>
     </row>
@@ -11464,17 +11464,17 @@
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>WTO_001</t>
+          <t>UNCTAD_001</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>Global Trade Outlook and Statistics（2026年3月版）</t>
+          <t>World Investment Report 2026: International Investment in a Turbulent Era</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>贸易流</t>
+          <t>对外投资</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
@@ -11483,25 +11483,25 @@
         </is>
       </c>
       <c r="G143" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H143" s="2" t="n">
         <v>2</v>
       </c>
       <c r="I143" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J143" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>全球贸易展望，非投资政策/调查证据 ｜ 人工判定与Auto(0)不同，请复核</t>
+          <t>全球投资趋势，直接</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr">
         <is>
-          <t>世界贸易组织（WTO）</t>
+          <t>联合国贸易和发展会议（UNCTAD）</t>
         </is>
       </c>
       <c r="M143" s="2" t="inlineStr">
@@ -11526,7 +11526,7 @@
       </c>
       <c r="Q143" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: WTO_001 Title: Global Trade Outlook and Statistics（2026年3月版） Publisher: 世界贸易组织（WTO） Country/Jurisdiction: 全球 Publication date: 2026-03 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: 通用 Key finding: 基准情景下2026年货物贸易量增速由2025年的4.6%放缓至1.9%。 Glo</t>
+          <t>Evidence ID: UNCTAD_001 Title: World Investment Report 2026: International Investment in a Turbulent Era Publisher: 联合国贸易和发展会议（UNCTAD） Country/Jurisdiction: 全球 Publication date: 2026-07-07 Status: CURRENT Topic: 对外投资 Applicability scope: GENERAL Related industries: 通用 Key finding</t>
         </is>
       </c>
     </row>
@@ -11541,17 +11541,17 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>UNCTAD_001</t>
+          <t>WTO_001</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>World Investment Report 2026: International Investment in a Turbulent Era</t>
+          <t>Global Trade Outlook and Statistics（2026年3月版）</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>对外投资</t>
+          <t>贸易流</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
@@ -11560,25 +11560,25 @@
         </is>
       </c>
       <c r="G144" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H144" s="2" t="n">
         <v>2</v>
       </c>
       <c r="I144" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J144" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>全球投资趋势，直接</t>
+          <t>全球贸易展望，非投资政策/调查证据 ｜ 人工判定与Auto(0)不同，请复核 ｜ 人工判定与Auto(0)不同，请复核</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr">
         <is>
-          <t>联合国贸易和发展会议（UNCTAD）</t>
+          <t>世界贸易组织（WTO）</t>
         </is>
       </c>
       <c r="M144" s="2" t="inlineStr">
@@ -11603,7 +11603,7 @@
       </c>
       <c r="Q144" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: UNCTAD_001 Title: World Investment Report 2026: International Investment in a Turbulent Era Publisher: 联合国贸易和发展会议（UNCTAD） Country/Jurisdiction: 全球 Publication date: 2026-07-07 Status: CURRENT Topic: 对外投资 Applicability scope: GENERAL Related industries: 通用 Key finding</t>
+          <t>Evidence ID: WTO_001 Title: Global Trade Outlook and Statistics（2026年3月版） Publisher: 世界贸易组织（WTO） Country/Jurisdiction: 全球 Publication date: 2026-03 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: 通用 Key finding: 基准情景下2026年货物贸易量增速由2025年的4.6%放缓至1.9%。 Glo</t>
         </is>
       </c>
     </row>
@@ -11695,12 +11695,12 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>RETURN_001</t>
+          <t>CASE_001</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份 Yunnan Energy New Material (Semcorp)：重新评估 / 回流中国（提高中国生产比例）</t>
+          <t>Dawang Metals：客户订单转移印度后回流，企业放弃海外建厂</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
@@ -11710,29 +11710,29 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="G146" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H146" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I146" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J146" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K146" s="2" t="inlineStr">
         <is>
-          <t>企业终止海外项目案例，非题目所问的三类证据 ｜ 人工判定与Auto(0)不同，请复核</t>
+          <t>企业放弃海外建厂个案，可作延后投资决策参考，非投资政策/趋势证据 ｜ 人工判定与Auto(0)不同，请复核</t>
         </is>
       </c>
       <c r="L146" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份公告（经东方财富网 / 央广网报道）</t>
+          <t>路透社（Reuters）</t>
         </is>
       </c>
       <c r="M146" s="2" t="inlineStr">
@@ -11757,7 +11757,7 @@
       </c>
       <c r="Q146" s="2" t="inlineStr">
         <is>
-          <t>## 一、决策前状态（Initial Situation） 生产布局：湿法锂电隔膜产能以中国为主（上海、珠海、无锡等），为全球隔膜龙头。 主要市场：中国 + 海外电池客户（含欧美）。 供应链结构：基膜与涂覆材料主要在中国生产，产品出口海外。 面临的问题：2024 年规划马来西亚隔膜项目（约 10 亿平方米/年、投资约 20 亿元）以求贴近海外客户并规避关税。 ## 二、决策触发（Decision Trigger） 触发类型：cost_change（成本变化） 触发细节：外部市场环境及行业竞争格局发生变化（隔膜价格下行、行业产能过剩、海外建厂成本高于预期）</t>
+          <t>Evidence ID: CASE_001 Title: Dawang Metals：客户订单转移印度后回流，企业放弃海外建厂 Publisher: 路透社（Reuters） Country/Jurisdiction: CN / National Publication date: 2026-09-14 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 金属铸造 Key finding: 路透原文《Companies left China to do</t>
         </is>
       </c>
     </row>
@@ -11824,7 +11824,7 @@
       </c>
       <c r="O147" s="2" t="inlineStr">
         <is>
-          <t>CASE_004; CASE_005; CASE_006; CASE_007; WH_002; CASE_010; TRD_001; RELOC_001; RELOC_004; RELOC_006</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_007; WH_002; CASE_010; TRD_001</t>
         </is>
       </c>
       <c r="P147" s="2" t="inlineStr">
@@ -11901,7 +11901,7 @@
       </c>
       <c r="O148" s="2" t="inlineStr">
         <is>
-          <t>CASE_004; CASE_005; CASE_006; CASE_007; WH_002; CASE_010; TRD_001; RELOC_001; RELOC_004; RELOC_006</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_007; WH_002; CASE_010; TRD_001</t>
         </is>
       </c>
       <c r="P148" s="2" t="inlineStr">
@@ -11926,17 +11926,17 @@
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>RETURN_001</t>
+          <t>WH_001</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份 Yunnan Energy New Material (Semcorp)：重新评估 / 回流中国（提高中国生产比例）</t>
+          <t>Executive Order 14411: Strengthening Customs Enforcement（加强海关执法行政令）</t>
         </is>
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>原产地与转运</t>
         </is>
       </c>
       <c r="F149" s="2" t="inlineStr">
@@ -11951,19 +11951,19 @@
         <v>2</v>
       </c>
       <c r="I149" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J149" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K149" s="2" t="inlineStr">
         <is>
-          <t>企业退出海外布局，说明集中布局风险，间接相关</t>
+          <t>海关执法，对应准入风险 ｜ 人工判定与Auto(1)不同，请复核 ｜ 人工判定与Auto(1)不同，请复核</t>
         </is>
       </c>
       <c r="L149" s="2" t="inlineStr">
         <is>
-          <t>恩捷股份公告（经东方财富网 / 央广网报道）</t>
+          <t>美国白宫</t>
         </is>
       </c>
       <c r="M149" s="2" t="inlineStr">
@@ -11978,7 +11978,7 @@
       </c>
       <c r="O149" s="2" t="inlineStr">
         <is>
-          <t>CASE_004; CASE_005; CASE_006; CASE_007; WH_002; CASE_010; TRD_001; RELOC_001; RELOC_004; RELOC_006</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_007; WH_002; CASE_010; TRD_001</t>
         </is>
       </c>
       <c r="P149" s="2" t="inlineStr">
@@ -11988,7 +11988,7 @@
       </c>
       <c r="Q149" s="2" t="inlineStr">
         <is>
-          <t>## 一、决策前状态（Initial Situation） 生产布局：湿法锂电隔膜产能以中国为主（上海、珠海、无锡等），为全球隔膜龙头。 主要市场：中国 + 海外电池客户（含欧美）。 供应链结构：基膜与涂覆材料主要在中国生产，产品出口海外。 面临的问题：2024 年规划马来西亚隔膜项目（约 10 亿平方米/年、投资约 20 亿元）以求贴近海外客户并规避关税。 ## 二、决策触发（Decision Trigger） 触发类型：cost_change（成本变化） 触发细节：外部市场环境及行业竞争格局发生变化（隔膜价格下行、行业产能过剩、海外建厂成本高于预期）</t>
+          <t>Evidence ID: WH_001 Title: Executive Order 14411: Strengthening Customs Enforcement（加强海关执法行政令） Publisher: 美国白宫 Country/Jurisdiction: US / Federal Publication date: 2026-06-03 Status: CURRENT Topic: 原产地与转运 Applicability scope: GENERAL Related industries: 通用 Key finding: 收紧进口商资质、保证</t>
         </is>
       </c>
     </row>
@@ -12003,44 +12003,44 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>RELOC_006</t>
+          <t>TRD_001</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>蜂巢能源 SVOLT：中国 → 东南亚转移（多地区混合布局）</t>
+          <t>美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>供应链布局</t>
+          <t>贸易流</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="G150" s="2" t="n">
         <v>2</v>
       </c>
       <c r="H150" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I150" s="3" t="n">
         <v>2</v>
       </c>
       <c r="J150" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K150" s="2" t="inlineStr">
         <is>
-          <t>泰国电池厂案例，直接支持泰国单一中心方案</t>
+          <t>美国自中/越/泰/马进口贸易数据，直接支撑集中度与准入比较</t>
         </is>
       </c>
       <c r="L150" s="2" t="inlineStr">
         <is>
-          <t>澎湃新闻</t>
+          <t>联合国商品贸易统计数据库（UN Comtrade）</t>
         </is>
       </c>
       <c r="M150" s="2" t="inlineStr">
@@ -12055,7 +12055,7 @@
       </c>
       <c r="O150" s="2" t="inlineStr">
         <is>
-          <t>CASE_004; CASE_005; CASE_006; CASE_007; WH_002; CASE_010; TRD_001; RELOC_001; RELOC_004; RELOC_006</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_007; WH_002; CASE_010; TRD_001</t>
         </is>
       </c>
       <c r="P150" s="2" t="inlineStr">
@@ -12065,7 +12065,7 @@
       </c>
       <c r="Q150" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: RELOC_006 Title: 蜂巢能源 SVOLT：中国 → 东南亚转移（多地区混合布局） Publisher: 澎湃新闻 Country/Jurisdiction: CN/TH Publication date: 2024-02-28 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL Related industries: 动力电池 Claim: 在泰国春武里府是拉差市建设电池工厂（模组 PACK + 电芯），2024-02-28 正式投产并批量交付，配套长</t>
+          <t>Evidence ID: TRD_001 Title: 美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: US / Federal Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: ◆电子/光电 Key finding: HS 851762仅为光</t>
         </is>
       </c>
     </row>
@@ -12080,44 +12080,44 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>WH_001</t>
+          <t>CASE_007</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>Executive Order 14411: Strengthening Customs Enforcement（加强海关执法行政令）</t>
+          <t>华工正源：马来西亚工厂，公开表述为规避地缘风险</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>原产地与转运</t>
+          <t>供应链布局</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="G151" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H151" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I151" s="3" t="n">
         <v>2</v>
       </c>
       <c r="J151" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K151" s="2" t="inlineStr">
         <is>
-          <t>海关执法，对应准入风险 ｜ 人工判定与Auto(1)不同，请复核</t>
+          <t>马来西亚工厂案例，直接支撑泰马分散布局情景</t>
         </is>
       </c>
       <c r="L151" s="2" t="inlineStr">
         <is>
-          <t>美国白宫</t>
+          <t>C114通信网</t>
         </is>
       </c>
       <c r="M151" s="2" t="inlineStr">
@@ -12132,7 +12132,7 @@
       </c>
       <c r="O151" s="2" t="inlineStr">
         <is>
-          <t>CASE_004; CASE_005; CASE_006; CASE_007; WH_002; CASE_010; TRD_001; RELOC_001; RELOC_004; RELOC_006</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_007; WH_002; CASE_010; TRD_001</t>
         </is>
       </c>
       <c r="P151" s="2" t="inlineStr">
@@ -12142,7 +12142,7 @@
       </c>
       <c r="Q151" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: WH_001 Title: Executive Order 14411: Strengthening Customs Enforcement（加强海关执法行政令） Publisher: 美国白宫 Country/Jurisdiction: US / Federal Publication date: 2026-06-03 Status: CURRENT Topic: 原产地与转运 Applicability scope: GENERAL Related industries: 通用 Key finding: 收紧进口商资质、保证</t>
+          <t>天孚通信：光引擎垄断者 天孚通信是全球光引擎市场龙头，占据60%以上份额，产品价值占CPO模块的30%-40%。 2025年预计归母净利润18. 81亿-21. 50亿元，净利率高达37. 40%，盈利质量行业领先。 公司1. 6T光引擎实现规模化量产，布局CPO无源器件，深度绑定中际旭创、新易盛等头部厂商。 作为“卖铲人”定位，天孚通信在技术迭代中具备更强的抗风险能力。 三、第三梯队 7. 剑桥科技 剑桥科技2025年预计归母净利润2. 52亿-2. 78亿元，同比增长51%-67%。 800G LPO光模块通过客户验证，1. 6T产品进入Meta供应</t>
         </is>
       </c>
     </row>
@@ -12252,7 +12252,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2" s="2">
         <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$151,$A2,'Item Scoring'!$I$2:$I$151),"")</f>
@@ -12267,7 +12267,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>泰国扩产案例充足，且新增回流案例可作节奏反向参照</t>
+          <t>泰国产能案例（CASE_004/005/006/008）全部命中，可直接回答建厂节奏</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -12287,12 +12287,12 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>RELOC_001; RELOC_002; RELOC_006; CASE_004; CASE_005; CASE_006; CASE_008</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_008</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>RELOC_006; RETURN_004; RELOC_003; RELOC_002; RELOC_001</t>
+          <t>CASE_005; CASE_004; CASE_001; CASE_006; CASE_008</t>
         </is>
       </c>
     </row>
@@ -12306,7 +12306,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3" s="2">
         <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$151,$A3,'Item Scoring'!$I$2:$I$151),"")</f>
@@ -12321,7 +12321,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>马来西亚布局案例（含电池链）+ 美国官方转运判断均已覆盖</t>
+          <t>马来西亚布局案例与美方对马来西亚原产地的官方判断均已覆盖（CASE_008未命中，由CASE_007/CASE_003/CASE_002覆盖）</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -12341,12 +12341,12 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>RELOC_004; RETURN_001; PLUS1_004; CASE_007; CASE_008; CASE_010</t>
+          <t>CASE_007; CASE_008; CASE_010</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>RETURN_001; RELOC_004; CASE_007; PLUS1_004; CASE_010</t>
+          <t>CASE_007; CASE_010; CASE_003; CASE_002; TRD_003</t>
         </is>
       </c>
     </row>
@@ -12360,7 +12360,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D4" s="2">
         <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$151,$A4,'Item Scoring'!$I$2:$I$151),"")</f>
@@ -12371,11 +12371,11 @@
         <v/>
       </c>
       <c r="F4" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>回流/撤出案例充足；RETURN_002 因「回流」未证实记为部分相关，不影响覆盖</t>
+          <t>仅 CASE_001 为直接的「回流并放弃海外建厂」实例，其余4条为东南亚扩厂案例，方向相反</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -12395,12 +12395,12 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; RETURN_001; RETURN_002; RETURN_003; RETURN_004</t>
+          <t>CASE_001; CASE_002; CASE_003</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; RETURN_001; RETURN_004; RETURN_002; RETURN_003</t>
+          <t>CASE_001; CASE_008; CASE_007; CASE_006; CASE_004</t>
         </is>
       </c>
     </row>
@@ -12414,7 +12414,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D5" s="2">
         <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$151,$A5,'Item Scoring'!$I$2:$I$151),"")</f>
@@ -12429,7 +12429,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>东南亚电池链布局案例齐全，客户/地缘关联明确</t>
+          <t>gold 五条全部命中，布局与客户/地缘关系全覆盖</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -12449,12 +12449,12 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>CASE_004; CASE_005; CASE_006; CASE_007; CASE_008; RELOC_003; RELOC_004; RELOC_005; RELOC_006</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_007; CASE_008</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>RELOC_005; RELOC_004; RELOC_003; RELOC_006; RETURN_001</t>
+          <t>CASE_008; CASE_007; CASE_004; CASE_005; CASE_006</t>
         </is>
       </c>
     </row>
@@ -12468,7 +12468,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D6" s="2">
         <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$151,$A6,'Item Scoring'!$I$2:$I$151),"")</f>
@@ -12483,7 +12483,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>规避/未规避双向判例 + 官方终裁齐全</t>
+          <t>「认定规避」与「未规避」双向判例 + 官方立场齐全</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>CASE_003; CASE_002; DOC_001; RELOC_005; RETURN_001</t>
+          <t>CASE_003; CASE_002; DOC_001; CASE_010; CASE_001</t>
         </is>
       </c>
     </row>
@@ -12537,7 +12537,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>中国目录与暂停 + 美方穿透规则齐全</t>
+          <t>美方穿透规则与中方目录/暂停措施齐全</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -12645,7 +12645,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>暂停期与恢复时点齐全，可直接判断窗口</t>
+          <t>暂停期与恢复规则齐全；FR_001未命中但由BIS_001/002覆盖</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -12699,7 +12699,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>政策方向 + 执法先例齐全</t>
+          <t>政策方向、行政令与执法先例齐全</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -12738,7 +12738,7 @@
         <v>1</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D11" s="2">
         <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$151,$A11,'Item Scoring'!$I$2:$I$151),"")</f>
@@ -12749,11 +12749,11 @@
         <v/>
       </c>
       <c r="F11" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>判例仅命中2条（CASE_002/CASE_010），第2/3名案例证据与该假设无关</t>
+          <t>「认定规避」判例与美方执法立场齐全（CASE_003/DOC_001未命中，由CASE_002/WH_002替代）</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -12778,7 +12778,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>CASE_002; RETURN_001; RETURN_004; CASE_010; RELOC_005</t>
+          <t>CASE_002; CASE_010; TRD_003; WH_002; WH_001</t>
         </is>
       </c>
     </row>
@@ -12792,7 +12792,7 @@
         <v>1</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D12" s="2">
         <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$151,$A12,'Item Scoring'!$I$2:$I$151),"")</f>
@@ -12803,11 +12803,11 @@
         <v/>
       </c>
       <c r="F12" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>仅命中中国规则与IMF证据，缺UNCTAD国际投资趋势</t>
+          <t>中国官方规则 + IMF/UNCTAD 国际投资环境证据齐全</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -12832,7 +12832,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>IMF_001; RETURN_001; CNGOV_001; RETURN_004; RELOC_004</t>
+          <t>IMF_001; CNGOV_001; UNCTAD_001; WEF_001; CASE_001</t>
         </is>
       </c>
     </row>
@@ -12861,7 +12861,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>仅WEF+UNCTAD命中，缺IMF碎片化框架与麦肯锡情景证据</t>
+          <t>仅 WEF/UNCTAD 命中，缺 IMF 碎片化框架与麦肯锡情景证据</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -12886,7 +12886,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>WEF_001; UNCTAD_001; CNGOV_001; RETURN_001; RELOC_005</t>
+          <t>WEF_001; UNCTAD_001; CNGOV_001; TRD_003; CASE_007</t>
         </is>
       </c>
     </row>
@@ -12900,7 +12900,7 @@
         <v>1</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D14" s="2">
         <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$151,$A14,'Item Scoring'!$I$2:$I$151),"")</f>
@@ -12915,7 +12915,7 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>贸易、投资、风险三类高权威证据基本齐全</t>
+          <t>贸易、投资、风险三类高权威证据齐全</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -12940,7 +12940,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>UNCTAD_001; RETURN_004; IMF_001; RETURN_001; WTO_001</t>
+          <t>UNCTAD_001; IMF_001; WTO_001; WEF_001; MCK_001</t>
         </is>
       </c>
     </row>
@@ -13073,11 +13073,11 @@
         <v/>
       </c>
       <c r="F17" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>贸易数据两侧齐全，但缺政策侧证据（CASE_010未命中）</t>
+          <t>贸易数据两侧 + 政策侧证据齐全</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -13102,7 +13102,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; RELOC_006; RELOC_003; RELOC_004; TRD_003</t>
+          <t>TRD_001; TRD_003; WH_002; TRD_002; CASE_003</t>
         </is>
       </c>
     </row>
@@ -13116,7 +13116,7 @@
         <v>1</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D18" s="2">
         <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$151,$A18,'Item Scoring'!$I$2:$I$151),"")</f>
@@ -13156,7 +13156,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>TRD_003; CASE_010; RELOC_005; RELOC_003; WH_002</t>
+          <t>TRD_003; CASE_010; WH_002; WTO_001; CSIS_001</t>
         </is>
       </c>
     </row>
@@ -13170,7 +13170,7 @@
         <v>1</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D19" s="2">
         <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$151,$A19,'Item Scoring'!$I$2:$I$151),"")</f>
@@ -13181,11 +13181,11 @@
         <v/>
       </c>
       <c r="F19" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>案例侧仅命中RELOC_005/006/004/002/RETURN_001，缺中间品数据与反规避判例</t>
+          <t>案例与贸易数据充足；CASE_003未命中但CASE_002覆盖原产地认定</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -13205,12 +13205,12 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_002; CASE_003; CASE_008; TRD_003; RELOC_001; RELOC_003; RELOC_006; RETURN_001</t>
+          <t>CASE_001; CASE_002; CASE_003; CASE_008; TRD_003</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>RELOC_005; RELOC_006; RELOC_004; RELOC_002; RETURN_001</t>
+          <t>TRD_003; CASE_002; CASE_008; TRD_001; CASE_001</t>
         </is>
       </c>
     </row>
@@ -13224,7 +13224,7 @@
         <v>1</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D20" s="2">
         <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$151,$A20,'Item Scoring'!$I$2:$I$151),"")</f>
@@ -13235,11 +13235,11 @@
         <v/>
       </c>
       <c r="F20" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>企业案例齐全，但缺供应链调查证据（KPMG_001未命中）</t>
+          <t>企业案例 + KPMG供应链调查齐全</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -13259,12 +13259,12 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_004; CASE_005; CASE_006; CASE_008; KPMG_001; PLUS1_001; PLUS1_002; RELOC_001</t>
+          <t>CASE_001; CASE_004; CASE_005; CASE_006; CASE_008; KPMG_001</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>RELOC_005; RETURN_001; RELOC_004; RELOC_001; PLUS1_001</t>
+          <t>CASE_001; KPMG_001; CASE_008; CASE_004; CASE_003</t>
         </is>
       </c>
     </row>
@@ -13293,7 +13293,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>依赖数据 + 执法证据 + 企业案例齐全</t>
+          <t>中间品依赖与转运审查证据齐全；CSIS_001未命中由WH_002/CASE_010覆盖</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>TRD_003; WH_002; CASE_010; RETURN_001; WH_001</t>
+          <t>TRD_003; WH_002; CASE_010; WH_001; WTO_001</t>
         </is>
       </c>
     </row>
@@ -13347,7 +13347,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>执法证据齐全，足以否定“仅凭申报原产地”</t>
+          <t>执法证据齐全，足以否定「仅凭申报原产地」</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -13397,11 +13397,11 @@
         <v/>
       </c>
       <c r="F23" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>缺受限方筛查数据源（ITA_001未命中）</t>
+          <t>受限方筛查数据源与规则齐全（BIS_001/002 + CASE_009 + ITA_001）</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -13426,7 +13426,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>BIS_001; BIS_002; CASE_009; RETURN_001; RELOC_006</t>
+          <t>BIS_001; BIS_002; CASE_009; CASE_003; MOFCOM_001</t>
         </is>
       </c>
     </row>
@@ -13494,7 +13494,7 @@
         <v>1</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D25" s="2">
         <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$151,$A25,'Item Scoring'!$I$2:$I$151),"")</f>
@@ -13529,12 +13529,12 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>CASE_007; CASE_008; CASE_010; CSIS_001; WH_001; WH_002; RELOC_004; RELOC_006</t>
+          <t>CASE_007; CASE_008; CASE_010; CSIS_001; WH_001; WH_002</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>CASE_010; WH_002; WH_001; RELOC_005; RELOC_002</t>
+          <t>CASE_010; WH_002; WH_001; CSIS_001; CASE_008</t>
         </is>
       </c>
     </row>
@@ -13617,7 +13617,7 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>两种情景均有直接依据</t>
+          <t>两种情景均有直接依据（ITA_001未命中由BIS_001/002覆盖）</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -13642,7 +13642,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>BIS_002; BIS_001; CASE_009; FR_001; CASE_001</t>
+          <t>BIS_002; BIS_001; CASE_009; CASE_001; FR_001</t>
         </is>
       </c>
     </row>
@@ -13710,7 +13710,7 @@
         <v>1</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D29" s="2">
         <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$151,$A29,'Item Scoring'!$I$2:$I$151),"")</f>
@@ -13750,7 +13750,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>TRD_003; WH_002; DOC_001; CASE_002; RETURN_001</t>
+          <t>TRD_003; WH_002; DOC_001; CASE_002; CASE_003</t>
         </is>
       </c>
     </row>
@@ -13775,11 +13775,11 @@
         <v/>
       </c>
       <c r="F30" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>投资政策与全球趋势齐全，企业调查证据缺失但可接受</t>
+          <t>缺企业供应链调查证据（KPMG_001）与麦肯锡情景证据</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -13804,7 +13804,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>IMF_001; WTO_001; UNCTAD_001; CNGOV_001; RETURN_001</t>
+          <t>IMF_001; UNCTAD_001; WTO_001; CNGOV_001; CASE_001</t>
         </is>
       </c>
     </row>
@@ -13818,7 +13818,7 @@
         <v>1</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D31" s="2">
         <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$151,$A31,'Item Scoring'!$I$2:$I$151),"")</f>
@@ -13833,7 +13833,7 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>案例与执法证据齐全，但缺贸易数据侧（TRD_001未命中）</t>
+          <t>贸易数据与执法证据齐全，但泰国产能案例（CASE_004/005/006）未命中，情景A支撑不足</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -13853,12 +13853,12 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>CASE_004; CASE_005; CASE_006; CASE_007; WH_002; CASE_010; TRD_001; RELOC_001; RELOC_004; RELOC_006</t>
+          <t>CASE_004; CASE_005; CASE_006; CASE_007; WH_002; CASE_010; TRD_001</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>CASE_010; WH_002; RETURN_001; RELOC_006; WH_001</t>
+          <t>CASE_010; WH_002; WH_001; TRD_001; CASE_007</t>
         </is>
       </c>
     </row>
@@ -14034,7 +14034,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AI-assisted pre-scoring (content-based). Review flagged rows before finalising.</t>
+          <t>AI-assisted pre-scoring (content-based, keyed by evidence_id). Review flagged rows before finalising.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(eval): v0.9.1 — EU question set, industry re-derivation, screening lexicon
Task 2/3 question set
* add Q041-Q043 (EU battery regulation / EU countervailing duty / CRMA +
  FDI screening) so EU_001-EU_004 are actually measurable; 43 questions total
  (Company 8 / Policy·Trade 14 / Supply Chain 7 / Market Access 8 / Scenario 6)

Task 1 annotations
* re-derive all 49 rows of `industry` from evidence_metadata.build_meta(), so
  the human-readable sheet and the Task 4 filter agree; also fix two wrong
  related_industries tags (TRD_001, MOFCOM_002)

Task 4
* investment_policy lexicon was missing 外资安全审查 / 收购 / screening
  phrasings, so Q043's question was not detected as an investment question and
  the F1 macro-drift rule pushed EU_004 out of the Top-10; Q043 gold now ranks
  Top-2 and the full variant reaches P@5 0.800 / R@10 0.925
* treat target attainment as >= (was strictly >), so P@5 = 0.800 counts

docs/reports regenerated; 115 tests pass
</commit_message>
<xml_diff>
--- a/Task2_manual_scoring_v3.xlsx
+++ b/Task2_manual_scoring_v3.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Rubric" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Item Scoring'!$A$1:$Q$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Item Scoring'!$A$1:$Q$216</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q201"/>
+  <dimension ref="A1:Q216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2686,12 +2686,12 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>CASE_009</t>
+          <t>MOFCOM_002</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>BIS 50%穿透规则：发布→暂停→2026-11-10恢复的完整时间线</t>
+          <t>商务部公告2025年第72号（暂停实施2024年第46号公告第二款，涉及对美两用物项出口管制）</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2705,25 +2705,25 @@
         </is>
       </c>
       <c r="G29" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H29" s="2" t="n">
         <v>2</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J29" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>BIS规则时间线合成案例，内容重复BIS_001/002</t>
+          <t>暂停措施涉及镓、锗、石墨，直接回答</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>美国商务部工业与安全局（BIS）</t>
+          <t>商务部</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: CASE_009 Title: BIS 50%穿透规则：发布→暂停→2026-11-10恢复的完整时间线 Publisher: 美国商务部工业与安全局（BIS） Country/Jurisdiction: US / Federal Publication date: 2025-09-30 Status: CURRENT Topic: 出口管制 Applicability scope: GENERAL Related industries: 通用 Key finding: 政策事件型案例，由BIS_001和BIS_002组成。可用</t>
+          <t>Evidence ID: MOFCOM_002 Title: 商务部公告2025年第72号（暂停实施2024年第46号公告第二款，涉及对美两用物项出口管制） Publisher: 商务部 Country/Jurisdiction: CN / National Publication date: 2025-11-09 Status: CURRENT Topic: 出口管制 Applicability scope: GENERAL Related industries: 电池材料 Key finding: 目前仅见第三方转述：暂停期至2026-11-27，涉</t>
         </is>
       </c>
     </row>
@@ -2763,12 +2763,12 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>MOFCOM_002</t>
+          <t>CASE_009</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>商务部公告2025年第72号（暂停实施2024年第46号公告第二款，涉及对美两用物项出口管制）</t>
+          <t>BIS 50%穿透规则：发布→暂停→2026-11-10恢复的完整时间线</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2782,25 +2782,25 @@
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H30" s="2" t="n">
         <v>2</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>暂停措施涉及镓、锗、石墨，直接回答</t>
+          <t>BIS规则时间线合成案例，内容重复BIS_001/002</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>商务部</t>
+          <t>美国商务部工业与安全局（BIS）</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: MOFCOM_002 Title: 商务部公告2025年第72号（暂停实施2024年第46号公告第二款，涉及对美两用物项出口管制） Publisher: 商务部 Country/Jurisdiction: CN / National Publication date: 2025-11-09 Status: CURRENT Topic: 出口管制 Applicability scope: GENERAL Related industries: ◆随产业 Key finding: 目前仅见第三方转述：暂停期至2026-11-27，涉</t>
+          <t>Evidence ID: CASE_009 Title: BIS 50%穿透规则：发布→暂停→2026-11-10恢复的完整时间线 Publisher: 美国商务部工业与安全局（BIS） Country/Jurisdiction: US / Federal Publication date: 2025-09-30 Status: CURRENT Topic: 出口管制 Applicability scope: GENERAL Related industries: 通用 Key finding: 政策事件型案例，由BIS_001和BIS_002组成。可用</t>
         </is>
       </c>
     </row>
@@ -3595,7 +3595,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: MOFCOM_002 Title: 商务部公告2025年第72号（暂停实施2024年第46号公告第二款，涉及对美两用物项出口管制） Publisher: 商务部 Country/Jurisdiction: CN / National Publication date: 2025-11-09 Status: CURRENT Topic: 出口管制 Applicability scope: GENERAL Related industries: ◆随产业 Key finding: 目前仅见第三方转述：暂停期至2026-11-27，涉</t>
+          <t>Evidence ID: MOFCOM_002 Title: 商务部公告2025年第72号（暂停实施2024年第46号公告第二款，涉及对美两用物项出口管制） Publisher: 商务部 Country/Jurisdiction: CN / National Publication date: 2025-11-09 Status: CURRENT Topic: 出口管制 Applicability scope: GENERAL Related industries: 电池材料 Key finding: 目前仅见第三方转述：暂停期至2026-11-27，涉</t>
         </is>
       </c>
     </row>
@@ -6444,7 +6444,7 @@
       </c>
       <c r="Q77" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: TRD_001 Title: 美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: US / Federal Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: ◆电子/光电 Key finding: HS 851762仅为光</t>
+          <t>Evidence ID: TRD_001 Title: 美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: US / Federal Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: 动力电池 Key finding: HS 851762仅为光模块</t>
         </is>
       </c>
     </row>
@@ -6613,44 +6613,44 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>TRD_002</t>
+          <t>DHS_001</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>美国自越南、泰国、马来西亚、柬埔寨进口光伏组件HS 854140，2018–2025年度</t>
+          <t>Notice Regarding the Uyghur Forced Labor Prevention Act Entity List（UFLPA 实体清单更新公告）</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>贸易流</t>
+          <t>劳工</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>A+</t>
+          <t>S</t>
         </is>
       </c>
       <c r="G80" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
         <v>2</v>
       </c>
       <c r="I80" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J80" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t>同区域同模式的贸易转移数据（光伏组件），可作模式类比，非EV/电池口径</t>
+          <t>强迫劳动清单不能支持美国 EV/电池进口来源是否转移的判断</t>
         </is>
       </c>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t>联合国商品贸易统计数据库（UN Comtrade）</t>
+          <t>美国国土安全部（DHS，Federal Register）</t>
         </is>
       </c>
       <c r="M80" s="2" t="inlineStr">
@@ -6675,7 +6675,7 @@
       </c>
       <c r="Q80" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: TRD_002 Title: 美国自越南、泰国、马来西亚、柬埔寨进口光伏组件HS 854140，2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: US / Federal Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: ◆光伏 Key finding: HS 2022版起光伏组件编码调整（旧</t>
+          <t>Evidence ID: DHS_001 Title: Notice Regarding the Uyghur Forced Labor Prevention Act Entity List（UFLPA 实体清单更新公告） Publisher: 美国国土安全部（DHS，Federal Register） Country/Jurisdiction: US/CN / Federal Publication date: 2026-08-03 Status: CURRENT Topic: 劳工 Applicability scope: GENERAL Relat</t>
         </is>
       </c>
     </row>
@@ -6690,44 +6690,44 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>DHS_001</t>
+          <t>TRD_002</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Notice Regarding the Uyghur Forced Labor Prevention Act Entity List（UFLPA 实体清单更新公告）</t>
+          <t>美国自越南、泰国、马来西亚、柬埔寨进口光伏组件HS 854140，2018–2025年度</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>劳工</t>
+          <t>贸易流</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="G81" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H81" s="2" t="n">
         <v>2</v>
       </c>
       <c r="I81" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J81" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K81" s="2" t="inlineStr">
         <is>
-          <t>强迫劳动清单不能支持美国 EV/电池进口来源是否转移的判断</t>
+          <t>同区域同模式的贸易转移数据（光伏组件），可作模式类比，非EV/电池口径</t>
         </is>
       </c>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t>美国国土安全部（DHS，Federal Register）</t>
+          <t>联合国商品贸易统计数据库（UN Comtrade）</t>
         </is>
       </c>
       <c r="M81" s="2" t="inlineStr">
@@ -6752,7 +6752,7 @@
       </c>
       <c r="Q81" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: DHS_001 Title: Notice Regarding the Uyghur Forced Labor Prevention Act Entity List（UFLPA 实体清单更新公告） Publisher: 美国国土安全部（DHS，Federal Register） Country/Jurisdiction: US/CN / Federal Publication date: 2026-08-03 Status: CURRENT Topic: 劳工 Applicability scope: GENERAL Relat</t>
+          <t>Evidence ID: TRD_002 Title: 美国自越南、泰国、马来西亚、柬埔寨进口光伏组件HS 854140，2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: US / Federal Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: ◆光伏 Key finding: HS 2022版起光伏组件编码调整（旧</t>
         </is>
       </c>
     </row>
@@ -7522,7 +7522,7 @@
       </c>
       <c r="Q91" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: TRD_001 Title: 美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: US / Federal Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: ◆电子/光电 Key finding: HS 851762仅为光</t>
+          <t>Evidence ID: TRD_001 Title: 美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: US / Federal Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: 动力电池 Key finding: HS 851762仅为光模块</t>
         </is>
       </c>
     </row>
@@ -8215,7 +8215,7 @@
       </c>
       <c r="Q100" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: TRD_001 Title: 美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: US / Federal Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: ◆电子/光电 Key finding: HS 851762仅为光</t>
+          <t>Evidence ID: TRD_001 Title: 美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: US / Federal Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: 动力电池 Key finding: HS 851762仅为光模块</t>
         </is>
       </c>
     </row>
@@ -12835,7 +12835,7 @@
       </c>
       <c r="Q160" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: MOFCOM_002 Title: 商务部公告2025年第72号（暂停实施2024年第46号公告第二款，涉及对美两用物项出口管制） Publisher: 商务部 Country/Jurisdiction: CN / National Publication date: 2025-11-09 Status: CURRENT Topic: 出口管制 Applicability scope: GENERAL Related industries: ◆随产业 Key finding: 目前仅见第三方转述：暂停期至2026-11-27，涉</t>
+          <t>Evidence ID: MOFCOM_002 Title: 商务部公告2025年第72号（暂停实施2024年第46号公告第二款，涉及对美两用物项出口管制） Publisher: 商务部 Country/Jurisdiction: CN / National Publication date: 2025-11-09 Status: CURRENT Topic: 出口管制 Applicability scope: GENERAL Related industries: 电池材料 Key finding: 目前仅见第三方转述：暂停期至2026-11-27，涉</t>
         </is>
       </c>
     </row>
@@ -13297,7 +13297,7 @@
       </c>
       <c r="Q166" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: TRD_001 Title: 美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: US / Federal Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: ◆电子/光电 Key finding: HS 851762仅为光</t>
+          <t>Evidence ID: TRD_001 Title: 美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: US / Federal Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: 动力电池 Key finding: HS 851762仅为光模块</t>
         </is>
       </c>
     </row>
@@ -14683,7 +14683,7 @@
       </c>
       <c r="Q184" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: TRD_001 Title: 美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: US / Federal Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: ◆电子/光电 Key finding: HS 851762仅为光</t>
+          <t>Evidence ID: TRD_001 Title: 美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: US / Federal Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: 动力电池 Key finding: HS 851762仅为光模块</t>
         </is>
       </c>
     </row>
@@ -15314,44 +15314,44 @@
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>DHS_001</t>
+          <t>TRD_001</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>Notice Regarding the Uyghur Forced Labor Prevention Act Entity List（UFLPA 实体清单更新公告）</t>
+          <t>美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度</t>
         </is>
       </c>
       <c r="E193" s="2" t="inlineStr">
         <is>
-          <t>劳工</t>
+          <t>贸易流</t>
         </is>
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="G193" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H193" s="2" t="n">
         <v>2</v>
       </c>
       <c r="I193" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J193" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>强迫劳动清单不提供供给集中度数据</t>
+          <t>美国自中/越/泰/马进口 EV(870380) 与锂电池(850760) 数据，可部分反映电池供给来源集中度（美国市场口径），但不提供全球份额</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
         <is>
-          <t>美国国土安全部（DHS，Federal Register）</t>
+          <t>联合国商品贸易统计数据库（UN Comtrade）</t>
         </is>
       </c>
       <c r="M193" s="2" t="inlineStr">
@@ -15376,7 +15376,7 @@
       </c>
       <c r="Q193" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: DHS_001 Title: Notice Regarding the Uyghur Forced Labor Prevention Act Entity List（UFLPA 实体清单更新公告） Publisher: 美国国土安全部（DHS，Federal Register） Country/Jurisdiction: US/CN / Federal Publication date: 2026-08-03 Status: CURRENT Topic: 劳工 Applicability scope: GENERAL Relat</t>
+          <t>Evidence ID: TRD_001 Title: 美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: US / Federal Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: 动力电池 Key finding: HS 851762仅为光模块</t>
         </is>
       </c>
     </row>
@@ -15391,17 +15391,17 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>EU_003</t>
+          <t>DHS_001</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>Commission Implementing Regulation (EU) 2024/2754 imposing a definitive countervailing duty on imports of new battery electric vehicles originating in China（对华纯电动车最终反补贴税）</t>
+          <t>Notice Regarding the Uyghur Forced Labor Prevention Act Entity List（UFLPA 实体清单更新公告）</t>
         </is>
       </c>
       <c r="E194" s="2" t="inlineStr">
         <is>
-          <t>关税</t>
+          <t>劳工</t>
         </is>
       </c>
       <c r="F194" s="2" t="inlineStr">
@@ -15423,12 +15423,12 @@
       </c>
       <c r="K194" s="2" t="inlineStr">
         <is>
-          <t>欧盟反补贴税属政策回应，不含集中度数据</t>
+          <t>强迫劳动清单不提供供给集中度数据</t>
         </is>
       </c>
       <c r="L194" s="2" t="inlineStr">
         <is>
-          <t>欧盟委员会（EUR-Lex / Official Journal）</t>
+          <t>美国国土安全部（DHS，Federal Register）</t>
         </is>
       </c>
       <c r="M194" s="2" t="inlineStr">
@@ -15453,7 +15453,7 @@
       </c>
       <c r="Q194" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: EU_003 Title: Commission Implementing Regulation (EU) 2024/2754 imposing a definitive countervailing duty on imports of new battery electric vehicles originating in China（对华纯电动车最终反补贴税） Publisher: 欧盟委员会（EUR-Lex / Official Journal） Country/Jurisdiction: EU/CN / EU-wide</t>
+          <t>Evidence ID: DHS_001 Title: Notice Regarding the Uyghur Forced Labor Prevention Act Entity List（UFLPA 实体清单更新公告） Publisher: 美国国土安全部（DHS，Federal Register） Country/Jurisdiction: US/CN / Federal Publication date: 2026-08-03 Status: CURRENT Topic: 劳工 Applicability scope: GENERAL Relat</t>
         </is>
       </c>
     </row>
@@ -15468,17 +15468,17 @@
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>IRS_001</t>
+          <t>EU_003</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>Clean Vehicle Credits Under Sections 25E and 30D; Transfer of Credits; Critical Minerals and Battery Components; Foreign Entities of Concern（清洁车辆抵免与FEOC最终规则）</t>
+          <t>Commission Implementing Regulation (EU) 2024/2754 imposing a definitive countervailing duty on imports of new battery electric vehicles originating in China（对华纯电动车最终反补贴税）</t>
         </is>
       </c>
       <c r="E195" s="2" t="inlineStr">
         <is>
-          <t>本地化政策</t>
+          <t>关税</t>
         </is>
       </c>
       <c r="F195" s="2" t="inlineStr">
@@ -15500,12 +15500,12 @@
       </c>
       <c r="K195" s="2" t="inlineStr">
         <is>
-          <t>IRA FEOC 规则属政策回应，不含集中度数据</t>
+          <t>欧盟反补贴税属政策回应，不含集中度数据</t>
         </is>
       </c>
       <c r="L195" s="2" t="inlineStr">
         <is>
-          <t>美国财政部/国税局（Federal Register）</t>
+          <t>欧盟委员会（EUR-Lex / Official Journal）</t>
         </is>
       </c>
       <c r="M195" s="2" t="inlineStr">
@@ -15530,7 +15530,7 @@
       </c>
       <c r="Q195" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: IRS_001 Title: Clean Vehicle Credits Under Sections 25E and 30D; Transfer of Credits; Critical Minerals and Battery Components; Foreign Entities of Concern（清洁车辆抵免与FEOC最终规则） Publisher: 美国财政部/国税局（Federal Register） Country/Jurisdiction: US / Federal Publication date: 20</t>
+          <t>Evidence ID: EU_003 Title: Commission Implementing Regulation (EU) 2024/2754 imposing a definitive countervailing duty on imports of new battery electric vehicles originating in China（对华纯电动车最终反补贴税） Publisher: 欧盟委员会（EUR-Lex / Official Journal） Country/Jurisdiction: EU/CN / EU-wide</t>
         </is>
       </c>
     </row>
@@ -15545,17 +15545,17 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>EU_001</t>
+          <t>IRS_001</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>Regulation (EU) 2023/1542 concerning batteries and waste batteries（欧盟电池与废电池法规）</t>
+          <t>Clean Vehicle Credits Under Sections 25E and 30D; Transfer of Credits; Critical Minerals and Battery Components; Foreign Entities of Concern（清洁车辆抵免与FEOC最终规则）</t>
         </is>
       </c>
       <c r="E196" s="2" t="inlineStr">
         <is>
-          <t>市场准入</t>
+          <t>本地化政策</t>
         </is>
       </c>
       <c r="F196" s="2" t="inlineStr">
@@ -15577,12 +15577,12 @@
       </c>
       <c r="K196" s="2" t="inlineStr">
         <is>
-          <t>欧盟电池法规属准入合规，与供给集中度无关</t>
+          <t>IRA FEOC 规则属政策回应，不含集中度数据</t>
         </is>
       </c>
       <c r="L196" s="2" t="inlineStr">
         <is>
-          <t>欧洲议会与欧盟理事会（EUR-Lex / Official Journal）</t>
+          <t>美国财政部/国税局（Federal Register）</t>
         </is>
       </c>
       <c r="M196" s="2" t="inlineStr">
@@ -15607,7 +15607,7 @@
       </c>
       <c r="Q196" s="2" t="inlineStr">
         <is>
-          <t>Evidence ID: EU_001 Title: Regulation (EU) 2023/1542 concerning batteries and waste batteries（欧盟电池与废电池法规） Publisher: 欧洲议会与欧盟理事会（EUR-Lex / Official Journal） Country/Jurisdiction: EU / EU-wide Publication date: 2023-07-28 Effective date: 2023-08-17 Status: CURRENT Topic: 市场准入 Appli</t>
+          <t>Evidence ID: IRS_001 Title: Clean Vehicle Credits Under Sections 25E and 30D; Transfer of Credits; Critical Minerals and Battery Components; Foreign Entities of Concern（清洁车辆抵免与FEOC最终规则） Publisher: 美国财政部/国税局（Federal Register） Country/Jurisdiction: US / Federal Publication date: 20</t>
         </is>
       </c>
     </row>
@@ -15996,10 +15996,1165 @@
         </is>
       </c>
     </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>Q041</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>EU_001</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>Regulation (EU) 2023/1542 concerning batteries and waste batteries（欧盟电池与废电池法规）</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>市场准入</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H202" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I202" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J202" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K202" s="2" t="inlineStr">
+        <is>
+          <t>本题 expected 证据：欧盟电池法规第 7/9/77 条（碳足迹、再生材料含量、尽职调查、电池护照）</t>
+        </is>
+      </c>
+      <c r="L202" s="2" t="inlineStr">
+        <is>
+          <t>欧洲议会与欧盟理事会（EUR-Lex / Official Journal）</t>
+        </is>
+      </c>
+      <c r="M202" s="2" t="inlineStr">
+        <is>
+          <t>Market Access</t>
+        </is>
+      </c>
+      <c r="N202" s="2" t="inlineStr">
+        <is>
+          <t>market_access</t>
+        </is>
+      </c>
+      <c r="O202" s="2" t="inlineStr">
+        <is>
+          <t>EU_001</t>
+        </is>
+      </c>
+      <c r="P202" s="2" t="inlineStr">
+        <is>
+          <t>我们准备向欧盟出口 EV 电池。欧盟电池法规对进入欧盟市场的电池提出了哪些强制合规要求（碳足迹、再生材料含量、供应链尽职调查、电池护照）？</t>
+        </is>
+      </c>
+      <c r="Q202" s="2" t="inlineStr">
+        <is>
+          <t>Evidence ID: EU_001 Title: Regulation (EU) 2023/1542 concerning batteries and waste batteries（欧盟电池与废电池法规） Publisher: 欧洲议会与欧盟理事会（EUR-Lex / Official Journal） Country/Jurisdiction: EU / EU-wide Publication date: 2023-07-28 Effective date: 2023-08-17 Status: CURRENT Topic: 市场准入 Appli</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>Q041</t>
+        </is>
+      </c>
+      <c r="B203" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C203" s="2" t="inlineStr">
+        <is>
+          <t>DHS_001</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>Notice Regarding the Uyghur Forced Labor Prevention Act Entity List（UFLPA 实体清单更新公告）</t>
+        </is>
+      </c>
+      <c r="E203" s="2" t="inlineStr">
+        <is>
+          <t>劳工</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G203" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H203" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I203" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J203" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K203" s="2" t="inlineStr">
+        <is>
+          <t>美国 UFLPA 进口限制与欧盟电池合规要求属不同辖区/不同域</t>
+        </is>
+      </c>
+      <c r="L203" s="2" t="inlineStr">
+        <is>
+          <t>美国国土安全部（DHS，Federal Register）</t>
+        </is>
+      </c>
+      <c r="M203" s="2" t="inlineStr">
+        <is>
+          <t>Market Access</t>
+        </is>
+      </c>
+      <c r="N203" s="2" t="inlineStr">
+        <is>
+          <t>market_access</t>
+        </is>
+      </c>
+      <c r="O203" s="2" t="inlineStr">
+        <is>
+          <t>EU_001</t>
+        </is>
+      </c>
+      <c r="P203" s="2" t="inlineStr">
+        <is>
+          <t>我们准备向欧盟出口 EV 电池。欧盟电池法规对进入欧盟市场的电池提出了哪些强制合规要求（碳足迹、再生材料含量、供应链尽职调查、电池护照）？</t>
+        </is>
+      </c>
+      <c r="Q203" s="2" t="inlineStr">
+        <is>
+          <t>Evidence ID: DHS_001 Title: Notice Regarding the Uyghur Forced Labor Prevention Act Entity List（UFLPA 实体清单更新公告） Publisher: 美国国土安全部（DHS，Federal Register） Country/Jurisdiction: US/CN / Federal Publication date: 2026-08-03 Status: CURRENT Topic: 劳工 Applicability scope: GENERAL Relat</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>Q041</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>EU_003</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>Commission Implementing Regulation (EU) 2024/2754 imposing a definitive countervailing duty on imports of new battery electric vehicles originating in China（对华纯电动车最终反补贴税）</t>
+        </is>
+      </c>
+      <c r="E204" s="2" t="inlineStr">
+        <is>
+          <t>关税</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G204" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H204" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I204" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J204" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K204" s="2" t="inlineStr">
+        <is>
+          <t>欧盟对华纯电反补贴税属同一辖区(EU)的市场准入措施，可作欧盟侧贸易壁垒背景，但不回答电池产品合规要求 ｜ 人工判定与Auto(0)不同，请复核</t>
+        </is>
+      </c>
+      <c r="L204" s="2" t="inlineStr">
+        <is>
+          <t>欧盟委员会（EUR-Lex / Official Journal）</t>
+        </is>
+      </c>
+      <c r="M204" s="2" t="inlineStr">
+        <is>
+          <t>Market Access</t>
+        </is>
+      </c>
+      <c r="N204" s="2" t="inlineStr">
+        <is>
+          <t>market_access</t>
+        </is>
+      </c>
+      <c r="O204" s="2" t="inlineStr">
+        <is>
+          <t>EU_001</t>
+        </is>
+      </c>
+      <c r="P204" s="2" t="inlineStr">
+        <is>
+          <t>我们准备向欧盟出口 EV 电池。欧盟电池法规对进入欧盟市场的电池提出了哪些强制合规要求（碳足迹、再生材料含量、供应链尽职调查、电池护照）？</t>
+        </is>
+      </c>
+      <c r="Q204" s="2" t="inlineStr">
+        <is>
+          <t>Evidence ID: EU_003 Title: Commission Implementing Regulation (EU) 2024/2754 imposing a definitive countervailing duty on imports of new battery electric vehicles originating in China（对华纯电动车最终反补贴税） Publisher: 欧盟委员会（EUR-Lex / Official Journal） Country/Jurisdiction: EU/CN / EU-wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>Q041</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C205" s="2" t="inlineStr">
+        <is>
+          <t>CSIS_001</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>The Visibility Gap: How AI Can Stop Chinese Transshipment Under USMCA</t>
+        </is>
+      </c>
+      <c r="E205" s="2" t="inlineStr">
+        <is>
+          <t>原产地与转运</t>
+        </is>
+      </c>
+      <c r="F205" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G205" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H205" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I205" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J205" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K205" s="2" t="inlineStr">
+        <is>
+          <t>转运可视化分析，与欧盟电池产品合规要求无关 ｜ 人工判定与Auto(1)不同，请复核</t>
+        </is>
+      </c>
+      <c r="L205" s="2" t="inlineStr">
+        <is>
+          <t>战略与国际研究中心（CSIS）</t>
+        </is>
+      </c>
+      <c r="M205" s="2" t="inlineStr">
+        <is>
+          <t>Market Access</t>
+        </is>
+      </c>
+      <c r="N205" s="2" t="inlineStr">
+        <is>
+          <t>market_access</t>
+        </is>
+      </c>
+      <c r="O205" s="2" t="inlineStr">
+        <is>
+          <t>EU_001</t>
+        </is>
+      </c>
+      <c r="P205" s="2" t="inlineStr">
+        <is>
+          <t>我们准备向欧盟出口 EV 电池。欧盟电池法规对进入欧盟市场的电池提出了哪些强制合规要求（碳足迹、再生材料含量、供应链尽职调查、电池护照）？</t>
+        </is>
+      </c>
+      <c r="Q205" s="2" t="inlineStr">
+        <is>
+          <t>The EV battery example shows the problem that a product passport is designed to solve. At its simplest, a product passport is a digital record that travels with a good through its supply chain, showing where its inputs came from and whether it qualiﬁes for preferential treatment</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>Q041</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t>SNE_001</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>January-August 2026 Global EV Battery Usage Reaches 844.2 GWh, Up 19.7% Year-on-Year（2026年1–8月全球动力电池装车量快报）</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t>供应链布局</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G206" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H206" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I206" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J206" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K206" s="2" t="inlineStr">
+        <is>
+          <t>电池装车量市场数据，不回答合规要求</t>
+        </is>
+      </c>
+      <c r="L206" s="2" t="inlineStr">
+        <is>
+          <t>SNE Research</t>
+        </is>
+      </c>
+      <c r="M206" s="2" t="inlineStr">
+        <is>
+          <t>Market Access</t>
+        </is>
+      </c>
+      <c r="N206" s="2" t="inlineStr">
+        <is>
+          <t>market_access</t>
+        </is>
+      </c>
+      <c r="O206" s="2" t="inlineStr">
+        <is>
+          <t>EU_001</t>
+        </is>
+      </c>
+      <c r="P206" s="2" t="inlineStr">
+        <is>
+          <t>我们准备向欧盟出口 EV 电池。欧盟电池法规对进入欧盟市场的电池提出了哪些强制合规要求（碳足迹、再生材料含量、供应链尽职调查、电池护照）？</t>
+        </is>
+      </c>
+      <c r="Q206" s="2" t="inlineStr">
+        <is>
+          <t>Evidence ID: SNE_001 Title: January-August 2026 Global EV Battery Usage Reaches 844.2 GWh, Up 19.7% Year-on-Year（2026年1–8月全球动力电池装车量快报） Publisher: SNE Research Country/Jurisdiction: 全球 / Global Publication date: 2026-10-02 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>Q042</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C207" s="2" t="inlineStr">
+        <is>
+          <t>EU_003</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>Commission Implementing Regulation (EU) 2024/2754 imposing a definitive countervailing duty on imports of new battery electric vehicles originating in China（对华纯电动车最终反补贴税）</t>
+        </is>
+      </c>
+      <c r="E207" s="2" t="inlineStr">
+        <is>
+          <t>关税</t>
+        </is>
+      </c>
+      <c r="F207" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G207" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H207" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I207" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J207" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K207" s="2" t="inlineStr">
+        <is>
+          <t>本题 expected 证据：欧盟对华纯电最终反补贴税税率（BYD 17.0% / Geely 18.8% / SAIC 35.3% / Tesla 7.8% 等）</t>
+        </is>
+      </c>
+      <c r="L207" s="2" t="inlineStr">
+        <is>
+          <t>欧盟委员会（EUR-Lex / Official Journal）</t>
+        </is>
+      </c>
+      <c r="M207" s="2" t="inlineStr">
+        <is>
+          <t>Policy / Trade Risk</t>
+        </is>
+      </c>
+      <c r="N207" s="2" t="inlineStr">
+        <is>
+          <t>tariff</t>
+        </is>
+      </c>
+      <c r="O207" s="2" t="inlineStr">
+        <is>
+          <t>EU_003</t>
+        </is>
+      </c>
+      <c r="P207" s="2" t="inlineStr">
+        <is>
+          <t>欧盟对中国产纯电动车征收的最终反补贴税税率是多少？不同企业（比亚迪/吉利/上汽/特斯拉）的税率差异如何？</t>
+        </is>
+      </c>
+      <c r="Q207" s="2" t="inlineStr">
+        <is>
+          <t>Evidence ID: EU_003 Title: Commission Implementing Regulation (EU) 2024/2754 imposing a definitive countervailing duty on imports of new battery electric vehicles originating in China（对华纯电动车最终反补贴税） Publisher: 欧盟委员会（EUR-Lex / Official Journal） Country/Jurisdiction: EU/CN / EU-wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>Q042</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
+        <is>
+          <t>CASE_002</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>美国对东南亚四国光伏产品反规避认定：视为中国原产并适用对华双反</t>
+        </is>
+      </c>
+      <c r="E208" s="2" t="inlineStr">
+        <is>
+          <t>反规避</t>
+        </is>
+      </c>
+      <c r="F208" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G208" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H208" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I208" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J208" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K208" s="2" t="inlineStr">
+        <is>
+          <t>美国对东南亚光伏的反规避裁定，辖区与措施类型均不同</t>
+        </is>
+      </c>
+      <c r="L208" s="2" t="inlineStr">
+        <is>
+          <t>美国商务部（经律所解读）</t>
+        </is>
+      </c>
+      <c r="M208" s="2" t="inlineStr">
+        <is>
+          <t>Policy / Trade Risk</t>
+        </is>
+      </c>
+      <c r="N208" s="2" t="inlineStr">
+        <is>
+          <t>tariff</t>
+        </is>
+      </c>
+      <c r="O208" s="2" t="inlineStr">
+        <is>
+          <t>EU_003</t>
+        </is>
+      </c>
+      <c r="P208" s="2" t="inlineStr">
+        <is>
+          <t>欧盟对中国产纯电动车征收的最终反补贴税税率是多少？不同企业（比亚迪/吉利/上汽/特斯拉）的税率差异如何？</t>
+        </is>
+      </c>
+      <c r="Q208" s="2" t="inlineStr">
+        <is>
+          <t>Evidence ID: CASE_002 Title: 美国对东南亚四国光伏产品反规避认定：视为中国原产并适用对华双反 Publisher: 美国商务部（经律所解读） Country/Jurisdiction: 柬埔寨/马来西亚/泰国/越南 Publication date: 2023-08-18 Status: CURRENT Topic: 反规避 Applicability scope: GENERAL Related industries: 光伏 Key finding: 2022年4月立案，2023年8月终裁。使用中国组件在东南亚完成的电池和组</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>Q042</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C209" s="2" t="inlineStr">
+        <is>
+          <t>DHS_001</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>Notice Regarding the Uyghur Forced Labor Prevention Act Entity List（UFLPA 实体清单更新公告）</t>
+        </is>
+      </c>
+      <c r="E209" s="2" t="inlineStr">
+        <is>
+          <t>劳工</t>
+        </is>
+      </c>
+      <c r="F209" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G209" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H209" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I209" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J209" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K209" s="2" t="inlineStr">
+        <is>
+          <t>强迫劳动实体清单与欧盟反补贴税率无关</t>
+        </is>
+      </c>
+      <c r="L209" s="2" t="inlineStr">
+        <is>
+          <t>美国国土安全部（DHS，Federal Register）</t>
+        </is>
+      </c>
+      <c r="M209" s="2" t="inlineStr">
+        <is>
+          <t>Policy / Trade Risk</t>
+        </is>
+      </c>
+      <c r="N209" s="2" t="inlineStr">
+        <is>
+          <t>tariff</t>
+        </is>
+      </c>
+      <c r="O209" s="2" t="inlineStr">
+        <is>
+          <t>EU_003</t>
+        </is>
+      </c>
+      <c r="P209" s="2" t="inlineStr">
+        <is>
+          <t>欧盟对中国产纯电动车征收的最终反补贴税税率是多少？不同企业（比亚迪/吉利/上汽/特斯拉）的税率差异如何？</t>
+        </is>
+      </c>
+      <c r="Q209" s="2" t="inlineStr">
+        <is>
+          <t>Evidence ID: DHS_001 Title: Notice Regarding the Uyghur Forced Labor Prevention Act Entity List（UFLPA 实体清单更新公告） Publisher: 美国国土安全部（DHS，Federal Register） Country/Jurisdiction: US/CN / Federal Publication date: 2026-08-03 Status: CURRENT Topic: 劳工 Applicability scope: GENERAL Relat</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>Q042</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C210" s="2" t="inlineStr">
+        <is>
+          <t>TRD_001</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度</t>
+        </is>
+      </c>
+      <c r="E210" s="2" t="inlineStr">
+        <is>
+          <t>贸易流</t>
+        </is>
+      </c>
+      <c r="F210" s="2" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="G210" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H210" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I210" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J210" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K210" s="2" t="inlineStr">
+        <is>
+          <t>美国 EV/锂电池进口数据，不含欧盟税率信息；作为跨辖区贸易流数据不可用于本题计算 ｜ 人工判定与Auto(1)不同，请复核</t>
+        </is>
+      </c>
+      <c r="L210" s="2" t="inlineStr">
+        <is>
+          <t>联合国商品贸易统计数据库（UN Comtrade）</t>
+        </is>
+      </c>
+      <c r="M210" s="2" t="inlineStr">
+        <is>
+          <t>Policy / Trade Risk</t>
+        </is>
+      </c>
+      <c r="N210" s="2" t="inlineStr">
+        <is>
+          <t>tariff</t>
+        </is>
+      </c>
+      <c r="O210" s="2" t="inlineStr">
+        <is>
+          <t>EU_003</t>
+        </is>
+      </c>
+      <c r="P210" s="2" t="inlineStr">
+        <is>
+          <t>欧盟对中国产纯电动车征收的最终反补贴税税率是多少？不同企业（比亚迪/吉利/上汽/特斯拉）的税率差异如何？</t>
+        </is>
+      </c>
+      <c r="Q210" s="2" t="inlineStr">
+        <is>
+          <t>Evidence ID: TRD_001 Title: 美国自中国、越南、泰国、马来西亚进口 HS 870380, 850760，2018–2025年度 Publisher: 联合国商品贸易统计数据库（UN Comtrade） Country/Jurisdiction: US / Federal Publication date: 持续更新 Status: CURRENT Topic: 贸易流 Applicability scope: GENERAL Related industries: 动力电池 Key finding: HS 851762仅为光模块</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>Q042</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C211" s="2" t="inlineStr">
+        <is>
+          <t>SNE_001</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>January-August 2026 Global EV Battery Usage Reaches 844.2 GWh, Up 19.7% Year-on-Year（2026年1–8月全球动力电池装车量快报）</t>
+        </is>
+      </c>
+      <c r="E211" s="2" t="inlineStr">
+        <is>
+          <t>供应链布局</t>
+        </is>
+      </c>
+      <c r="F211" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G211" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H211" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I211" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J211" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K211" s="2" t="inlineStr">
+        <is>
+          <t>电池装车量数据与税率无关</t>
+        </is>
+      </c>
+      <c r="L211" s="2" t="inlineStr">
+        <is>
+          <t>SNE Research</t>
+        </is>
+      </c>
+      <c r="M211" s="2" t="inlineStr">
+        <is>
+          <t>Policy / Trade Risk</t>
+        </is>
+      </c>
+      <c r="N211" s="2" t="inlineStr">
+        <is>
+          <t>tariff</t>
+        </is>
+      </c>
+      <c r="O211" s="2" t="inlineStr">
+        <is>
+          <t>EU_003</t>
+        </is>
+      </c>
+      <c r="P211" s="2" t="inlineStr">
+        <is>
+          <t>欧盟对中国产纯电动车征收的最终反补贴税税率是多少？不同企业（比亚迪/吉利/上汽/特斯拉）的税率差异如何？</t>
+        </is>
+      </c>
+      <c r="Q211" s="2" t="inlineStr">
+        <is>
+          <t>Evidence ID: SNE_001 Title: January-August 2026 Global EV Battery Usage Reaches 844.2 GWh, Up 19.7% Year-on-Year（2026年1–8月全球动力电池装车量快报） Publisher: SNE Research Country/Jurisdiction: 全球 / Global Publication date: 2026-10-02 Status: CURRENT Topic: 供应链布局 Applicability scope: GENERAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>Q043</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C212" s="2" t="inlineStr">
+        <is>
+          <t>EU_002</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>Regulation (EU) 2024/1252 establishing a framework for ensuring a secure and sustainable supply of critical raw materials（欧盟关键原材料法案 CRMA）</t>
+        </is>
+      </c>
+      <c r="E212" s="2" t="inlineStr">
+        <is>
+          <t>本地化政策</t>
+        </is>
+      </c>
+      <c r="F212" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G212" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H212" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I212" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J212" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K212" s="2" t="inlineStr">
+        <is>
+          <t>本题 expected 证据：CRMA 本土开采 10%/加工 40%/回收 25% 目标与单一第三国 ≤65% 上限</t>
+        </is>
+      </c>
+      <c r="L212" s="2" t="inlineStr">
+        <is>
+          <t>欧洲议会与欧盟理事会（EUR-Lex / Official Journal）</t>
+        </is>
+      </c>
+      <c r="M212" s="2" t="inlineStr">
+        <is>
+          <t>Policy / Trade Risk</t>
+        </is>
+      </c>
+      <c r="N212" s="2" t="inlineStr">
+        <is>
+          <t>investment_policy</t>
+        </is>
+      </c>
+      <c r="O212" s="2" t="inlineStr">
+        <is>
+          <t>EU_002; EU_004</t>
+        </is>
+      </c>
+      <c r="P212" s="2" t="inlineStr">
+        <is>
+          <t>如果中国电池企业要在欧盟建厂或收购当地电池资产，欧盟层面的外资安全审查框架和关键原材料法案会带来哪些约束（审查范围、本土化与单一第三国依赖目标）？</t>
+        </is>
+      </c>
+      <c r="Q212" s="2" t="inlineStr">
+        <is>
+          <t>Evidence ID: EU_002 Title: Regulation (EU) 2024/1252 establishing a framework for ensuring a secure and sustainable supply of critical raw materials（欧盟关键原材料法案 CRMA） Publisher: 欧洲议会与欧盟理事会（EUR-Lex / Official Journal） Country/Jurisdiction: EU / EU-wide Publication date: 2024-05-03 E</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>Q043</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C213" s="2" t="inlineStr">
+        <is>
+          <t>EU_004</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>Regulation (EU) 2019/452 establishing a framework for the screening of foreign direct investments into the Union（欧盟外资安全审查框架条例）</t>
+        </is>
+      </c>
+      <c r="E213" s="2" t="inlineStr">
+        <is>
+          <t>对外投资</t>
+        </is>
+      </c>
+      <c r="F213" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G213" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H213" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I213" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J213" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K213" s="2" t="inlineStr">
+        <is>
+          <t>本题 expected 证据：欧盟外资安全审查框架（成员国可按安全/公共秩序审查外资）</t>
+        </is>
+      </c>
+      <c r="L213" s="2" t="inlineStr">
+        <is>
+          <t>欧洲议会与欧盟理事会（EUR-Lex / Official Journal）</t>
+        </is>
+      </c>
+      <c r="M213" s="2" t="inlineStr">
+        <is>
+          <t>Policy / Trade Risk</t>
+        </is>
+      </c>
+      <c r="N213" s="2" t="inlineStr">
+        <is>
+          <t>investment_policy</t>
+        </is>
+      </c>
+      <c r="O213" s="2" t="inlineStr">
+        <is>
+          <t>EU_002; EU_004</t>
+        </is>
+      </c>
+      <c r="P213" s="2" t="inlineStr">
+        <is>
+          <t>如果中国电池企业要在欧盟建厂或收购当地电池资产，欧盟层面的外资安全审查框架和关键原材料法案会带来哪些约束（审查范围、本土化与单一第三国依赖目标）？</t>
+        </is>
+      </c>
+      <c r="Q213" s="2" t="inlineStr">
+        <is>
+          <t>Evidence ID: EU_004 Title: Regulation (EU) 2019/452 establishing a framework for the screening of foreign direct investments into the Union（欧盟外资安全审查框架条例） Publisher: 欧洲议会与欧盟理事会（EUR-Lex / Official Journal） Country/Jurisdiction: EU / EU-wide Publication date: 2019-03-21 Effective da</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>Q043</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C214" s="2" t="inlineStr">
+        <is>
+          <t>DHS_001</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>Notice Regarding the Uyghur Forced Labor Prevention Act Entity List（UFLPA 实体清单更新公告）</t>
+        </is>
+      </c>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
+          <t>劳工</t>
+        </is>
+      </c>
+      <c r="F214" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G214" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H214" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I214" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J214" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K214" s="2" t="inlineStr">
+        <is>
+          <t>美国强迫劳动清单与欧盟层面投资约束无关</t>
+        </is>
+      </c>
+      <c r="L214" s="2" t="inlineStr">
+        <is>
+          <t>美国国土安全部（DHS，Federal Register）</t>
+        </is>
+      </c>
+      <c r="M214" s="2" t="inlineStr">
+        <is>
+          <t>Policy / Trade Risk</t>
+        </is>
+      </c>
+      <c r="N214" s="2" t="inlineStr">
+        <is>
+          <t>investment_policy</t>
+        </is>
+      </c>
+      <c r="O214" s="2" t="inlineStr">
+        <is>
+          <t>EU_002; EU_004</t>
+        </is>
+      </c>
+      <c r="P214" s="2" t="inlineStr">
+        <is>
+          <t>如果中国电池企业要在欧盟建厂或收购当地电池资产，欧盟层面的外资安全审查框架和关键原材料法案会带来哪些约束（审查范围、本土化与单一第三国依赖目标）？</t>
+        </is>
+      </c>
+      <c r="Q214" s="2" t="inlineStr">
+        <is>
+          <t>Evidence ID: DHS_001 Title: Notice Regarding the Uyghur Forced Labor Prevention Act Entity List（UFLPA 实体清单更新公告） Publisher: 美国国土安全部（DHS，Federal Register） Country/Jurisdiction: US/CN / Federal Publication date: 2026-08-03 Status: CURRENT Topic: 劳工 Applicability scope: GENERAL Relat</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>Q043</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C215" s="2" t="inlineStr">
+        <is>
+          <t>EU_001</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>Regulation (EU) 2023/1542 concerning batteries and waste batteries（欧盟电池与废电池法规）</t>
+        </is>
+      </c>
+      <c r="E215" s="2" t="inlineStr">
+        <is>
+          <t>市场准入</t>
+        </is>
+      </c>
+      <c r="F215" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G215" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H215" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I215" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J215" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K215" s="2" t="inlineStr">
+        <is>
+          <t>欧盟电池法规的合规与尽责要求，属同一辖区监管约束，可补足建厂后的产品侧义务 ｜ 人工判定与Auto(0)不同，请复核</t>
+        </is>
+      </c>
+      <c r="L215" s="2" t="inlineStr">
+        <is>
+          <t>欧洲议会与欧盟理事会（EUR-Lex / Official Journal）</t>
+        </is>
+      </c>
+      <c r="M215" s="2" t="inlineStr">
+        <is>
+          <t>Policy / Trade Risk</t>
+        </is>
+      </c>
+      <c r="N215" s="2" t="inlineStr">
+        <is>
+          <t>investment_policy</t>
+        </is>
+      </c>
+      <c r="O215" s="2" t="inlineStr">
+        <is>
+          <t>EU_002; EU_004</t>
+        </is>
+      </c>
+      <c r="P215" s="2" t="inlineStr">
+        <is>
+          <t>如果中国电池企业要在欧盟建厂或收购当地电池资产，欧盟层面的外资安全审查框架和关键原材料法案会带来哪些约束（审查范围、本土化与单一第三国依赖目标）？</t>
+        </is>
+      </c>
+      <c r="Q215" s="2" t="inlineStr">
+        <is>
+          <t>Evidence ID: EU_001 Title: Regulation (EU) 2023/1542 concerning batteries and waste batteries（欧盟电池与废电池法规） Publisher: 欧洲议会与欧盟理事会（EUR-Lex / Official Journal） Country/Jurisdiction: EU / EU-wide Publication date: 2023-07-28 Effective date: 2023-08-17 Status: CURRENT Topic: 市场准入 Appli</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>Q043</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C216" s="2" t="inlineStr">
+        <is>
+          <t>EU_003</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>Commission Implementing Regulation (EU) 2024/2754 imposing a definitive countervailing duty on imports of new battery electric vehicles originating in China（对华纯电动车最终反补贴税）</t>
+        </is>
+      </c>
+      <c r="E216" s="2" t="inlineStr">
+        <is>
+          <t>关税</t>
+        </is>
+      </c>
+      <c r="F216" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G216" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H216" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I216" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J216" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K216" s="2" t="inlineStr">
+        <is>
+          <t>欧盟对华纯电反补贴税，属同一辖区贸易措施，影响对欧建厂/出口的成本判断 ｜ 人工判定与Auto(0)不同，请复核</t>
+        </is>
+      </c>
+      <c r="L216" s="2" t="inlineStr">
+        <is>
+          <t>欧盟委员会（EUR-Lex / Official Journal）</t>
+        </is>
+      </c>
+      <c r="M216" s="2" t="inlineStr">
+        <is>
+          <t>Policy / Trade Risk</t>
+        </is>
+      </c>
+      <c r="N216" s="2" t="inlineStr">
+        <is>
+          <t>investment_policy</t>
+        </is>
+      </c>
+      <c r="O216" s="2" t="inlineStr">
+        <is>
+          <t>EU_002; EU_004</t>
+        </is>
+      </c>
+      <c r="P216" s="2" t="inlineStr">
+        <is>
+          <t>如果中国电池企业要在欧盟建厂或收购当地电池资产，欧盟层面的外资安全审查框架和关键原材料法案会带来哪些约束（审查范围、本土化与单一第三国依赖目标）？</t>
+        </is>
+      </c>
+      <c r="Q216" s="2" t="inlineStr">
+        <is>
+          <t>Evidence ID: EU_003 Title: Commission Implementing Regulation (EU) 2024/2754 imposing a definitive countervailing duty on imports of new battery electric vehicles originating in China（对华纯电动车最终反补贴税） Publisher: 欧盟委员会（EUR-Lex / Official Journal） Country/Jurisdiction: EU/CN / EU-wide</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q201"/>
+  <autoFilter ref="A1:Q216"/>
   <dataValidations count="1">
-    <dataValidation sqref="I2:J201" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:J216" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"0,1,2"</formula1>
     </dataValidation>
   </dataValidations>
@@ -16013,7 +17168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -16105,11 +17260,11 @@
         <v>4</v>
       </c>
       <c r="D2" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A2,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A2,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E2" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A2,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A2,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F2" s="3" t="n">
@@ -16159,11 +17314,11 @@
         <v>2</v>
       </c>
       <c r="D3" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A3,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A3,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E3" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A3,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A3,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F3" s="3" t="n">
@@ -16213,11 +17368,11 @@
         <v>1</v>
       </c>
       <c r="D4" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A4,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A4,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E4" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A4,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A4,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F4" s="3" t="n">
@@ -16267,11 +17422,11 @@
         <v>5</v>
       </c>
       <c r="D5" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A5,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A5,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E5" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A5,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A5,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F5" s="3" t="n">
@@ -16321,11 +17476,11 @@
         <v>4</v>
       </c>
       <c r="D6" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A6,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A6,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E6" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A6,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A6,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F6" s="3" t="n">
@@ -16375,11 +17530,11 @@
         <v>4</v>
       </c>
       <c r="D7" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A7,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A7,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E7" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A7,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A7,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F7" s="3" t="n">
@@ -16412,7 +17567,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>BIS_002; BIS_001; CASE_009; MOFCOM_002; MOFCOM_001</t>
+          <t>BIS_002; BIS_001; MOFCOM_002; CASE_009; MOFCOM_001</t>
         </is>
       </c>
     </row>
@@ -16429,11 +17584,11 @@
         <v>4</v>
       </c>
       <c r="D8" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A8,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A8,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E8" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A8,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A8,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F8" s="3" t="n">
@@ -16483,11 +17638,11 @@
         <v>3</v>
       </c>
       <c r="D9" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A9,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A9,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E9" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A9,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A9,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F9" s="3" t="n">
@@ -16537,11 +17692,11 @@
         <v>4</v>
       </c>
       <c r="D10" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A10,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A10,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E10" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A10,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A10,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F10" s="3" t="n">
@@ -16591,11 +17746,11 @@
         <v>3</v>
       </c>
       <c r="D11" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A11,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A11,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E11" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A11,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A11,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F11" s="3" t="n">
@@ -16645,11 +17800,11 @@
         <v>3</v>
       </c>
       <c r="D12" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A12,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A12,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E12" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A12,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A12,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F12" s="3" t="n">
@@ -16699,11 +17854,11 @@
         <v>2</v>
       </c>
       <c r="D13" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A13,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A13,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E13" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A13,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A13,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F13" s="3" t="n">
@@ -16753,11 +17908,11 @@
         <v>5</v>
       </c>
       <c r="D14" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A14,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A14,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E14" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A14,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A14,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F14" s="3" t="n">
@@ -16807,11 +17962,11 @@
         <v>4</v>
       </c>
       <c r="D15" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A15,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A15,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E15" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A15,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A15,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F15" s="3" t="n">
@@ -16861,11 +18016,11 @@
         <v>2</v>
       </c>
       <c r="D16" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A16,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A16,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E16" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A16,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A16,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F16" s="3" t="n">
@@ -16915,11 +18070,11 @@
         <v>2</v>
       </c>
       <c r="D17" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A17,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A17,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E17" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A17,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A17,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F17" s="3" t="n">
@@ -16952,7 +18107,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; TRD_003; CASE_003; TRD_002; DHS_001</t>
+          <t>TRD_001; TRD_003; CASE_003; DHS_001; TRD_002</t>
         </is>
       </c>
     </row>
@@ -16969,11 +18124,11 @@
         <v>4</v>
       </c>
       <c r="D18" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A18,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A18,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E18" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A18,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A18,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F18" s="3" t="n">
@@ -17023,11 +18178,11 @@
         <v>3</v>
       </c>
       <c r="D19" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A19,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A19,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E19" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A19,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A19,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F19" s="3" t="n">
@@ -17077,11 +18232,11 @@
         <v>3</v>
       </c>
       <c r="D20" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A20,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A20,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E20" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A20,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A20,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F20" s="3" t="n">
@@ -17131,11 +18286,11 @@
         <v>4</v>
       </c>
       <c r="D21" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A21,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A21,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E21" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A21,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A21,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F21" s="3" t="n">
@@ -17185,11 +18340,11 @@
         <v>4</v>
       </c>
       <c r="D22" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A22,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A22,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E22" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A22,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A22,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F22" s="3" t="n">
@@ -17239,11 +18394,11 @@
         <v>3</v>
       </c>
       <c r="D23" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A23,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A23,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E23" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A23,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A23,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F23" s="3" t="n">
@@ -17293,11 +18448,11 @@
         <v>5</v>
       </c>
       <c r="D24" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A24,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A24,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E24" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A24,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A24,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F24" s="3" t="n">
@@ -17347,11 +18502,11 @@
         <v>5</v>
       </c>
       <c r="D25" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A25,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A25,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E25" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A25,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A25,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F25" s="3" t="n">
@@ -17401,11 +18556,11 @@
         <v>3</v>
       </c>
       <c r="D26" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A26,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A26,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E26" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A26,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A26,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F26" s="3" t="n">
@@ -17455,11 +18610,11 @@
         <v>4</v>
       </c>
       <c r="D27" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A27,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A27,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E27" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A27,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A27,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F27" s="3" t="n">
@@ -17509,11 +18664,11 @@
         <v>4</v>
       </c>
       <c r="D28" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A28,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A28,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E28" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A28,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A28,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F28" s="3" t="n">
@@ -17563,11 +18718,11 @@
         <v>5</v>
       </c>
       <c r="D29" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A29,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A29,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E29" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A29,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A29,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F29" s="3" t="n">
@@ -17617,11 +18772,11 @@
         <v>3</v>
       </c>
       <c r="D30" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A30,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A30,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E30" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A30,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A30,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F30" s="3" t="n">
@@ -17671,11 +18826,11 @@
         <v>3</v>
       </c>
       <c r="D31" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A31,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A31,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E31" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A31,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A31,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F31" s="3" t="n">
@@ -17725,11 +18880,11 @@
         <v>1</v>
       </c>
       <c r="D32" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A32,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A32,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E32" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A32,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A32,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F32" s="3" t="n">
@@ -17779,11 +18934,11 @@
         <v>2</v>
       </c>
       <c r="D33" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A33,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A33,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E33" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A33,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A33,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F33" s="3" t="n">
@@ -17833,11 +18988,11 @@
         <v>1</v>
       </c>
       <c r="D34" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A34,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A34,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E34" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A34,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A34,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F34" s="3" t="n">
@@ -17887,11 +19042,11 @@
         <v>1</v>
       </c>
       <c r="D35" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A35,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A35,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E35" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A35,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A35,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F35" s="3" t="n">
@@ -17941,11 +19096,11 @@
         <v>2</v>
       </c>
       <c r="D36" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A36,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A36,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E36" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A36,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A36,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F36" s="3" t="n">
@@ -17995,11 +19150,11 @@
         <v>1</v>
       </c>
       <c r="D37" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A37,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A37,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E37" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A37,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A37,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F37" s="3" t="n">
@@ -18049,11 +19204,11 @@
         <v>1</v>
       </c>
       <c r="D38" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A38,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A38,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E38" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A38,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A38,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F38" s="3" t="n">
@@ -18103,11 +19258,11 @@
         <v>1</v>
       </c>
       <c r="D39" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A39,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A39,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E39" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A39,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A39,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F39" s="3" t="n">
@@ -18157,11 +19312,11 @@
         <v>1</v>
       </c>
       <c r="D40" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A40,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A40,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E40" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A40,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A40,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F40" s="3" t="n">
@@ -18194,7 +19349,7 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>SNE_001; DHS_001; EU_003; IRS_001; EU_001</t>
+          <t>SNE_001; TRD_001; DHS_001; EU_003; IRS_001</t>
         </is>
       </c>
     </row>
@@ -18211,11 +19366,11 @@
         <v>3</v>
       </c>
       <c r="D41" s="2">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A41,'Item Scoring'!$I$2:$I$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A41,'Item Scoring'!$I$2:$I$216),"")</f>
         <v/>
       </c>
       <c r="E41" s="3">
-        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$201,$A41,'Item Scoring'!$J$2:$J$201),"")</f>
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A41,'Item Scoring'!$J$2:$J$216),"")</f>
         <v/>
       </c>
       <c r="F41" s="3" t="n">
@@ -18249,12 +19404,174 @@
       <c r="L41" s="2" t="inlineStr">
         <is>
           <t>USMCA_001; WB_001; IRS_001; WTO_004; CASE_002</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Q041</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="2">
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A42,'Item Scoring'!$I$2:$I$216),"")</f>
+        <v/>
+      </c>
+      <c r="E42" s="3">
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A42,'Item Scoring'!$J$2:$J$216),"")</f>
+        <v/>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>gold（EU_001）命中且排名第1，欧盟电池法规合规要求可直接作答</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Market Access</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>market_access</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>我们准备向欧盟出口 EV 电池。欧盟电池法规对进入欧盟市场的电池提出了哪些强制合规要求（碳足迹、再生材料含量、供应链尽职调查、电池护照）？</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>EU_001</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>EU_001; DHS_001; EU_003; CSIS_001; SNE_001</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Q042</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="2">
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A43,'Item Scoring'!$I$2:$I$216),"")</f>
+        <v/>
+      </c>
+      <c r="E43" s="3">
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A43,'Item Scoring'!$J$2:$J$216),"")</f>
+        <v/>
+      </c>
+      <c r="F43" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>gold（EU_003）命中且排名第1，各企业反补贴税率可直接作答</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Policy / Trade Risk</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>tariff</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>欧盟对中国产纯电动车征收的最终反补贴税税率是多少？不同企业（比亚迪/吉利/上汽/特斯拉）的税率差异如何？</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>EU_003</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>EU_003; CASE_002; DHS_001; TRD_001; SNE_001</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Q043</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" s="2">
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A44,'Item Scoring'!$I$2:$I$216),"")</f>
+        <v/>
+      </c>
+      <c r="E44" s="3">
+        <f>IFERROR(AVERAGEIF('Item Scoring'!$A$2:$A$216,$A44,'Item Scoring'!$J$2:$J$216),"")</f>
+        <v/>
+      </c>
+      <c r="F44" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>两份 gold（EU_002/EU_004）全部命中，分别排名第1–2</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Policy / Trade Risk</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>investment_policy</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>如果中国电池企业要在欧盟建厂或收购当地电池资产，欧盟层面的外资安全审查框架和关键原材料法案会带来哪些约束（审查范围、本土化与单一第三国依赖目标）？</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
+          <t>EU_002; EU_004</t>
+        </is>
+      </c>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>EU_002; EU_004; DHS_001; EU_001; EU_003</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"0,1,2"</formula1>
     </dataValidation>
   </dataValidations>
@@ -18329,7 +19646,7 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>AVERAGE('Question Scoring'!$D$2:$D$41)</f>
+        <f>AVERAGE('Question Scoring'!$D$2:$D$44)</f>
         <v/>
       </c>
       <c r="C5" t="inlineStr">
@@ -18349,7 +19666,7 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>AVERAGE('Question Scoring'!$E$2:$E$41)</f>
+        <f>AVERAGE('Question Scoring'!$E$2:$E$44)</f>
         <v/>
       </c>
       <c r="C6" t="inlineStr">
@@ -18369,7 +19686,7 @@
         </is>
       </c>
       <c r="B7" s="8">
-        <f>AVERAGE('Question Scoring'!$B$2:$B$41)</f>
+        <f>AVERAGE('Question Scoring'!$B$2:$B$44)</f>
         <v/>
       </c>
       <c r="C7" t="inlineStr">
@@ -18389,7 +19706,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>IFERROR(AVERAGE('Question Scoring'!$F$2:$F$41),"")</f>
+        <f>IFERROR(AVERAGE('Question Scoring'!$F$2:$F$44),"")</f>
         <v/>
       </c>
       <c r="C8" t="inlineStr">

</xml_diff>